<commit_message>
Mise à jour des prix du 28 mars 2026
</commit_message>
<xml_diff>
--- a/analyse-prix-composants.xlsx
+++ b/analyse-prix-composants.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuille1!$A:$AC</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuille1!$A:$AE</definedName>
     <definedName name="Print_Titles" localSheetId="0">Feuille1!$7:$7</definedName>
   </definedNames>
   <calcPr/>
@@ -54,12 +54,6 @@
     <t xml:space="preserve">(c) 2025, 2026 Alexia Gossa</t>
   </si>
   <si>
-    <t xml:space="preserve">Chaque samedi sur Twitch, depuis le 6 décembre 2025, on fait le point sur les prix de l'IT en regardant quelques composants.</t>
-  </si>
-  <si>
-    <t>https://www.twitch.tv/alexia_vassiliki</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -124,6 +118,12 @@
   </si>
   <si>
     <t xml:space="preserve">14 mar 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 mar 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 mar 2026</t>
   </si>
   <si>
     <t>Min</t>
@@ -620,6 +620,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
@@ -628,12 +634,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.049989318521683403"/>
         <bgColor theme="0" tint="-0.049989318521683403"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -700,7 +700,7 @@
     <xf fontId="2" fillId="3" borderId="2" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="4" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -758,14 +758,18 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="1"/>
     </xf>
-    <xf fontId="3" fillId="8" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="1"/>
+    </xf>
+    <xf fontId="3" fillId="9" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="1"/>
     </xf>
-    <xf fontId="3" fillId="8" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="3" fillId="9" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="3" fillId="8" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="3" fillId="9" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="15" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -778,18 +782,14 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="1"/>
     </xf>
-    <xf fontId="3" fillId="9" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="3" fillId="10" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="4" fillId="9" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="4" fillId="10" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="14" fillId="9" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="14" fillId="10" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="1"/>
-    </xf>
-    <xf fontId="5" fillId="9" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
       <protection locked="1"/>
     </xf>
     <xf fontId="5" fillId="10" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -800,12 +800,16 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="1"/>
     </xf>
-    <xf fontId="5" fillId="9" borderId="0" numFmtId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="5" fillId="10" borderId="0" numFmtId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="1"/>
     </xf>
     <xf fontId="16" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf fontId="17" fillId="8" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="1"/>
     </xf>
     <xf fontId="10" fillId="12" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1342,12 +1346,12 @@
     <col bestFit="1" min="12" max="12" style="4" width="11.7109375"/>
     <col bestFit="1" min="13" max="13" style="4" width="13.00390625"/>
     <col bestFit="1" min="14" max="15" style="4" width="14.140625"/>
-    <col customWidth="1" min="16" max="22" style="1" width="12.7109375"/>
-    <col customWidth="1" min="23" max="26" style="2" width="12.7109375"/>
-    <col customWidth="1" min="27" max="27" style="2" width="14.140625"/>
-    <col customWidth="1" min="28" max="29" style="2" width="12.7109375"/>
-    <col customWidth="1" min="30" max="30" style="5" width="42.28125"/>
-    <col min="31" max="16384" style="1" width="9.140625"/>
+    <col customWidth="1" min="16" max="24" style="1" width="12.7109375"/>
+    <col customWidth="1" min="25" max="28" style="2" width="12.7109375"/>
+    <col customWidth="1" min="29" max="29" style="2" width="14.140625"/>
+    <col customWidth="1" min="30" max="31" style="2" width="12.7109375"/>
+    <col customWidth="1" min="32" max="32" style="5" width="42.28125"/>
+    <col min="33" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="33">
@@ -1362,28 +1366,30 @@
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
-      <c r="W1" s="7" t="s">
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="Z1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AB1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="AA1" s="7" t="s">
+      <c r="AC1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AB1" s="7" t="s">
+      <c r="AD1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AC1" s="7" t="s">
+      <c r="AE1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="AD1" s="5"/>
+      <c r="AF1" s="5"/>
     </row>
     <row r="2" ht="23.25">
       <c r="A2" s="2"/>
@@ -1397,13 +1403,15 @@
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
-      <c r="W2" s="7"/>
-      <c r="X2" s="7"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
       <c r="Y2" s="7"/>
       <c r="Z2" s="7"/>
       <c r="AA2" s="7"/>
       <c r="AB2" s="7"/>
       <c r="AC2" s="7"/>
+      <c r="AD2" s="7"/>
+      <c r="AE2" s="7"/>
     </row>
     <row r="3" ht="18">
       <c r="A3" s="2"/>
@@ -1415,19 +1423,19 @@
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
-      <c r="W3" s="7"/>
-      <c r="X3" s="7"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="1"/>
       <c r="Y3" s="7"/>
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
       <c r="AB3" s="7"/>
       <c r="AC3" s="7"/>
+      <c r="AD3" s="7"/>
+      <c r="AE3" s="7"/>
     </row>
     <row r="4" ht="54">
       <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="B4" s="3"/>
       <c r="G4" s="4"/>
       <c r="N4" s="4"/>
       <c r="Q4" s="1"/>
@@ -1436,19 +1444,19 @@
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
-      <c r="W4" s="7"/>
-      <c r="X4" s="7"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
       <c r="Y4" s="7"/>
       <c r="Z4" s="7"/>
       <c r="AA4" s="7"/>
       <c r="AB4" s="7"/>
       <c r="AC4" s="7"/>
+      <c r="AD4" s="7"/>
+      <c r="AE4" s="7"/>
     </row>
     <row r="5" ht="23.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="9" t="s">
-        <v>10</v>
-      </c>
+      <c r="B5" s="9"/>
       <c r="N5" s="4"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
@@ -1456,15 +1464,17 @@
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
-      <c r="W5" s="7"/>
-      <c r="X5" s="7"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
       <c r="Y5" s="7"/>
       <c r="Z5" s="7"/>
       <c r="AA5" s="7"/>
       <c r="AB5" s="7"/>
       <c r="AC5" s="7"/>
+      <c r="AD5" s="7"/>
+      <c r="AE5" s="7"/>
     </row>
-    <row r="6" ht="37.5" customHeight="1">
+    <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2"/>
       <c r="N6" s="4"/>
       <c r="Q6" s="1"/>
@@ -1473,103 +1483,111 @@
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
-      <c r="W6" s="7"/>
-      <c r="X6" s="7"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
       <c r="Y6" s="7"/>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
       <c r="AB6" s="7"/>
       <c r="AC6" s="7"/>
+      <c r="AD6" s="7"/>
+      <c r="AE6" s="7"/>
     </row>
     <row r="7" ht="18">
       <c r="A7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="E7" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="F7" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="G7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="H7" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="I7" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="J7" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="K7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="12" t="s">
+      <c r="L7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="M7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="N7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="O7" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="P7" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="Q7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="P7" s="12" t="s">
+      <c r="R7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="S7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="R7" s="12" t="s">
+      <c r="T7" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="S7" s="12" t="s">
+      <c r="U7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="T7" s="12" t="s">
+      <c r="V7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="U7" s="12" t="s">
+      <c r="W7" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="V7" s="12" t="s">
+      <c r="X7" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="W7" s="13" t="s">
+      <c r="Y7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="X7" s="13" t="s">
+      <c r="Z7" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="Y7" s="13" t="s">
+      <c r="AA7" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="Z7" s="13" t="s">
+      <c r="AB7" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="AA7" s="13" t="s">
+      <c r="AC7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="AB7" s="13" t="s">
+      <c r="AD7" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="AC7" s="13" t="s">
+      <c r="AE7" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="AD7" s="5" t="s">
+      <c r="AF7" s="5" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1634,38 +1652,44 @@
       <c r="V8" s="18">
         <v>366.26999999999998</v>
       </c>
-      <c r="W8" s="19">
-        <f>MIN(C8:V8)</f>
+      <c r="W8" s="18">
+        <v>370.38999999999999</v>
+      </c>
+      <c r="X8" s="19">
+        <v>415.97000000000003</v>
+      </c>
+      <c r="Y8" s="20">
+        <f>MIN(C8:X8)</f>
         <v>171.88</v>
       </c>
-      <c r="X8" s="20">
-        <f>MAX(C8:V8)</f>
-        <v>367.56</v>
-      </c>
-      <c r="Y8" s="20">
-        <f>AVERAGE(C8:V8)</f>
-        <v>336.27687500000013</v>
-      </c>
-      <c r="Z8" s="20">
-        <f>AVERAGE(Q8:V8)</f>
-        <v>366.58999999999997</v>
+      <c r="Z8" s="21">
+        <f>MAX(C8:X8)</f>
+        <v>415.97000000000003</v>
       </c>
       <c r="AA8" s="21">
+        <f>AVERAGE(C8:X8)</f>
+        <v>342.5994444444446</v>
+      </c>
+      <c r="AB8" s="21">
+        <f>AVERAGE(Q8:X8)</f>
+        <v>373.23749999999995</v>
+      </c>
+      <c r="AC8" s="22">
+        <f>(AB8/AA8)-1</f>
+        <v>8.9428211435770733e-002</v>
+      </c>
+      <c r="AD8" s="22">
+        <f>(AB8/Y8)-1</f>
+        <v>1.1715004654410053</v>
+      </c>
+      <c r="AE8" s="22">
         <f>(Z8/Y8)-1</f>
-        <v>9.0143352854696879e-002</v>
-      </c>
-      <c r="AB8" s="21">
-        <f>(Z8/W8)-1</f>
-        <v>1.1328252269024901</v>
-      </c>
-      <c r="AC8" s="21">
-        <f>(X8/W8)-1</f>
-        <v>1.1384686990923902</v>
-      </c>
-      <c r="AD8" s="22" t="s">
+        <v>1.4201186874563652</v>
+      </c>
+      <c r="AF8" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="AE8" s="23">
+      <c r="AG8" s="24">
         <f>C2*1</f>
         <v>0</v>
       </c>
@@ -1678,7 +1702,7 @@
         <v>45</v>
       </c>
       <c r="C9" s="16"/>
-      <c r="D9" s="24">
+      <c r="D9" s="25">
         <v>200.47999999999999</v>
       </c>
       <c r="E9" s="16"/>
@@ -1731,58 +1755,64 @@
       <c r="V9" s="18">
         <v>978.75</v>
       </c>
-      <c r="W9" s="19">
-        <f>MIN(C9:V9)</f>
+      <c r="W9" s="18">
+        <v>978.75</v>
+      </c>
+      <c r="X9" s="18">
+        <v>978.75</v>
+      </c>
+      <c r="Y9" s="20">
+        <f>MIN(C9:X9)</f>
         <v>200.47999999999999</v>
       </c>
-      <c r="X9" s="20">
-        <f>MAX(C9:V9)</f>
+      <c r="Z9" s="21">
+        <f>MAX(C9:X9)</f>
         <v>978.75</v>
       </c>
-      <c r="Y9" s="20">
-        <f>AVERAGE(C9:V9)</f>
-        <v>778.50750000000005</v>
-      </c>
-      <c r="Z9" s="20">
-        <f>AVERAGE(Q9:V9)</f>
-        <v>849.6583333333333</v>
-      </c>
       <c r="AA9" s="21">
+        <f>AVERAGE(C9:X9)</f>
+        <v>800.75666666666666</v>
+      </c>
+      <c r="AB9" s="21">
+        <f>AVERAGE(Q9:X9)</f>
+        <v>881.93124999999998</v>
+      </c>
+      <c r="AC9" s="22">
+        <f>(AB9/AA9)-1</f>
+        <v>0.10137234782101934</v>
+      </c>
+      <c r="AD9" s="22">
+        <f>(AB9/Y9)-1</f>
+        <v>3.3990984138068638</v>
+      </c>
+      <c r="AE9" s="22">
         <f>(Z9/Y9)-1</f>
-        <v>9.1393895798477454e-002</v>
-      </c>
-      <c r="AB9" s="21">
-        <f>(Z9/W9)-1</f>
-        <v>3.2381201782388933</v>
-      </c>
-      <c r="AC9" s="21">
-        <f>(X9/W9)-1</f>
         <v>3.8820331205107745</v>
       </c>
-      <c r="AD9" s="22" t="s">
+      <c r="AF9" s="23" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="10" ht="36">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="27"/>
-      <c r="D10" s="24">
+      <c r="C10" s="28"/>
+      <c r="D10" s="25">
         <v>284.13</v>
       </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28">
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="29">
         <v>403.11000000000001</v>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="29">
         <v>325.23000000000002</v>
       </c>
-      <c r="I10" s="28">
+      <c r="I10" s="29">
         <v>647.89999999999998</v>
       </c>
       <c r="J10" s="18">
@@ -1824,35 +1854,41 @@
       <c r="V10" s="18">
         <v>696.10000000000002</v>
       </c>
-      <c r="W10" s="19">
-        <f>MIN(C10:V10)</f>
+      <c r="W10" s="18">
+        <v>710</v>
+      </c>
+      <c r="X10" s="19">
+        <v>717.78999999999996</v>
+      </c>
+      <c r="Y10" s="20">
+        <f>MIN(C10:X10)</f>
         <v>284.13</v>
       </c>
-      <c r="X10" s="20">
-        <f>MAX(C10:V10)</f>
-        <v>700</v>
-      </c>
-      <c r="Y10" s="20">
-        <f>AVERAGE(C10:V10)</f>
-        <v>585.23470588235296</v>
-      </c>
-      <c r="Z10" s="20">
-        <f>AVERAGE(Q10:V10)</f>
-        <v>644.01999999999998</v>
+      <c r="Z10" s="21">
+        <f>MAX(C10:X10)</f>
+        <v>717.78999999999996</v>
       </c>
       <c r="AA10" s="21">
+        <f>AVERAGE(C10:X10)</f>
+        <v>598.77789473684209</v>
+      </c>
+      <c r="AB10" s="21">
+        <f>AVERAGE(Q10:X10)</f>
+        <v>661.48874999999998</v>
+      </c>
+      <c r="AC10" s="22">
+        <f>(AB10/AA10)-1</f>
+        <v>0.10473141345793802</v>
+      </c>
+      <c r="AD10" s="22">
+        <f>(AB10/Y10)-1</f>
+        <v>1.3281200506810262</v>
+      </c>
+      <c r="AE10" s="22">
         <f>(Z10/Y10)-1</f>
-        <v>0.10044738209607207</v>
-      </c>
-      <c r="AB10" s="21">
-        <f>(Z10/W10)-1</f>
-        <v>1.2666385105409494</v>
-      </c>
-      <c r="AC10" s="21">
-        <f>(X10/W10)-1</f>
-        <v>1.4636610002463661</v>
-      </c>
-      <c r="AD10" s="22" t="s">
+        <v>1.5262731848097699</v>
+      </c>
+      <c r="AF10" s="23" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1890,13 +1926,13 @@
       <c r="O11" s="18">
         <v>731.50999999999999</v>
       </c>
-      <c r="P11" s="29">
+      <c r="P11" s="19">
         <v>863.05999999999995</v>
       </c>
-      <c r="Q11" s="29">
+      <c r="Q11" s="19">
         <v>863.60000000000002</v>
       </c>
-      <c r="R11" s="29">
+      <c r="R11" s="19">
         <v>822.25</v>
       </c>
       <c r="S11" s="18">
@@ -1912,34 +1948,40 @@
         <v>807.03999999999996</v>
       </c>
       <c r="W11" s="19">
-        <f>MIN(C11:V11)</f>
+        <v>824.09000000000003</v>
+      </c>
+      <c r="X11" s="19">
+        <v>827.74000000000001</v>
+      </c>
+      <c r="Y11" s="20">
+        <f>MIN(C11:X11)</f>
         <v>685.71000000000004</v>
       </c>
-      <c r="X11" s="20">
-        <f>MAX(C11:V11)</f>
+      <c r="Z11" s="21">
+        <f>MAX(C11:X11)</f>
         <v>863.60000000000002</v>
       </c>
-      <c r="Y11" s="20">
-        <f>AVERAGE(C11:V11)</f>
-        <v>779.84928571428566</v>
-      </c>
-      <c r="Z11" s="20">
-        <f>AVERAGE(Q11:V11)</f>
-        <v>803.48333333333323</v>
-      </c>
       <c r="AA11" s="21">
+        <f>AVERAGE(C11:X11)</f>
+        <v>785.60749999999996</v>
+      </c>
+      <c r="AB11" s="21">
+        <f>AVERAGE(Q11:X11)</f>
+        <v>809.09124999999995</v>
+      </c>
+      <c r="AC11" s="22">
+        <f>(AB11/AA11)-1</f>
+        <v>2.989247174956966e-002</v>
+      </c>
+      <c r="AD11" s="22">
+        <f>(AB11/Y11)-1</f>
+        <v>0.17993211415904664</v>
+      </c>
+      <c r="AE11" s="22">
         <f>(Z11/Y11)-1</f>
-        <v>3.0305916863667459e-002</v>
-      </c>
-      <c r="AB11" s="21">
-        <f>(Z11/W11)-1</f>
-        <v>0.17175385123934772</v>
-      </c>
-      <c r="AC11" s="21">
-        <f>(X11/W11)-1</f>
         <v>0.25942453807002952</v>
       </c>
-      <c r="AD11" s="22" t="s">
+      <c r="AF11" s="23" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1965,7 +2007,7 @@
       <c r="I12" s="17">
         <v>550.98000000000002</v>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="25">
         <v>546.98000000000002</v>
       </c>
       <c r="K12" s="17">
@@ -1992,10 +2034,10 @@
       <c r="R12" s="18">
         <v>575.98000000000002</v>
       </c>
-      <c r="S12" s="24">
+      <c r="S12" s="25">
         <v>479</v>
       </c>
-      <c r="T12" s="24">
+      <c r="T12" s="25">
         <v>465</v>
       </c>
       <c r="U12" s="18">
@@ -2004,76 +2046,82 @@
       <c r="V12" s="18">
         <v>573.98000000000002</v>
       </c>
-      <c r="W12" s="19">
-        <f>MIN(C12:V12)</f>
+      <c r="W12" s="18">
+        <v>552.98000000000002</v>
+      </c>
+      <c r="X12" s="18">
+        <v>555.91999999999996</v>
+      </c>
+      <c r="Y12" s="20">
+        <f>MIN(C12:X12)</f>
         <v>465</v>
       </c>
-      <c r="X12" s="20">
-        <f>MAX(C12:V12)</f>
+      <c r="Z12" s="21">
+        <f>MAX(C12:X12)</f>
         <v>623.12</v>
       </c>
-      <c r="Y12" s="20">
-        <f>AVERAGE(C12:V12)</f>
-        <v>552.69647058823512</v>
-      </c>
-      <c r="Z12" s="20">
-        <f>AVERAGE(Q12:V12)</f>
-        <v>537.15333333333331</v>
-      </c>
       <c r="AA12" s="21">
+        <f>AVERAGE(C12:X12)</f>
+        <v>552.88105263157877</v>
+      </c>
+      <c r="AB12" s="21">
+        <f>AVERAGE(Q12:X12)</f>
+        <v>541.47749999999996</v>
+      </c>
+      <c r="AC12" s="22">
+        <f>(AB12/AA12)-1</f>
+        <v>-2.0625688974691192e-002</v>
+      </c>
+      <c r="AD12" s="22">
+        <f>(AB12/Y12)-1</f>
+        <v>0.16446774193548386</v>
+      </c>
+      <c r="AE12" s="22">
         <f>(Z12/Y12)-1</f>
-        <v>-2.8122374724700583e-002</v>
-      </c>
-      <c r="AB12" s="21">
-        <f>(Z12/W12)-1</f>
-        <v>0.15516845878136198</v>
-      </c>
-      <c r="AC12" s="21">
-        <f>(X12/W12)-1</f>
         <v>0.34004301075268817</v>
       </c>
-      <c r="AD12" s="22" t="s">
+      <c r="AF12" s="23" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="13" ht="36">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="24">
+      <c r="C13" s="28"/>
+      <c r="D13" s="25">
         <v>684.98000000000002</v>
       </c>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="28">
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="29">
         <v>839</v>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="29">
         <v>857.05999999999995</v>
       </c>
-      <c r="I13" s="28">
+      <c r="I13" s="29">
         <v>826.44000000000005</v>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="29">
         <v>853.54999999999995</v>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="29">
         <v>853.20000000000005</v>
       </c>
-      <c r="L13" s="28">
+      <c r="L13" s="29">
         <v>940.37</v>
       </c>
-      <c r="M13" s="28">
+      <c r="M13" s="29">
         <v>928.10000000000002</v>
       </c>
-      <c r="N13" s="28">
+      <c r="N13" s="29">
         <v>1084.8299999999999</v>
       </c>
-      <c r="O13" s="28">
+      <c r="O13" s="29">
         <v>1084.8299999999999</v>
       </c>
       <c r="P13" s="17" t="s">
@@ -2091,41 +2139,47 @@
       <c r="T13" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="U13" s="24">
+      <c r="U13" s="25">
         <v>592.17999999999995</v>
       </c>
-      <c r="V13" s="24">
+      <c r="V13" s="25">
         <v>606.50999999999999</v>
       </c>
-      <c r="W13" s="19">
-        <f>MIN(C13:V13)</f>
+      <c r="W13" s="25">
+        <v>608.62</v>
+      </c>
+      <c r="X13" s="25">
+        <v>623.23000000000002</v>
+      </c>
+      <c r="Y13" s="20">
+        <f>MIN(C13:X13)</f>
         <v>592.17999999999995</v>
       </c>
-      <c r="X13" s="20">
-        <f>MAX(C13:V13)</f>
+      <c r="Z13" s="21">
+        <f>MAX(C13:X13)</f>
         <v>1426.5699999999999</v>
       </c>
-      <c r="Y13" s="20">
-        <f>AVERAGE(C13:V13)</f>
-        <v>890.58615384615393</v>
-      </c>
-      <c r="Z13" s="20">
-        <f>AVERAGE(Q13:V13)</f>
-        <v>875.0866666666667</v>
-      </c>
       <c r="AA13" s="21">
+        <f>AVERAGE(C13:X13)</f>
+        <v>853.96466666666674</v>
+      </c>
+      <c r="AB13" s="21">
+        <f>AVERAGE(Q13:X13)</f>
+        <v>771.42200000000003</v>
+      </c>
+      <c r="AC13" s="22">
+        <f>(AB13/AA13)-1</f>
+        <v>-9.665817555293077e-002</v>
+      </c>
+      <c r="AD13" s="22">
+        <f>(AB13/Y13)-1</f>
+        <v>0.30268161707588925</v>
+      </c>
+      <c r="AE13" s="22">
         <f>(Z13/Y13)-1</f>
-        <v>-1.7403692065669274e-002</v>
-      </c>
-      <c r="AB13" s="21">
-        <f>(Z13/W13)-1</f>
-        <v>0.4777376248212819</v>
-      </c>
-      <c r="AC13" s="21">
-        <f>(X13/W13)-1</f>
         <v>1.4090141511027054</v>
       </c>
-      <c r="AD13" s="22" t="s">
+      <c r="AF13" s="23" t="s">
         <v>56</v>
       </c>
     </row>
@@ -2182,35 +2236,41 @@
       <c r="V14" s="18">
         <v>669.10000000000002</v>
       </c>
-      <c r="W14" s="19">
-        <f>MIN(C14:V14)</f>
+      <c r="W14" s="18">
+        <v>678.97000000000003</v>
+      </c>
+      <c r="X14" s="18">
+        <v>599.99000000000001</v>
+      </c>
+      <c r="Y14" s="20">
+        <f>MIN(C14:X14)</f>
         <v>580.98000000000002</v>
       </c>
-      <c r="X14" s="20">
-        <f>MAX(C14:V14)</f>
+      <c r="Z14" s="21">
+        <f>MAX(C14:X14)</f>
         <v>709.99000000000001</v>
       </c>
-      <c r="Y14" s="20">
-        <f>AVERAGE(C14:V14)</f>
-        <v>654.09846153846149</v>
-      </c>
-      <c r="Z14" s="20">
-        <f>AVERAGE(Q14:V14)</f>
-        <v>689.16500000000008</v>
-      </c>
       <c r="AA14" s="21">
+        <f>AVERAGE(C14:X14)</f>
+        <v>652.14933333333317</v>
+      </c>
+      <c r="AB14" s="21">
+        <f>AVERAGE(Q14:X14)</f>
+        <v>676.74375000000009</v>
+      </c>
+      <c r="AC14" s="22">
+        <f>(AB14/AA14)-1</f>
+        <v>3.7712860244688784e-002</v>
+      </c>
+      <c r="AD14" s="22">
+        <f>(AB14/Y14)-1</f>
+        <v>0.16483140555612952</v>
+      </c>
+      <c r="AE14" s="22">
         <f>(Z14/Y14)-1</f>
-        <v>5.3610489128901095e-002</v>
-      </c>
-      <c r="AB14" s="21">
-        <f>(Z14/W14)-1</f>
-        <v>0.18621122930221357</v>
-      </c>
-      <c r="AC14" s="21">
-        <f>(X14/W14)-1</f>
         <v>0.22205583668973117</v>
       </c>
-      <c r="AD14" s="22" t="s">
+      <c r="AF14" s="23" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2267,49 +2327,55 @@
       <c r="V15" s="17">
         <v>684.46000000000004</v>
       </c>
-      <c r="W15" s="19">
-        <f>MIN(C15:V15)</f>
+      <c r="W15" s="17">
+        <v>689</v>
+      </c>
+      <c r="X15" s="17">
+        <v>679</v>
+      </c>
+      <c r="Y15" s="20">
+        <f>MIN(C15:X15)</f>
         <v>622.63</v>
       </c>
-      <c r="X15" s="20">
-        <f>MAX(C15:V15)</f>
+      <c r="Z15" s="21">
+        <f>MAX(C15:X15)</f>
         <v>728.61000000000001</v>
       </c>
-      <c r="Y15" s="20">
-        <f>AVERAGE(C15:V15)</f>
-        <v>681.98230769230759</v>
-      </c>
-      <c r="Z15" s="20">
-        <f>AVERAGE(Q15:V15)</f>
-        <v>700.15166666666664</v>
-      </c>
       <c r="AA15" s="21">
+        <f>AVERAGE(C15:X15)</f>
+        <v>682.25133333333326</v>
+      </c>
+      <c r="AB15" s="21">
+        <f>AVERAGE(Q15:X15)</f>
+        <v>696.11374999999998</v>
+      </c>
+      <c r="AC15" s="22">
+        <f>(AB15/AA15)-1</f>
+        <v>2.0318636240603594e-002</v>
+      </c>
+      <c r="AD15" s="22">
+        <f>(AB15/Y15)-1</f>
+        <v>0.11802153767084778</v>
+      </c>
+      <c r="AE15" s="22">
         <f>(Z15/Y15)-1</f>
-        <v>2.6641979959627582e-002</v>
-      </c>
-      <c r="AB15" s="21">
-        <f>(Z15/W15)-1</f>
-        <v>0.1245067964387625</v>
-      </c>
-      <c r="AC15" s="21">
-        <f>(X15/W15)-1</f>
         <v>0.17021344940012528</v>
       </c>
-      <c r="AD15" s="22" t="s">
+      <c r="AF15" s="23" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="16" ht="18">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="27"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="31">
         <v>9100</v>
       </c>
@@ -2358,35 +2424,41 @@
       <c r="V16" s="17">
         <v>10867.4</v>
       </c>
-      <c r="W16" s="19">
-        <f>MIN(C16:V16)</f>
+      <c r="W16" s="17">
+        <v>10757.610000000001</v>
+      </c>
+      <c r="X16" s="17">
+        <v>10790.610000000001</v>
+      </c>
+      <c r="Y16" s="20">
+        <f>MIN(C16:X16)</f>
         <v>9100</v>
       </c>
-      <c r="X16" s="20">
-        <f>MAX(C16:V16)</f>
+      <c r="Z16" s="21">
+        <f>MAX(C16:X16)</f>
         <v>11315.18</v>
       </c>
-      <c r="Y16" s="20">
-        <f>AVERAGE(C16:V16)</f>
-        <v>9667.948124999999</v>
-      </c>
-      <c r="Z16" s="20">
-        <f>AVERAGE(Q16:V16)</f>
-        <v>10549.688333333334</v>
-      </c>
       <c r="AA16" s="21">
+        <f>AVERAGE(C16:X16)</f>
+        <v>9790.8549999999977</v>
+      </c>
+      <c r="AB16" s="21">
+        <f>AVERAGE(Q16:X16)</f>
+        <v>10605.793750000001</v>
+      </c>
+      <c r="AC16" s="22">
+        <f>(AB16/AA16)-1</f>
+        <v>8.3234686858298268e-002</v>
+      </c>
+      <c r="AD16" s="22">
+        <f>(AB16/Y16)-1</f>
+        <v>0.16547184065934073</v>
+      </c>
+      <c r="AE16" s="22">
         <f>(Z16/Y16)-1</f>
-        <v>9.1202414093769724e-002</v>
-      </c>
-      <c r="AB16" s="21">
-        <f>(Z16/W16)-1</f>
-        <v>0.15930641025641035</v>
-      </c>
-      <c r="AC16" s="21">
-        <f>(X16/W16)-1</f>
         <v>0.24342637362637376</v>
       </c>
-      <c r="AD16" s="22" t="s">
+      <c r="AF16" s="23" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2441,76 +2513,82 @@
       <c r="V17" s="18">
         <v>1611.1400000000001</v>
       </c>
-      <c r="W17" s="19">
-        <f>MIN(C17:V17)</f>
+      <c r="W17" s="18">
+        <v>1610.1400000000001</v>
+      </c>
+      <c r="X17" s="18">
+        <v>1610.8900000000001</v>
+      </c>
+      <c r="Y17" s="20">
+        <f>MIN(C17:X17)</f>
         <v>1297.6199999999999</v>
       </c>
-      <c r="X17" s="20">
-        <f>MAX(C17:V17)</f>
+      <c r="Z17" s="21">
+        <f>MAX(C17:X17)</f>
         <v>1697.6199999999999</v>
       </c>
-      <c r="Y17" s="20">
-        <f>AVERAGE(C17:V17)</f>
-        <v>1520.7341666666664</v>
-      </c>
-      <c r="Z17" s="20">
-        <f>AVERAGE(Q17:V17)</f>
-        <v>1571.7133333333334</v>
-      </c>
       <c r="AA17" s="21">
+        <f>AVERAGE(C17:X17)</f>
+        <v>1533.5599999999997</v>
+      </c>
+      <c r="AB17" s="21">
+        <f>AVERAGE(Q17:X17)</f>
+        <v>1581.4137499999999</v>
+      </c>
+      <c r="AC17" s="22">
+        <f>(AB17/AA17)-1</f>
+        <v>3.1204354573671766e-002</v>
+      </c>
+      <c r="AD17" s="22">
+        <f>(AB17/Y17)-1</f>
+        <v>0.21870327985080373</v>
+      </c>
+      <c r="AE17" s="22">
         <f>(Z17/Y17)-1</f>
-        <v>3.3522733811136352e-002</v>
-      </c>
-      <c r="AB17" s="21">
-        <f>(Z17/W17)-1</f>
-        <v>0.21122773487872681</v>
-      </c>
-      <c r="AC17" s="21">
-        <f>(X17/W17)-1</f>
         <v>0.30825665449052875</v>
       </c>
-      <c r="AD17" s="22" t="s">
+      <c r="AF17" s="23" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="18" ht="18">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28">
+      <c r="C18" s="28"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29">
         <v>2279</v>
       </c>
-      <c r="G18" s="28" t="s">
+      <c r="G18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="I18" s="28" t="s">
+      <c r="I18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="J18" s="28" t="s">
+      <c r="J18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="28" t="s">
+      <c r="K18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="L18" s="28" t="s">
+      <c r="L18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="M18" s="28" t="s">
+      <c r="M18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="N18" s="28" t="s">
+      <c r="N18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="O18" s="28" t="s">
+      <c r="O18" s="29" t="s">
         <v>66</v>
       </c>
       <c r="P18" s="17" t="s">
@@ -2534,35 +2612,41 @@
       <c r="V18" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="W18" s="19">
-        <f>MIN(C18:V18)</f>
+      <c r="W18" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="X18" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="Y18" s="20">
+        <f>MIN(C18:X18)</f>
         <v>2279</v>
       </c>
-      <c r="X18" s="20">
-        <f>MAX(C18:V18)</f>
+      <c r="Z18" s="21">
+        <f>MAX(C18:X18)</f>
         <v>2279</v>
       </c>
-      <c r="Y18" s="20">
-        <f>AVERAGE(C18:V18)</f>
+      <c r="AA18" s="21">
+        <f>AVERAGE(C18:X18)</f>
         <v>2279</v>
       </c>
-      <c r="Z18" s="20" t="e">
-        <f>AVERAGE(Q18:V18)</f>
+      <c r="AB18" s="21" t="e">
+        <f>AVERAGE(Q18:X18)</f>
         <v>#NUM!</v>
       </c>
-      <c r="AA18" s="21" t="e">
+      <c r="AC18" s="22" t="e">
+        <f>(AB18/AA18)-1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD18" s="22" t="e">
+        <f>(AB18/Y18)-1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE18" s="22">
         <f>(Z18/Y18)-1</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="AB18" s="21" t="e">
-        <f>(Z18/W18)-1</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="AC18" s="21">
-        <f>(X18/W18)-1</f>
         <v>0</v>
       </c>
-      <c r="AD18" s="22" t="s">
+      <c r="AF18" s="23" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2573,13 +2657,13 @@
       <c r="B19" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="25">
         <v>176.69</v>
       </c>
       <c r="D19" s="17"/>
       <c r="E19" s="17"/>
       <c r="F19" s="17"/>
-      <c r="G19" s="24">
+      <c r="G19" s="25">
         <v>150</v>
       </c>
       <c r="H19" s="17">
@@ -2594,19 +2678,19 @@
       <c r="K19" s="17">
         <v>199</v>
       </c>
-      <c r="L19" s="24">
+      <c r="L19" s="25">
         <v>145</v>
       </c>
-      <c r="M19" s="24">
+      <c r="M19" s="25">
         <v>150</v>
       </c>
-      <c r="N19" s="24">
+      <c r="N19" s="25">
         <v>150</v>
       </c>
-      <c r="O19" s="24">
+      <c r="O19" s="25">
         <v>148.05000000000001</v>
       </c>
-      <c r="P19" s="29">
+      <c r="P19" s="19">
         <v>219.69</v>
       </c>
       <c r="Q19" s="30">
@@ -2627,35 +2711,41 @@
       <c r="V19" s="30">
         <v>228</v>
       </c>
-      <c r="W19" s="19">
-        <f>MIN(C19:V19)</f>
+      <c r="W19" s="30">
+        <v>228</v>
+      </c>
+      <c r="X19" s="30">
+        <v>228</v>
+      </c>
+      <c r="Y19" s="20">
+        <f>MIN(C19:X19)</f>
         <v>145</v>
       </c>
-      <c r="X19" s="20">
-        <f>MAX(C19:V19)</f>
+      <c r="Z19" s="21">
+        <f>MAX(C19:X19)</f>
         <v>237.69999999999999</v>
       </c>
-      <c r="Y19" s="20">
-        <f>AVERAGE(C19:V19)</f>
-        <v>194.28999999999996</v>
-      </c>
-      <c r="Z19" s="20">
-        <f>AVERAGE(Q19:V19)</f>
-        <v>236.08333333333334</v>
-      </c>
       <c r="AA19" s="21">
+        <f>AVERAGE(C19:X19)</f>
+        <v>197.83842105263156</v>
+      </c>
+      <c r="AB19" s="21">
+        <f>AVERAGE(Q19:X19)</f>
+        <v>234.0625</v>
+      </c>
+      <c r="AC19" s="22">
+        <f>(AB19/AA19)-1</f>
+        <v>0.18309931283636582</v>
+      </c>
+      <c r="AD19" s="22">
+        <f>(AB19/Y19)-1</f>
+        <v>0.61422413793103448</v>
+      </c>
+      <c r="AE19" s="22">
         <f>(Z19/Y19)-1</f>
-        <v>0.21510800006862629</v>
-      </c>
-      <c r="AB19" s="21">
-        <f>(Z19/W19)-1</f>
-        <v>0.62816091954023001</v>
-      </c>
-      <c r="AC19" s="21">
-        <f>(X19/W19)-1</f>
         <v>0.63931034482758609</v>
       </c>
-      <c r="AD19" s="22" t="s">
+      <c r="AF19" s="23" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2679,22 +2769,22 @@
       <c r="I20" s="17">
         <v>180</v>
       </c>
-      <c r="J20" s="24">
+      <c r="J20" s="25">
         <v>176.91999999999999</v>
       </c>
-      <c r="K20" s="24">
+      <c r="K20" s="25">
         <v>176.91999999999999</v>
       </c>
-      <c r="L20" s="24">
+      <c r="L20" s="25">
         <v>176.91999999999999</v>
       </c>
-      <c r="M20" s="24">
+      <c r="M20" s="25">
         <v>176.91999999999999</v>
       </c>
-      <c r="N20" s="24">
+      <c r="N20" s="25">
         <v>179</v>
       </c>
-      <c r="O20" s="24">
+      <c r="O20" s="25">
         <v>180</v>
       </c>
       <c r="P20" s="18">
@@ -2718,74 +2808,80 @@
       <c r="V20" s="17">
         <v>229.94999999999999</v>
       </c>
-      <c r="W20" s="19">
-        <f>MIN(C20:V20)</f>
+      <c r="W20" s="17">
+        <v>229.94</v>
+      </c>
+      <c r="X20" s="17">
+        <v>230</v>
+      </c>
+      <c r="Y20" s="20">
+        <f>MIN(C20:X20)</f>
         <v>176.91999999999999</v>
       </c>
-      <c r="X20" s="20">
-        <f>MAX(C20:V20)</f>
-        <v>229.94999999999999</v>
-      </c>
-      <c r="Y20" s="20">
-        <f>AVERAGE(C20:V20)</f>
-        <v>191.38866666666667</v>
-      </c>
-      <c r="Z20" s="20">
-        <f>AVERAGE(Q20:V20)</f>
-        <v>213.44999999999999</v>
+      <c r="Z20" s="21">
+        <f>MAX(C20:X20)</f>
+        <v>230</v>
       </c>
       <c r="AA20" s="21">
+        <f>AVERAGE(C20:X20)</f>
+        <v>195.92764705882354</v>
+      </c>
+      <c r="AB20" s="21">
+        <f>AVERAGE(Q20:X20)</f>
+        <v>218.17000000000002</v>
+      </c>
+      <c r="AC20" s="22">
+        <f>(AB20/AA20)-1</f>
+        <v>0.11352329941725192</v>
+      </c>
+      <c r="AD20" s="22">
+        <f>(AB20/Y20)-1</f>
+        <v>0.23315622880397946</v>
+      </c>
+      <c r="AE20" s="22">
         <f>(Z20/Y20)-1</f>
-        <v>0.11526980002298992</v>
-      </c>
-      <c r="AB20" s="21">
-        <f>(Z20/W20)-1</f>
-        <v>0.20647750395659048</v>
-      </c>
-      <c r="AC20" s="21">
-        <f>(X20/W20)-1</f>
-        <v>0.29973999547818231</v>
-      </c>
-      <c r="AD20" s="22" t="s">
+        <v>0.30002260908885381</v>
+      </c>
+      <c r="AF20" s="23" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="21" ht="18">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28">
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29">
         <v>396.77999999999997</v>
       </c>
-      <c r="H21" s="28">
+      <c r="H21" s="29">
         <v>396.77999999999997</v>
       </c>
-      <c r="I21" s="28" t="s">
+      <c r="I21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="J21" s="28" t="s">
+      <c r="J21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K21" s="28" t="s">
+      <c r="K21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="L21" s="28" t="s">
+      <c r="L21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="M21" s="28" t="s">
+      <c r="M21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="N21" s="28" t="s">
+      <c r="N21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="O21" s="28" t="s">
+      <c r="O21" s="29" t="s">
         <v>43</v>
       </c>
       <c r="P21" s="17" t="s">
@@ -2809,35 +2905,41 @@
       <c r="V21" s="17">
         <v>453.04000000000002</v>
       </c>
-      <c r="W21" s="19">
-        <f>MIN(C21:V21)</f>
-        <v>396.77999999999997</v>
-      </c>
-      <c r="X21" s="20">
-        <f>MAX(C21:V21)</f>
+      <c r="W21" s="17">
         <v>453.04000000000002</v>
       </c>
+      <c r="X21" s="17">
+        <v>349</v>
+      </c>
       <c r="Y21" s="20">
-        <f>AVERAGE(C21:V21)</f>
-        <v>420.24833333333328</v>
-      </c>
-      <c r="Z21" s="20">
-        <f>AVERAGE(Q21:V21)</f>
-        <v>431.98249999999996</v>
+        <f>MIN(C21:X21)</f>
+        <v>349</v>
+      </c>
+      <c r="Z21" s="21">
+        <f>MAX(C21:X21)</f>
+        <v>453.04000000000002</v>
       </c>
       <c r="AA21" s="21">
+        <f>AVERAGE(C21:X21)</f>
+        <v>415.44124999999997</v>
+      </c>
+      <c r="AB21" s="21">
+        <f>AVERAGE(Q21:X21)</f>
+        <v>421.66166666666663</v>
+      </c>
+      <c r="AC21" s="22">
+        <f>(AB21/AA21)-1</f>
+        <v>1.4973035697987802e-002</v>
+      </c>
+      <c r="AD21" s="22">
+        <f>(AB21/Y21)-1</f>
+        <v>0.20819961795606479</v>
+      </c>
+      <c r="AE21" s="22">
         <f>(Z21/Y21)-1</f>
-        <v>2.792198263725032e-002</v>
-      </c>
-      <c r="AB21" s="21">
-        <f>(Z21/W21)-1</f>
-        <v>8.8720449619436481e-002</v>
-      </c>
-      <c r="AC21" s="21">
-        <f>(X21/W21)-1</f>
-        <v>0.14179142093855557</v>
-      </c>
-      <c r="AD21" s="32" t="s">
+        <v>0.29810888252148993</v>
+      </c>
+      <c r="AF21" s="32" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2900,35 +3002,41 @@
       <c r="V22" s="17">
         <v>600</v>
       </c>
-      <c r="W22" s="19">
-        <f>MIN(C22:V22)</f>
+      <c r="W22" s="17">
+        <v>600</v>
+      </c>
+      <c r="X22" s="17">
+        <v>600</v>
+      </c>
+      <c r="Y22" s="20">
+        <f>MIN(C22:X22)</f>
         <v>550</v>
       </c>
-      <c r="X22" s="20">
-        <f>MAX(C22:V22)</f>
+      <c r="Z22" s="21">
+        <f>MAX(C22:X22)</f>
         <v>600</v>
       </c>
-      <c r="Y22" s="20">
-        <f>AVERAGE(C22:V22)</f>
-        <v>567.5</v>
-      </c>
-      <c r="Z22" s="20">
-        <f>AVERAGE(Q22:V22)</f>
-        <v>596.66666666666663</v>
-      </c>
       <c r="AA22" s="21">
+        <f>AVERAGE(C22:X22)</f>
+        <v>571.11111111111109</v>
+      </c>
+      <c r="AB22" s="21">
+        <f>AVERAGE(Q22:X22)</f>
+        <v>597.5</v>
+      </c>
+      <c r="AC22" s="22">
+        <f>(AB22/AA22)-1</f>
+        <v>4.620622568093391e-002</v>
+      </c>
+      <c r="AD22" s="22">
+        <f>(AB22/Y22)-1</f>
+        <v>8.636363636363642e-002</v>
+      </c>
+      <c r="AE22" s="22">
         <f>(Z22/Y22)-1</f>
-        <v>5.1395007342143861e-002</v>
-      </c>
-      <c r="AB22" s="21">
-        <f>(Z22/W22)-1</f>
-        <v>8.4848484848484729e-002</v>
-      </c>
-      <c r="AC22" s="21">
-        <f>(X22/W22)-1</f>
         <v>9.0909090909090828e-002</v>
       </c>
-      <c r="AD22" s="22" t="s">
+      <c r="AF22" s="23" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2943,7 +3051,7 @@
       <c r="D23" s="17"/>
       <c r="E23" s="17"/>
       <c r="F23" s="17"/>
-      <c r="G23" s="24">
+      <c r="G23" s="25">
         <v>329</v>
       </c>
       <c r="H23" s="17">
@@ -2992,34 +3100,40 @@
         <v>518</v>
       </c>
       <c r="W23" s="19">
-        <f>MIN(C23:V23)</f>
+        <v>549</v>
+      </c>
+      <c r="X23" s="19">
+        <v>549</v>
+      </c>
+      <c r="Y23" s="20">
+        <f>MIN(C23:X23)</f>
         <v>329</v>
       </c>
-      <c r="X23" s="20">
-        <f>MAX(C23:V23)</f>
-        <v>529.95000000000005</v>
-      </c>
-      <c r="Y23" s="20">
-        <f>AVERAGE(C23:V23)</f>
-        <v>470.79687499999994</v>
-      </c>
-      <c r="Z23" s="20">
-        <f>AVERAGE(Q23:V23)</f>
-        <v>516.30833333333339</v>
+      <c r="Z23" s="21">
+        <f>MAX(C23:X23)</f>
+        <v>549</v>
       </c>
       <c r="AA23" s="21">
+        <f>AVERAGE(C23:X23)</f>
+        <v>479.48611111111109</v>
+      </c>
+      <c r="AB23" s="21">
+        <f>AVERAGE(Q23:X23)</f>
+        <v>524.48125000000005</v>
+      </c>
+      <c r="AC23" s="22">
+        <f>(AB23/AA23)-1</f>
+        <v>9.3840338325174688e-002</v>
+      </c>
+      <c r="AD23" s="22">
+        <f>(AB23/Y23)-1</f>
+        <v>0.59416793313069927</v>
+      </c>
+      <c r="AE23" s="22">
         <f>(Z23/Y23)-1</f>
-        <v>9.6668989855409393e-002</v>
-      </c>
-      <c r="AB23" s="21">
-        <f>(Z23/W23)-1</f>
-        <v>0.56932624113475194</v>
-      </c>
-      <c r="AC23" s="21">
-        <f>(X23/W23)-1</f>
-        <v>0.61079027355623117</v>
-      </c>
-      <c r="AD23" s="22" t="s">
+        <v>0.66869300911854102</v>
+      </c>
+      <c r="AF23" s="23" t="s">
         <v>79</v>
       </c>
     </row>
@@ -3034,7 +3148,7 @@
       <c r="D24" s="17"/>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
-      <c r="G24" s="24">
+      <c r="G24" s="25">
         <v>371.14999999999998</v>
       </c>
       <c r="H24" s="17">
@@ -3070,7 +3184,7 @@
       <c r="R24" s="18">
         <v>504.73000000000002</v>
       </c>
-      <c r="S24" s="18">
+      <c r="S24" s="19">
         <v>513.71000000000004</v>
       </c>
       <c r="T24" s="18">
@@ -3082,78 +3196,84 @@
       <c r="V24" s="18">
         <v>435.14999999999998</v>
       </c>
-      <c r="W24" s="19">
-        <f>MIN(C24:V24)</f>
+      <c r="W24" s="18">
+        <v>483.99000000000001</v>
+      </c>
+      <c r="X24" s="18">
+        <v>435.14999999999998</v>
+      </c>
+      <c r="Y24" s="20">
+        <f>MIN(C24:X24)</f>
         <v>371.14999999999998</v>
       </c>
-      <c r="X24" s="20">
-        <f>MAX(C24:V24)</f>
+      <c r="Z24" s="21">
+        <f>MAX(C24:X24)</f>
         <v>513.71000000000004</v>
       </c>
-      <c r="Y24" s="20">
-        <f>AVERAGE(C24:V24)</f>
-        <v>443.55937499999993</v>
-      </c>
-      <c r="Z24" s="20">
-        <f>AVERAGE(Q24:V24)</f>
-        <v>479.70499999999998</v>
-      </c>
       <c r="AA24" s="21">
+        <f>AVERAGE(C24:X24)</f>
+        <v>445.33833333333325</v>
+      </c>
+      <c r="AB24" s="21">
+        <f>AVERAGE(Q24:X24)</f>
+        <v>474.67125000000004</v>
+      </c>
+      <c r="AC24" s="22">
+        <f>(AB24/AA24)-1</f>
+        <v>6.5866588324233089e-002</v>
+      </c>
+      <c r="AD24" s="22">
+        <f>(AB24/Y24)-1</f>
+        <v>0.27892024787821645</v>
+      </c>
+      <c r="AE24" s="22">
         <f>(Z24/Y24)-1</f>
-        <v>8.1489935817499193e-002</v>
-      </c>
-      <c r="AB24" s="21">
-        <f>(Z24/W24)-1</f>
-        <v>0.29248282365620382</v>
-      </c>
-      <c r="AC24" s="21">
-        <f>(X24/W24)-1</f>
         <v>0.38410346221204383</v>
       </c>
-      <c r="AD24" s="22" t="s">
+      <c r="AF24" s="23" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="25" ht="36">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28">
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29">
         <v>433.49000000000001</v>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="25">
         <v>396</v>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="29">
         <v>541.24000000000001</v>
       </c>
-      <c r="H25" s="28">
+      <c r="H25" s="29">
         <v>531.65999999999997</v>
       </c>
-      <c r="I25" s="28">
+      <c r="I25" s="29">
         <v>524.17999999999995</v>
       </c>
-      <c r="J25" s="28">
+      <c r="J25" s="29">
         <v>519.91999999999996</v>
       </c>
-      <c r="K25" s="28">
+      <c r="K25" s="29">
         <v>519.74000000000001</v>
       </c>
-      <c r="L25" s="28">
+      <c r="L25" s="29">
         <v>429.80000000000001</v>
       </c>
-      <c r="M25" s="28">
+      <c r="M25" s="29">
         <v>534.13</v>
       </c>
-      <c r="N25" s="28">
+      <c r="N25" s="29">
         <v>525.30999999999995</v>
       </c>
-      <c r="O25" s="28">
+      <c r="O25" s="29">
         <v>524.61000000000001</v>
       </c>
       <c r="P25" s="17">
@@ -3177,35 +3297,41 @@
       <c r="V25" s="30">
         <v>609.25</v>
       </c>
-      <c r="W25" s="19">
-        <f>MIN(C25:V25)</f>
+      <c r="W25" s="33">
+        <v>587.11000000000001</v>
+      </c>
+      <c r="X25" s="33">
+        <v>587.11000000000001</v>
+      </c>
+      <c r="Y25" s="20">
+        <f>MIN(C25:X25)</f>
         <v>396</v>
       </c>
-      <c r="X25" s="20">
-        <f>MAX(C25:V25)</f>
+      <c r="Z25" s="21">
+        <f>MAX(C25:X25)</f>
         <v>609.25</v>
       </c>
-      <c r="Y25" s="20">
-        <f>AVERAGE(C25:V25)</f>
-        <v>521.28999999999996</v>
-      </c>
-      <c r="Z25" s="20">
-        <f>AVERAGE(Q25:V25)</f>
-        <v>555.745</v>
-      </c>
       <c r="AA25" s="21">
+        <f>AVERAGE(C25:X25)</f>
+        <v>527.87200000000007</v>
+      </c>
+      <c r="AB25" s="21">
+        <f>AVERAGE(Q25:X25)</f>
+        <v>563.58624999999995</v>
+      </c>
+      <c r="AC25" s="22">
+        <f>(AB25/AA25)-1</f>
+        <v>6.7657026703443091e-002</v>
+      </c>
+      <c r="AD25" s="22">
+        <f>(AB25/Y25)-1</f>
+        <v>0.42319760101010084</v>
+      </c>
+      <c r="AE25" s="22">
         <f>(Z25/Y25)-1</f>
-        <v>6.6095647336415597e-002</v>
-      </c>
-      <c r="AB25" s="21">
-        <f>(Z25/W25)-1</f>
-        <v>0.40339646464646473</v>
-      </c>
-      <c r="AC25" s="21">
-        <f>(X25/W25)-1</f>
         <v>0.53851010101010099</v>
       </c>
-      <c r="AD25" s="22" t="s">
+      <c r="AF25" s="23" t="s">
         <v>84</v>
       </c>
     </row>
@@ -3217,7 +3343,7 @@
         <v>85</v>
       </c>
       <c r="C26" s="17"/>
-      <c r="D26" s="24">
+      <c r="D26" s="25">
         <v>381.82999999999998</v>
       </c>
       <c r="E26" s="17"/>
@@ -3246,59 +3372,65 @@
       <c r="N26" s="18">
         <v>988.74000000000001</v>
       </c>
-      <c r="O26" s="29">
+      <c r="O26" s="19">
         <v>1543.1300000000001</v>
       </c>
-      <c r="P26" s="29">
+      <c r="P26" s="19">
         <v>1552.5699999999999</v>
       </c>
-      <c r="Q26" s="29">
+      <c r="Q26" s="19">
         <v>1542.1700000000001</v>
       </c>
-      <c r="R26" s="29">
+      <c r="R26" s="19">
         <v>1398</v>
       </c>
-      <c r="S26" s="29">
+      <c r="S26" s="19">
         <v>1534.8399999999999</v>
       </c>
-      <c r="T26" s="33">
+      <c r="T26" s="34">
         <v>370</v>
       </c>
       <c r="U26" s="30">
         <v>1655.4000000000001</v>
       </c>
-      <c r="V26" s="34">
+      <c r="V26" s="35">
         <v>700</v>
       </c>
-      <c r="W26" s="19">
-        <f>MIN(C26:V26)</f>
+      <c r="W26" s="30">
+        <v>1678.0799999999999</v>
+      </c>
+      <c r="X26" s="30">
+        <v>1565.48</v>
+      </c>
+      <c r="Y26" s="20">
+        <f>MIN(C26:X26)</f>
         <v>370</v>
       </c>
-      <c r="X26" s="20">
-        <f>MAX(C26:V26)</f>
-        <v>1655.4000000000001</v>
-      </c>
-      <c r="Y26" s="20">
-        <f>AVERAGE(C26:V26)</f>
-        <v>1091.3435294117646</v>
-      </c>
-      <c r="Z26" s="20">
-        <f>AVERAGE(Q26:V26)</f>
-        <v>1200.0683333333334</v>
+      <c r="Z26" s="21">
+        <f>MAX(C26:X26)</f>
+        <v>1678.0799999999999</v>
       </c>
       <c r="AA26" s="21">
+        <f>AVERAGE(C26:X26)</f>
+        <v>1147.1789473684209</v>
+      </c>
+      <c r="AB26" s="21">
+        <f>AVERAGE(Q26:X26)</f>
+        <v>1305.4962499999999</v>
+      </c>
+      <c r="AC26" s="22">
+        <f>(AB26/AA26)-1</f>
+        <v>0.13800576012552535</v>
+      </c>
+      <c r="AD26" s="22">
+        <f>(AB26/Y26)-1</f>
+        <v>2.5283682432432428</v>
+      </c>
+      <c r="AE26" s="22">
         <f>(Z26/Y26)-1</f>
-        <v>9.962472951131307e-002</v>
-      </c>
-      <c r="AB26" s="21">
-        <f>(Z26/W26)-1</f>
-        <v>2.2434279279279279</v>
-      </c>
-      <c r="AC26" s="21">
-        <f>(X26/W26)-1</f>
-        <v>3.4740540540540543</v>
-      </c>
-      <c r="AD26" s="22" t="s">
+        <v>3.535351351351351</v>
+      </c>
+      <c r="AF26" s="23" t="s">
         <v>86</v>
       </c>
     </row>
@@ -3344,75 +3476,81 @@
       <c r="S27" s="18">
         <v>149.99000000000001</v>
       </c>
-      <c r="T27" s="29">
+      <c r="T27" s="19">
         <v>159.99000000000001</v>
       </c>
-      <c r="U27" s="29">
+      <c r="U27" s="19">
         <v>159.99000000000001</v>
       </c>
-      <c r="V27" s="29">
+      <c r="V27" s="19">
         <v>164.99000000000001</v>
       </c>
       <c r="W27" s="19">
-        <f>MIN(C27:V27)</f>
+        <v>164.99000000000001</v>
+      </c>
+      <c r="X27" s="19">
+        <v>164.99000000000001</v>
+      </c>
+      <c r="Y27" s="20">
+        <f>MIN(C27:X27)</f>
         <v>109.98999999999999</v>
       </c>
-      <c r="X27" s="20">
-        <f>MAX(C27:V27)</f>
+      <c r="Z27" s="21">
+        <f>MAX(C27:X27)</f>
         <v>165.72999999999999</v>
       </c>
-      <c r="Y27" s="20">
-        <f>AVERAGE(C27:V27)</f>
-        <v>143.38500000000002</v>
-      </c>
-      <c r="Z27" s="20">
-        <f>AVERAGE(Q27:V27)</f>
-        <v>155.82333333333335</v>
-      </c>
       <c r="AA27" s="21">
+        <f>AVERAGE(C27:X27)</f>
+        <v>146.47142857142859</v>
+      </c>
+      <c r="AB27" s="21">
+        <f>AVERAGE(Q27:X27)</f>
+        <v>158.11500000000001</v>
+      </c>
+      <c r="AC27" s="22">
+        <f>(AB27/AA27)-1</f>
+        <v>7.94938066907247e-002</v>
+      </c>
+      <c r="AD27" s="22">
+        <f>(AB27/Y27)-1</f>
+        <v>0.43753977634330399</v>
+      </c>
+      <c r="AE27" s="22">
         <f>(Z27/Y27)-1</f>
-        <v>8.6747800211551596e-002</v>
-      </c>
-      <c r="AB27" s="21">
-        <f>(Z27/W27)-1</f>
-        <v>0.41670454889838493</v>
-      </c>
-      <c r="AC27" s="21">
-        <f>(X27/W27)-1</f>
         <v>0.50677334303118471</v>
       </c>
-      <c r="AD27" s="22" t="s">
+      <c r="AF27" s="23" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="28" ht="18">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="28"/>
-      <c r="K28" s="28">
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29">
         <v>69</v>
       </c>
-      <c r="L28" s="28">
+      <c r="L28" s="29">
         <v>68</v>
       </c>
-      <c r="M28" s="28">
+      <c r="M28" s="29">
         <v>80.060000000000002</v>
       </c>
-      <c r="N28" s="28">
+      <c r="N28" s="29">
         <v>74.560000000000002</v>
       </c>
-      <c r="O28" s="28">
+      <c r="O28" s="29">
         <v>76.189999999999998</v>
       </c>
       <c r="P28" s="17">
@@ -3436,35 +3574,41 @@
       <c r="V28" s="18">
         <v>85.700000000000003</v>
       </c>
-      <c r="W28" s="19">
-        <f>MIN(C28:V28)</f>
+      <c r="W28" s="18">
+        <v>82</v>
+      </c>
+      <c r="X28" s="18">
+        <v>82.890000000000001</v>
+      </c>
+      <c r="Y28" s="20">
+        <f>MIN(C28:X28)</f>
         <v>68</v>
       </c>
-      <c r="X28" s="20">
-        <f>MAX(C28:V28)</f>
+      <c r="Z28" s="21">
+        <f>MAX(C28:X28)</f>
         <v>85.700000000000003</v>
       </c>
-      <c r="Y28" s="20">
-        <f>AVERAGE(C28:V28)</f>
-        <v>77.984999999999999</v>
-      </c>
-      <c r="Z28" s="20">
-        <f>AVERAGE(Q28:V28)</f>
-        <v>82.170000000000002</v>
-      </c>
       <c r="AA28" s="21">
+        <f>AVERAGE(C28:X28)</f>
+        <v>78.622142857142862</v>
+      </c>
+      <c r="AB28" s="21">
+        <f>AVERAGE(Q28:X28)</f>
+        <v>82.238749999999996</v>
+      </c>
+      <c r="AC28" s="22">
+        <f>(AB28/AA28)-1</f>
+        <v>4.5999854639278137e-002</v>
+      </c>
+      <c r="AD28" s="22">
+        <f>(AB28/Y28)-1</f>
+        <v>0.20939338235294103</v>
+      </c>
+      <c r="AE28" s="22">
         <f>(Z28/Y28)-1</f>
-        <v>5.3664166185805051e-002</v>
-      </c>
-      <c r="AB28" s="21">
-        <f>(Z28/W28)-1</f>
-        <v>0.20838235294117657</v>
-      </c>
-      <c r="AC28" s="21">
-        <f>(X28/W28)-1</f>
         <v>0.26029411764705879</v>
       </c>
-      <c r="AD28" s="22" t="s">
+      <c r="AF28" s="23" t="s">
         <v>90</v>
       </c>
     </row>
@@ -3516,38 +3660,44 @@
       <c r="U29" s="30">
         <v>111</v>
       </c>
-      <c r="V29" s="33">
+      <c r="V29" s="34">
         <v>65.530000000000001</v>
       </c>
-      <c r="W29" s="19">
-        <f>MIN(C29:V29)</f>
+      <c r="W29" s="33">
+        <v>99.989999999999995</v>
+      </c>
+      <c r="X29" s="30">
+        <v>107</v>
+      </c>
+      <c r="Y29" s="20">
+        <f>MIN(C29:X29)</f>
         <v>55</v>
       </c>
-      <c r="X29" s="20">
-        <f>MAX(C29:V29)</f>
+      <c r="Z29" s="21">
+        <f>MAX(C29:X29)</f>
         <v>111</v>
       </c>
-      <c r="Y29" s="20">
-        <f>AVERAGE(C29:V29)</f>
-        <v>81.845833333333346</v>
-      </c>
-      <c r="Z29" s="20">
-        <f>AVERAGE(Q29:V29)</f>
-        <v>92.064999999999998</v>
-      </c>
       <c r="AA29" s="21">
+        <f>AVERAGE(C29:X29)</f>
+        <v>84.938571428571436</v>
+      </c>
+      <c r="AB29" s="21">
+        <f>AVERAGE(Q29:X29)</f>
+        <v>94.922499999999999</v>
+      </c>
+      <c r="AC29" s="22">
+        <f>(AB29/AA29)-1</f>
+        <v>0.11754293018483941</v>
+      </c>
+      <c r="AD29" s="22">
+        <f>(AB29/Y29)-1</f>
+        <v>0.72586363636363638</v>
+      </c>
+      <c r="AE29" s="22">
         <f>(Z29/Y29)-1</f>
-        <v>0.12485872830015765</v>
-      </c>
-      <c r="AB29" s="21">
-        <f>(Z29/W29)-1</f>
-        <v>0.67390909090909079</v>
-      </c>
-      <c r="AC29" s="21">
-        <f>(X29/W29)-1</f>
         <v>1.0181818181818181</v>
       </c>
-      <c r="AD29" s="22" t="s">
+      <c r="AF29" s="23" t="s">
         <v>92</v>
       </c>
     </row>
@@ -3591,73 +3741,79 @@
       <c r="S30" s="18">
         <v>90.579999999999998</v>
       </c>
-      <c r="T30" s="29">
+      <c r="T30" s="19">
         <v>100.68000000000001</v>
       </c>
-      <c r="U30" s="29">
+      <c r="U30" s="19">
         <v>92.530000000000001</v>
       </c>
       <c r="V30" s="18">
         <v>89.090000000000003</v>
       </c>
-      <c r="W30" s="19">
-        <f>MIN(C30:V30)</f>
+      <c r="W30" s="18">
+        <v>86.700000000000003</v>
+      </c>
+      <c r="X30" s="18">
+        <v>86.700000000000003</v>
+      </c>
+      <c r="Y30" s="20">
+        <f>MIN(C30:X30)</f>
         <v>47.359999999999999</v>
       </c>
-      <c r="X30" s="20">
-        <f>MAX(C30:V30)</f>
+      <c r="Z30" s="21">
+        <f>MAX(C30:X30)</f>
         <v>100.68000000000001</v>
       </c>
-      <c r="Y30" s="20">
-        <f>AVERAGE(C30:V30)</f>
-        <v>71.191818181818178</v>
-      </c>
-      <c r="Z30" s="20">
-        <f>AVERAGE(Q30:V30)</f>
-        <v>85.110000000000014</v>
-      </c>
       <c r="AA30" s="21">
+        <f>AVERAGE(C30:X30)</f>
+        <v>73.577692307692317</v>
+      </c>
+      <c r="AB30" s="21">
+        <f>AVERAGE(Q30:X30)</f>
+        <v>85.507500000000022</v>
+      </c>
+      <c r="AC30" s="22">
+        <f>(AB30/AA30)-1</f>
+        <v>0.16213892170494826</v>
+      </c>
+      <c r="AD30" s="22">
+        <f>(AB30/Y30)-1</f>
+        <v>0.8054793074324329</v>
+      </c>
+      <c r="AE30" s="22">
         <f>(Z30/Y30)-1</f>
-        <v>0.19550254753482932</v>
-      </c>
-      <c r="AB30" s="21">
-        <f>(Z30/W30)-1</f>
-        <v>0.79708614864864891</v>
-      </c>
-      <c r="AC30" s="21">
-        <f>(X30/W30)-1</f>
         <v>1.1258445945945947</v>
       </c>
-      <c r="AD30" s="22" t="s">
+      <c r="AF30" s="23" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="31" ht="18">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28">
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="29"/>
+      <c r="L31" s="29">
         <v>92.5</v>
       </c>
-      <c r="M31" s="28">
+      <c r="M31" s="29">
         <v>110.91</v>
       </c>
-      <c r="N31" s="28">
+      <c r="N31" s="29">
         <v>107.04000000000001</v>
       </c>
-      <c r="O31" s="28">
+      <c r="O31" s="29">
         <v>112</v>
       </c>
       <c r="P31" s="17">
@@ -3681,35 +3837,41 @@
       <c r="V31" s="18">
         <v>156</v>
       </c>
-      <c r="W31" s="19">
-        <f>MIN(C31:V31)</f>
+      <c r="W31" s="18">
+        <v>156</v>
+      </c>
+      <c r="X31" s="18">
+        <v>156</v>
+      </c>
+      <c r="Y31" s="20">
+        <f>MIN(C31:X31)</f>
         <v>92.5</v>
       </c>
-      <c r="X31" s="20">
-        <f>MAX(C31:V31)</f>
+      <c r="Z31" s="21">
+        <f>MAX(C31:X31)</f>
         <v>156</v>
       </c>
-      <c r="Y31" s="20">
-        <f>AVERAGE(C31:V31)</f>
-        <v>119.66800000000003</v>
-      </c>
-      <c r="Z31" s="20">
-        <f>AVERAGE(Q31:V31)</f>
-        <v>133.43800000000002</v>
-      </c>
       <c r="AA31" s="21">
+        <f>AVERAGE(C31:X31)</f>
+        <v>125.72333333333336</v>
+      </c>
+      <c r="AB31" s="21">
+        <f>AVERAGE(Q31:X31)</f>
+        <v>139.88428571428571</v>
+      </c>
+      <c r="AC31" s="22">
+        <f>(AB31/AA31)-1</f>
+        <v>0.11263583302716818</v>
+      </c>
+      <c r="AD31" s="22">
+        <f>(AB31/Y31)-1</f>
+        <v>0.51226254826254825</v>
+      </c>
+      <c r="AE31" s="22">
         <f>(Z31/Y31)-1</f>
-        <v>0.11506835578433638</v>
-      </c>
-      <c r="AB31" s="21">
-        <f>(Z31/W31)-1</f>
-        <v>0.44257297297297304</v>
-      </c>
-      <c r="AC31" s="21">
-        <f>(X31/W31)-1</f>
         <v>0.68648648648648658</v>
       </c>
-      <c r="AD31" s="22" t="s">
+      <c r="AF31" s="23" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3736,7 +3898,7 @@
       <c r="N32" s="17">
         <v>165.36000000000001</v>
       </c>
-      <c r="O32" s="29">
+      <c r="O32" s="19">
         <v>241.99000000000001</v>
       </c>
       <c r="P32" s="18">
@@ -3745,7 +3907,7 @@
       <c r="Q32" s="18">
         <v>224.84999999999999</v>
       </c>
-      <c r="R32" s="29">
+      <c r="R32" s="19">
         <v>257.87</v>
       </c>
       <c r="S32" s="18">
@@ -3760,35 +3922,41 @@
       <c r="V32" s="18">
         <v>238.24000000000001</v>
       </c>
-      <c r="W32" s="19">
-        <f>MIN(C32:V32)</f>
+      <c r="W32" s="18">
+        <v>235.97999999999999</v>
+      </c>
+      <c r="X32" s="18">
+        <v>238.24000000000001</v>
+      </c>
+      <c r="Y32" s="20">
+        <f>MIN(C32:X32)</f>
         <v>148.88</v>
       </c>
-      <c r="X32" s="20">
-        <f>MAX(C32:V32)</f>
+      <c r="Z32" s="21">
+        <f>MAX(C32:X32)</f>
         <v>257.87</v>
       </c>
-      <c r="Y32" s="20">
-        <f>AVERAGE(C32:V32)</f>
-        <v>219.03500000000003</v>
-      </c>
-      <c r="Z32" s="20">
-        <f>AVERAGE(Q32:V32)</f>
-        <v>234.87833333333336</v>
-      </c>
       <c r="AA32" s="21">
+        <f>AVERAGE(C32:X32)</f>
+        <v>222.04750000000004</v>
+      </c>
+      <c r="AB32" s="21">
+        <f>AVERAGE(Q32:X32)</f>
+        <v>235.43625000000003</v>
+      </c>
+      <c r="AC32" s="22">
+        <f>(AB32/AA32)-1</f>
+        <v>6.0296783345905602e-002</v>
+      </c>
+      <c r="AD32" s="22">
+        <f>(AB32/Y32)-1</f>
+        <v>0.58138265717356274</v>
+      </c>
+      <c r="AE32" s="22">
         <f>(Z32/Y32)-1</f>
-        <v>7.2332427846386826e-002</v>
-      </c>
-      <c r="AB32" s="21">
-        <f>(Z32/W32)-1</f>
-        <v>0.57763523195414668</v>
-      </c>
-      <c r="AC32" s="21">
-        <f>(X32/W32)-1</f>
         <v>0.73206609349811935</v>
       </c>
-      <c r="AD32" s="22" t="s">
+      <c r="AF32" s="23" t="s">
         <v>98</v>
       </c>
     </row>
@@ -3835,58 +4003,64 @@
       <c r="V33" s="18">
         <v>164.93000000000001</v>
       </c>
-      <c r="W33" s="19">
-        <f>MIN(C33:V33)</f>
+      <c r="W33" s="18">
+        <v>161.65000000000001</v>
+      </c>
+      <c r="X33" s="18">
+        <v>164.38999999999999</v>
+      </c>
+      <c r="Y33" s="20">
+        <f>MIN(C33:X33)</f>
         <v>144.94999999999999</v>
       </c>
-      <c r="X33" s="20">
-        <f>MAX(C33:V33)</f>
+      <c r="Z33" s="21">
+        <f>MAX(C33:X33)</f>
         <v>164.93000000000001</v>
       </c>
-      <c r="Y33" s="20">
-        <f>AVERAGE(C33:V33)</f>
-        <v>153.7225</v>
-      </c>
-      <c r="Z33" s="20">
-        <f>AVERAGE(Q33:V33)</f>
-        <v>153.55666666666664</v>
-      </c>
       <c r="AA33" s="21">
+        <f>AVERAGE(C33:X33)</f>
+        <v>155.58200000000002</v>
+      </c>
+      <c r="AB33" s="21">
+        <f>AVERAGE(Q33:X33)</f>
+        <v>155.92250000000001</v>
+      </c>
+      <c r="AC33" s="22">
+        <f>(AB33/AA33)-1</f>
+        <v>2.1885565168207055e-003</v>
+      </c>
+      <c r="AD33" s="22">
+        <f>(AB33/Y33)-1</f>
+        <v>7.5698516729907128e-002</v>
+      </c>
+      <c r="AE33" s="22">
         <f>(Z33/Y33)-1</f>
-        <v>-1.0787837390970889e-003</v>
-      </c>
-      <c r="AB33" s="21">
-        <f>(Z33/W33)-1</f>
-        <v>5.9376796596527504e-002</v>
-      </c>
-      <c r="AC33" s="21">
-        <f>(X33/W33)-1</f>
         <v>0.13784063470162145</v>
       </c>
-      <c r="AD33" s="22" t="s">
+      <c r="AF33" s="23" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="34" ht="18">
-      <c r="A34" s="25" t="s">
+      <c r="A34" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B34" s="26" t="s">
+      <c r="B34" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="C34" s="28"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="28"/>
-      <c r="F34" s="28"/>
-      <c r="G34" s="28"/>
-      <c r="H34" s="28"/>
-      <c r="I34" s="28"/>
-      <c r="J34" s="28"/>
-      <c r="K34" s="28"/>
-      <c r="L34" s="28"/>
-      <c r="M34" s="28"/>
-      <c r="N34" s="28"/>
-      <c r="O34" s="29">
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="29"/>
+      <c r="L34" s="29"/>
+      <c r="M34" s="29"/>
+      <c r="N34" s="29"/>
+      <c r="O34" s="19">
         <v>199.93000000000001</v>
       </c>
       <c r="P34" s="17">
@@ -3895,50 +4069,56 @@
       <c r="Q34" s="17">
         <v>175.99000000000001</v>
       </c>
-      <c r="R34" s="24">
+      <c r="R34" s="25">
         <v>144</v>
       </c>
-      <c r="S34" s="29">
+      <c r="S34" s="19">
         <v>199.40000000000001</v>
       </c>
-      <c r="T34" s="29">
+      <c r="T34" s="19">
         <v>189.99000000000001</v>
       </c>
-      <c r="U34" s="29">
+      <c r="U34" s="19">
         <v>199.94999999999999</v>
       </c>
       <c r="V34" s="18">
         <v>169</v>
       </c>
       <c r="W34" s="19">
-        <f>MIN(C34:V34)</f>
+        <v>181.33000000000001</v>
+      </c>
+      <c r="X34" s="18">
+        <v>169</v>
+      </c>
+      <c r="Y34" s="20">
+        <f>MIN(C34:X34)</f>
         <v>144</v>
       </c>
-      <c r="X34" s="20">
-        <f>MAX(C34:V34)</f>
+      <c r="Z34" s="21">
+        <f>MAX(C34:X34)</f>
         <v>199.94999999999999</v>
       </c>
-      <c r="Y34" s="20">
-        <f>AVERAGE(C34:V34)</f>
-        <v>180.02000000000001</v>
-      </c>
-      <c r="Z34" s="20">
-        <f>AVERAGE(Q34:V34)</f>
-        <v>179.72166666666666</v>
-      </c>
       <c r="AA34" s="21">
+        <f>AVERAGE(C34:X34)</f>
+        <v>179.04900000000001</v>
+      </c>
+      <c r="AB34" s="21">
+        <f>AVERAGE(Q34:X34)</f>
+        <v>178.58249999999998</v>
+      </c>
+      <c r="AC34" s="22">
+        <f>(AB34/AA34)-1</f>
+        <v>-2.6054320325722413e-003</v>
+      </c>
+      <c r="AD34" s="22">
+        <f>(AB34/Y34)-1</f>
+        <v>0.24015624999999985</v>
+      </c>
+      <c r="AE34" s="22">
         <f>(Z34/Y34)-1</f>
-        <v>-1.6572232714884283e-003</v>
-      </c>
-      <c r="AB34" s="21">
-        <f>(Z34/W34)-1</f>
-        <v>0.24806712962962951</v>
-      </c>
-      <c r="AC34" s="21">
-        <f>(X34/W34)-1</f>
         <v>0.38854166666666656</v>
       </c>
-      <c r="AD34" s="22" t="s">
+      <c r="AF34" s="23" t="s">
         <v>102</v>
       </c>
     </row>
@@ -3953,7 +4133,7 @@
       <c r="D35" s="17"/>
       <c r="E35" s="17"/>
       <c r="F35" s="17"/>
-      <c r="G35" s="24">
+      <c r="G35" s="25">
         <v>30731.380000000001</v>
       </c>
       <c r="H35" s="18">
@@ -3983,35 +4163,37 @@
       <c r="T35" s="17"/>
       <c r="U35" s="17"/>
       <c r="V35" s="17"/>
-      <c r="W35" s="19">
-        <f>MIN(C35:V35)</f>
+      <c r="W35" s="17"/>
+      <c r="X35" s="17"/>
+      <c r="Y35" s="20">
+        <f>MIN(C35:X35)</f>
         <v>30731.380000000001</v>
       </c>
-      <c r="X35" s="20">
-        <f>MAX(C35:V35)</f>
+      <c r="Z35" s="21">
+        <f>MAX(C35:X35)</f>
         <v>32790.889999999999</v>
       </c>
-      <c r="Y35" s="20">
-        <f>AVERAGE(C35:V35)</f>
+      <c r="AA35" s="21">
+        <f>AVERAGE(C35:X35)</f>
         <v>31912.133333333331</v>
       </c>
-      <c r="Z35" s="20" t="e">
-        <f>AVERAGE(Q35:V35)</f>
+      <c r="AB35" s="21" t="e">
+        <f>AVERAGE(Q35:X35)</f>
         <v>#NUM!</v>
       </c>
-      <c r="AA35" s="21" t="e">
+      <c r="AC35" s="22" t="e">
+        <f>(AB35/AA35)-1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD35" s="22" t="e">
+        <f>(AB35/Y35)-1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE35" s="22">
         <f>(Z35/Y35)-1</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="AB35" s="21" t="e">
-        <f>(Z35/W35)-1</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="AC35" s="21">
-        <f>(X35/W35)-1</f>
         <v>6.7016515366377982e-002</v>
       </c>
-      <c r="AD35" s="22" t="s">
+      <c r="AF35" s="23" t="s">
         <v>105</v>
       </c>
     </row>
@@ -4026,7 +4208,7 @@
       <c r="D36" s="17"/>
       <c r="E36" s="17"/>
       <c r="F36" s="17"/>
-      <c r="G36" s="24"/>
+      <c r="G36" s="25"/>
       <c r="H36" s="18"/>
       <c r="I36" s="18"/>
       <c r="J36" s="18"/>
@@ -4039,16 +4221,16 @@
       <c r="O36" s="18">
         <v>642.82000000000005</v>
       </c>
-      <c r="P36" s="29">
+      <c r="P36" s="19">
         <v>721.67999999999995</v>
       </c>
-      <c r="Q36" s="29">
+      <c r="Q36" s="19">
         <v>721.67999999999995</v>
       </c>
-      <c r="R36" s="29">
+      <c r="R36" s="19">
         <v>721.67999999999995</v>
       </c>
-      <c r="S36" s="29">
+      <c r="S36" s="19">
         <v>721.67999999999995</v>
       </c>
       <c r="T36" s="17" t="s">
@@ -4060,35 +4242,41 @@
       <c r="V36" s="17">
         <v>1150.8</v>
       </c>
-      <c r="W36" s="19">
-        <f>MIN(C36:V36)</f>
+      <c r="W36" s="17">
+        <v>1150.8</v>
+      </c>
+      <c r="X36" s="17">
+        <v>1150.8</v>
+      </c>
+      <c r="Y36" s="20">
+        <f>MIN(C36:X36)</f>
         <v>642.82000000000005</v>
       </c>
-      <c r="X36" s="20">
-        <f>MAX(C36:V36)</f>
+      <c r="Z36" s="21">
+        <f>MAX(C36:X36)</f>
         <v>1164</v>
       </c>
-      <c r="Y36" s="20">
-        <f>AVERAGE(C36:V36)</f>
-        <v>810.89499999999998</v>
-      </c>
-      <c r="Z36" s="20">
-        <f>AVERAGE(Q36:V36)</f>
-        <v>895.96800000000007</v>
-      </c>
       <c r="AA36" s="21">
+        <f>AVERAGE(C36:X36)</f>
+        <v>878.87599999999998</v>
+      </c>
+      <c r="AB36" s="21">
+        <f>AVERAGE(Q36:X36)</f>
+        <v>968.77714285714296</v>
+      </c>
+      <c r="AC36" s="22">
+        <f>(AB36/AA36)-1</f>
+        <v>0.1022910431700752</v>
+      </c>
+      <c r="AD36" s="22">
+        <f>(AB36/Y36)-1</f>
+        <v>0.50707374203842903</v>
+      </c>
+      <c r="AE36" s="22">
         <f>(Z36/Y36)-1</f>
-        <v>0.10491247325486053</v>
-      </c>
-      <c r="AB36" s="21">
-        <f>(Z36/W36)-1</f>
-        <v>0.39380853115957803</v>
-      </c>
-      <c r="AC36" s="21">
-        <f>(X36/W36)-1</f>
         <v>0.81077128900780915</v>
       </c>
-      <c r="AD36" s="22" t="s">
+      <c r="AF36" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4103,7 +4291,7 @@
       <c r="D37" s="17"/>
       <c r="E37" s="17"/>
       <c r="F37" s="17"/>
-      <c r="G37" s="24"/>
+      <c r="G37" s="25"/>
       <c r="H37" s="18"/>
       <c r="I37" s="18"/>
       <c r="J37" s="18"/>
@@ -4116,16 +4304,16 @@
       <c r="O37" s="18">
         <v>1151.71</v>
       </c>
-      <c r="P37" s="29">
+      <c r="P37" s="19">
         <v>1279.6800000000001</v>
       </c>
-      <c r="Q37" s="29">
+      <c r="Q37" s="19">
         <v>1279.6800000000001</v>
       </c>
-      <c r="R37" s="29">
+      <c r="R37" s="19">
         <v>1279.6800000000001</v>
       </c>
-      <c r="S37" s="29">
+      <c r="S37" s="19">
         <v>1279.6800000000001</v>
       </c>
       <c r="T37" s="30">
@@ -4137,35 +4325,41 @@
       <c r="V37" s="30">
         <v>2016</v>
       </c>
-      <c r="W37" s="19">
-        <f>MIN(C37:V37)</f>
+      <c r="W37" s="30">
+        <v>2016</v>
+      </c>
+      <c r="X37" s="30">
+        <v>2016</v>
+      </c>
+      <c r="Y37" s="20">
+        <f>MIN(C37:X37)</f>
         <v>1151.71</v>
       </c>
-      <c r="X37" s="20">
-        <f>MAX(C37:V37)</f>
+      <c r="Z37" s="21">
+        <f>MAX(C37:X37)</f>
         <v>2064</v>
       </c>
-      <c r="Y37" s="20">
-        <f>AVERAGE(C37:V37)</f>
-        <v>1507.348888888889</v>
-      </c>
-      <c r="Z37" s="20">
-        <f>AVERAGE(Q37:V37)</f>
-        <v>1663.8400000000001</v>
-      </c>
       <c r="AA37" s="21">
+        <f>AVERAGE(C37:X37)</f>
+        <v>1599.830909090909</v>
+      </c>
+      <c r="AB37" s="21">
+        <f>AVERAGE(Q37:X37)</f>
+        <v>1751.8800000000001</v>
+      </c>
+      <c r="AC37" s="22">
+        <f>(AB37/AA37)-1</f>
+        <v>9.5040725894895761e-002</v>
+      </c>
+      <c r="AD37" s="22">
+        <f>(AB37/Y37)-1</f>
+        <v>0.52111208550763655</v>
+      </c>
+      <c r="AE37" s="22">
         <f>(Z37/Y37)-1</f>
-        <v>0.10381877232580528</v>
-      </c>
-      <c r="AB37" s="21">
-        <f>(Z37/W37)-1</f>
-        <v>0.44466923096960187</v>
-      </c>
-      <c r="AC37" s="21">
-        <f>(X37/W37)-1</f>
         <v>0.79211780743416305</v>
       </c>
-      <c r="AD37" s="22" t="s">
+      <c r="AF37" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4180,7 +4374,7 @@
       <c r="D38" s="17"/>
       <c r="E38" s="17"/>
       <c r="F38" s="17"/>
-      <c r="G38" s="24"/>
+      <c r="G38" s="25"/>
       <c r="H38" s="18"/>
       <c r="I38" s="18"/>
       <c r="J38" s="18"/>
@@ -4193,56 +4387,62 @@
       <c r="O38" s="18">
         <v>2159.8299999999999</v>
       </c>
-      <c r="P38" s="29">
+      <c r="P38" s="19">
         <v>2403.1199999999999</v>
       </c>
-      <c r="Q38" s="29">
+      <c r="Q38" s="19">
         <v>2403.1199999999999</v>
       </c>
-      <c r="R38" s="29">
+      <c r="R38" s="19">
         <v>2403.1199999999999</v>
       </c>
-      <c r="S38" s="29">
+      <c r="S38" s="19">
         <v>2403.1199999999999</v>
       </c>
       <c r="T38" s="30">
         <v>3876</v>
       </c>
-      <c r="U38" s="35" t="s">
+      <c r="U38" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="V38" s="35" t="s">
+      <c r="V38" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="W38" s="19">
-        <f>MIN(C38:V38)</f>
+      <c r="W38" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="X38" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y38" s="20">
+        <f>MIN(C38:X38)</f>
         <v>2159.8299999999999</v>
       </c>
-      <c r="X38" s="20">
-        <f>MAX(C38:V38)</f>
+      <c r="Z38" s="21">
+        <f>MAX(C38:X38)</f>
         <v>3876</v>
       </c>
-      <c r="Y38" s="20">
-        <f>AVERAGE(C38:V38)</f>
+      <c r="AA38" s="21">
+        <f>AVERAGE(C38:X38)</f>
         <v>2544.02</v>
       </c>
-      <c r="Z38" s="20">
-        <f>AVERAGE(Q38:V38)</f>
+      <c r="AB38" s="21">
+        <f>AVERAGE(Q38:X38)</f>
         <v>2771.3400000000001</v>
       </c>
-      <c r="AA38" s="21">
+      <c r="AC38" s="22">
+        <f>(AB38/AA38)-1</f>
+        <v>8.9354643438337877e-002</v>
+      </c>
+      <c r="AD38" s="22">
+        <f>(AB38/Y38)-1</f>
+        <v>0.28312876476389359</v>
+      </c>
+      <c r="AE38" s="22">
         <f>(Z38/Y38)-1</f>
-        <v>8.9354643438337877e-002</v>
-      </c>
-      <c r="AB38" s="21">
-        <f>(Z38/W38)-1</f>
-        <v>0.28312876476389359</v>
-      </c>
-      <c r="AC38" s="21">
-        <f>(X38/W38)-1</f>
         <v>0.79458568498446636</v>
       </c>
-      <c r="AD38" s="22" t="s">
+      <c r="AF38" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4257,7 +4457,7 @@
       <c r="D39" s="17"/>
       <c r="E39" s="17"/>
       <c r="F39" s="17"/>
-      <c r="G39" s="24"/>
+      <c r="G39" s="25"/>
       <c r="H39" s="18"/>
       <c r="I39" s="18"/>
       <c r="J39" s="18"/>
@@ -4270,16 +4470,16 @@
       <c r="O39" s="18">
         <v>1320.5999999999999</v>
       </c>
-      <c r="P39" s="29">
+      <c r="P39" s="19">
         <v>1320.5999999999999</v>
       </c>
-      <c r="Q39" s="29">
+      <c r="Q39" s="19">
         <v>1320.5999999999999</v>
       </c>
-      <c r="R39" s="29">
+      <c r="R39" s="19">
         <v>1320.5999999999999</v>
       </c>
-      <c r="S39" s="29">
+      <c r="S39" s="19">
         <v>1320.5999999999999</v>
       </c>
       <c r="T39" s="30">
@@ -4291,35 +4491,41 @@
       <c r="V39" s="30">
         <v>2218.4400000000001</v>
       </c>
-      <c r="W39" s="19">
-        <f>MIN(C39:V39)</f>
+      <c r="W39" s="30">
+        <v>2218.4400000000001</v>
+      </c>
+      <c r="X39" s="30">
+        <v>2218.4400000000001</v>
+      </c>
+      <c r="Y39" s="20">
+        <f>MIN(C39:X39)</f>
         <v>1310.1800000000001</v>
       </c>
-      <c r="X39" s="20">
-        <f>MAX(C39:V39)</f>
+      <c r="Z39" s="21">
+        <f>MAX(C39:X39)</f>
         <v>2218.4400000000001</v>
       </c>
-      <c r="Y39" s="20">
-        <f>AVERAGE(C39:V39)</f>
-        <v>1599.068888888889</v>
-      </c>
-      <c r="Z39" s="20">
-        <f>AVERAGE(Q39:V39)</f>
-        <v>1740.04</v>
-      </c>
       <c r="AA39" s="21">
+        <f>AVERAGE(C39:X39)</f>
+        <v>1711.6818181818182</v>
+      </c>
+      <c r="AB39" s="21">
+        <f>AVERAGE(Q39:X39)</f>
+        <v>1859.6400000000001</v>
+      </c>
+      <c r="AC39" s="22">
+        <f>(AB39/AA39)-1</f>
+        <v>8.6440236874950171e-002</v>
+      </c>
+      <c r="AD39" s="22">
+        <f>(AB39/Y39)-1</f>
+        <v>0.41937749011586201</v>
+      </c>
+      <c r="AE39" s="22">
         <f>(Z39/Y39)-1</f>
-        <v>8.8158247646894505e-002</v>
-      </c>
-      <c r="AB39" s="21">
-        <f>(Z39/W39)-1</f>
-        <v>0.32809232319223303</v>
-      </c>
-      <c r="AC39" s="21">
-        <f>(X39/W39)-1</f>
         <v>0.69323299088674828</v>
       </c>
-      <c r="AD39" s="22" t="s">
+      <c r="AF39" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4347,44 +4553,50 @@
       <c r="Q40" s="17"/>
       <c r="R40" s="17"/>
       <c r="S40" s="17"/>
-      <c r="T40" s="29">
+      <c r="T40" s="19">
         <v>1896</v>
       </c>
-      <c r="U40" s="29">
+      <c r="U40" s="19">
         <v>1896</v>
       </c>
-      <c r="V40" s="29">
+      <c r="V40" s="19">
         <v>1592.6400000000001</v>
       </c>
       <c r="W40" s="19">
-        <f>MIN(C40:V40)</f>
         <v>1592.6400000000001</v>
       </c>
-      <c r="X40" s="20">
-        <f>MAX(C40:V40)</f>
+      <c r="X40" s="19">
+        <v>1592.6400000000001</v>
+      </c>
+      <c r="Y40" s="20">
+        <f>MIN(C40:X40)</f>
+        <v>1592.6400000000001</v>
+      </c>
+      <c r="Z40" s="21">
+        <f>MAX(C40:X40)</f>
         <v>1896</v>
       </c>
-      <c r="Y40" s="20">
-        <f>AVERAGE(C40:V40)</f>
-        <v>1794.8800000000001</v>
-      </c>
-      <c r="Z40" s="20">
-        <f>AVERAGE(Q40:V40)</f>
-        <v>1794.8800000000001</v>
-      </c>
       <c r="AA40" s="21">
+        <f>AVERAGE(C40:X40)</f>
+        <v>1713.9839999999999</v>
+      </c>
+      <c r="AB40" s="21">
+        <f>AVERAGE(Q40:X40)</f>
+        <v>1713.9839999999999</v>
+      </c>
+      <c r="AC40" s="22">
+        <f>(AB40/AA40)-1</f>
+        <v>0</v>
+      </c>
+      <c r="AD40" s="22">
+        <f>(AB40/Y40)-1</f>
+        <v>7.6190476190476142e-002</v>
+      </c>
+      <c r="AE40" s="22">
         <f>(Z40/Y40)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AB40" s="21">
-        <f>(Z40/W40)-1</f>
-        <v>0.12698412698412698</v>
-      </c>
-      <c r="AC40" s="21">
-        <f>(X40/W40)-1</f>
         <v>0.19047619047619047</v>
       </c>
-      <c r="AD40" s="22" t="s">
+      <c r="AF40" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4399,7 +4611,7 @@
       <c r="D41" s="17"/>
       <c r="E41" s="17"/>
       <c r="F41" s="17"/>
-      <c r="G41" s="24"/>
+      <c r="G41" s="25"/>
       <c r="H41" s="18"/>
       <c r="I41" s="18"/>
       <c r="J41" s="18"/>
@@ -4412,16 +4624,16 @@
       <c r="O41" s="18">
         <v>1480.5599999999999</v>
       </c>
-      <c r="P41" s="29">
+      <c r="P41" s="19">
         <v>1628.6199999999999</v>
       </c>
-      <c r="Q41" s="29">
+      <c r="Q41" s="19">
         <v>1628.6199999999999</v>
       </c>
-      <c r="R41" s="29">
+      <c r="R41" s="19">
         <v>1628.6199999999999</v>
       </c>
-      <c r="S41" s="29">
+      <c r="S41" s="19">
         <v>1628.6199999999999</v>
       </c>
       <c r="T41" s="17" t="s">
@@ -4434,34 +4646,40 @@
         <v>43</v>
       </c>
       <c r="W41" s="19">
-        <f>MIN(C41:V41)</f>
+        <v>1985.76</v>
+      </c>
+      <c r="X41" s="19">
+        <v>1985.76</v>
+      </c>
+      <c r="Y41" s="20">
+        <f>MIN(C41:X41)</f>
         <v>1480.5599999999999</v>
       </c>
-      <c r="X41" s="20">
-        <f>MAX(C41:V41)</f>
-        <v>1628.6199999999999</v>
-      </c>
-      <c r="Y41" s="20">
-        <f>AVERAGE(C41:V41)</f>
-        <v>1579.2666666666664</v>
-      </c>
-      <c r="Z41" s="20">
-        <f>AVERAGE(Q41:V41)</f>
-        <v>1628.6199999999999</v>
+      <c r="Z41" s="21">
+        <f>MAX(C41:X41)</f>
+        <v>1985.76</v>
       </c>
       <c r="AA41" s="21">
+        <f>AVERAGE(C41:X41)</f>
+        <v>1680.8899999999999</v>
+      </c>
+      <c r="AB41" s="21">
+        <f>AVERAGE(Q41:X41)</f>
+        <v>1771.4759999999999</v>
+      </c>
+      <c r="AC41" s="22">
+        <f>(AB41/AA41)-1</f>
+        <v>5.3891688331776599e-002</v>
+      </c>
+      <c r="AD41" s="22">
+        <f>(AB41/Y41)-1</f>
+        <v>0.19649051710163712</v>
+      </c>
+      <c r="AE41" s="22">
         <f>(Z41/Y41)-1</f>
-        <v>3.1250791506606479e-002</v>
-      </c>
-      <c r="AB41" s="21">
-        <f>(Z41/W41)-1</f>
-        <v>0.10000270168044523</v>
-      </c>
-      <c r="AC41" s="21">
-        <f>(X41/W41)-1</f>
-        <v>0.10000270168044523</v>
-      </c>
-      <c r="AD41" s="22" t="s">
+        <v>0.34122224023342529</v>
+      </c>
+      <c r="AF41" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4476,16 +4694,16 @@
       <c r="D42" s="17">
         <v>339.45999999999998</v>
       </c>
-      <c r="E42" s="36"/>
-      <c r="F42" s="36"/>
-      <c r="G42" s="36"/>
-      <c r="H42" s="36"/>
-      <c r="I42" s="36"/>
-      <c r="J42" s="36"/>
-      <c r="K42" s="36"/>
-      <c r="L42" s="36"/>
-      <c r="M42" s="36"/>
-      <c r="N42" s="36"/>
+      <c r="E42" s="37"/>
+      <c r="F42" s="37"/>
+      <c r="G42" s="37"/>
+      <c r="H42" s="37"/>
+      <c r="I42" s="37"/>
+      <c r="J42" s="37"/>
+      <c r="K42" s="37"/>
+      <c r="L42" s="37"/>
+      <c r="M42" s="37"/>
+      <c r="N42" s="37"/>
       <c r="O42" s="17"/>
       <c r="P42" s="17"/>
       <c r="Q42" s="17"/>
@@ -4494,32 +4712,34 @@
       <c r="T42" s="17"/>
       <c r="U42" s="17"/>
       <c r="V42" s="17"/>
-      <c r="W42" s="19">
-        <f>MIN(C42:V42)</f>
+      <c r="W42" s="17"/>
+      <c r="X42" s="17"/>
+      <c r="Y42" s="20">
+        <f>MIN(C42:X42)</f>
         <v>339.45999999999998</v>
       </c>
-      <c r="X42" s="20">
-        <f>MAX(C42:V42)</f>
+      <c r="Z42" s="21">
+        <f>MAX(C42:X42)</f>
         <v>339.45999999999998</v>
       </c>
-      <c r="Y42" s="20">
-        <f>AVERAGE(C42:V42)</f>
+      <c r="AA42" s="21">
+        <f>AVERAGE(C42:X42)</f>
         <v>339.45999999999998</v>
       </c>
-      <c r="Z42" s="20" t="e">
-        <f>AVERAGE(Q42:V42)</f>
+      <c r="AB42" s="21" t="e">
+        <f>AVERAGE(Q42:X42)</f>
         <v>#NUM!</v>
       </c>
-      <c r="AA42" s="21" t="e">
+      <c r="AC42" s="22" t="e">
+        <f>(AB42/AA42)-1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD42" s="22" t="e">
+        <f>(AB42/Y42)-1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE42" s="22">
         <f>(Z42/Y42)-1</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="AB42" s="21" t="e">
-        <f>(Z42/W42)-1</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="AC42" s="21">
-        <f>(X42/W42)-1</f>
         <v>0</v>
       </c>
     </row>
@@ -4534,7 +4754,7 @@
       <c r="D43" s="17"/>
       <c r="E43" s="17"/>
       <c r="F43" s="17"/>
-      <c r="G43" s="24">
+      <c r="G43" s="25">
         <v>378.99000000000001</v>
       </c>
       <c r="H43" s="17">
@@ -4582,74 +4802,80 @@
       <c r="V43" s="17">
         <v>378.99000000000001</v>
       </c>
-      <c r="W43" s="19">
-        <f>MIN(C43:V43)</f>
+      <c r="W43" s="17">
         <v>378.99000000000001</v>
       </c>
-      <c r="X43" s="20">
-        <f>MAX(C43:V43)</f>
+      <c r="X43" s="17">
         <v>378.99000000000001</v>
       </c>
       <c r="Y43" s="20">
-        <f>AVERAGE(C43:V43)</f>
+        <f>MIN(C43:X43)</f>
+        <v>378.99000000000001</v>
+      </c>
+      <c r="Z43" s="21">
+        <f>MAX(C43:X43)</f>
+        <v>378.99000000000001</v>
+      </c>
+      <c r="AA43" s="21">
+        <f>AVERAGE(C43:X43)</f>
         <v>378.9899999999999</v>
       </c>
-      <c r="Z43" s="20">
-        <f>AVERAGE(Q43:V43)</f>
+      <c r="AB43" s="21">
+        <f>AVERAGE(Q43:X43)</f>
         <v>378.99000000000001</v>
       </c>
-      <c r="AA43" s="21">
+      <c r="AC43" s="22">
+        <f>(AB43/AA43)-1</f>
+        <v>2.2204460492503131e-016</v>
+      </c>
+      <c r="AD43" s="22">
+        <f>(AB43/Y43)-1</f>
+        <v>0</v>
+      </c>
+      <c r="AE43" s="22">
         <f>(Z43/Y43)-1</f>
-        <v>2.2204460492503131e-016</v>
-      </c>
-      <c r="AB43" s="21">
-        <f>(Z43/W43)-1</f>
         <v>0</v>
       </c>
-      <c r="AC43" s="21">
-        <f>(X43/W43)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AD43" s="22" t="s">
+      <c r="AF43" s="23" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="44" ht="18">
-      <c r="A44" s="25" t="s">
+      <c r="A44" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="B44" s="26" t="s">
+      <c r="B44" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28">
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="H44" s="28">
+      <c r="H44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="I44" s="28">
+      <c r="I44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="J44" s="28">
+      <c r="J44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="K44" s="28">
+      <c r="K44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="L44" s="28">
+      <c r="L44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="M44" s="28">
+      <c r="M44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="N44" s="28">
+      <c r="N44" s="29">
         <v>88.329999999999998</v>
       </c>
-      <c r="O44" s="28">
+      <c r="O44" s="29">
         <v>88.329999999999998</v>
       </c>
       <c r="P44" s="17">
@@ -4674,34 +4900,40 @@
         <v>119.59</v>
       </c>
       <c r="W44" s="19">
-        <f>MIN(C44:V44)</f>
+        <v>128.36000000000001</v>
+      </c>
+      <c r="X44" s="19">
+        <v>128.36000000000001</v>
+      </c>
+      <c r="Y44" s="20">
+        <f>MIN(C44:X44)</f>
         <v>88.329999999999998</v>
       </c>
-      <c r="X44" s="20">
-        <f>MAX(C44:V44)</f>
-        <v>119.59</v>
-      </c>
-      <c r="Y44" s="20">
-        <f>AVERAGE(C44:V44)</f>
-        <v>99.611874999999998</v>
-      </c>
-      <c r="Z44" s="20">
-        <f>AVERAGE(Q44:V44)</f>
-        <v>118.41500000000001</v>
+      <c r="Z44" s="21">
+        <f>MAX(C44:X44)</f>
+        <v>128.36000000000001</v>
       </c>
       <c r="AA44" s="21">
+        <f>AVERAGE(C44:X44)</f>
+        <v>102.80611111111112</v>
+      </c>
+      <c r="AB44" s="21">
+        <f>AVERAGE(Q44:X44)</f>
+        <v>120.90125</v>
+      </c>
+      <c r="AC44" s="22">
+        <f>(AB44/AA44)-1</f>
+        <v>0.1760122885042501</v>
+      </c>
+      <c r="AD44" s="22">
+        <f>(AB44/Y44)-1</f>
+        <v>0.368745046982905</v>
+      </c>
+      <c r="AE44" s="22">
         <f>(Z44/Y44)-1</f>
-        <v>0.18876388984747061</v>
-      </c>
-      <c r="AB44" s="21">
-        <f>(Z44/W44)-1</f>
-        <v>0.34059775840597761</v>
-      </c>
-      <c r="AC44" s="21">
-        <f>(X44/W44)-1</f>
-        <v>0.35390014717536511</v>
-      </c>
-      <c r="AD44" s="22" t="s">
+        <v>0.45318691271368738</v>
+      </c>
+      <c r="AF44" s="23" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4721,7 +4953,7 @@
       <c r="G45" s="17">
         <v>39.950000000000003</v>
       </c>
-      <c r="H45" s="24">
+      <c r="H45" s="25">
         <v>29.989999999999998</v>
       </c>
       <c r="I45" s="17">
@@ -4763,38 +4995,44 @@
       <c r="U45" s="17">
         <v>39.990000000000002</v>
       </c>
-      <c r="V45" s="33">
+      <c r="V45" s="34">
         <v>32.990000000000002</v>
       </c>
-      <c r="W45" s="19">
-        <f>MIN(C45:V45)</f>
+      <c r="W45" s="34">
+        <v>32.990000000000002</v>
+      </c>
+      <c r="X45" s="36">
+        <v>34.759999999999998</v>
+      </c>
+      <c r="Y45" s="20">
+        <f>MIN(C45:X45)</f>
         <v>29.989999999999998</v>
       </c>
-      <c r="X45" s="20">
-        <f>MAX(C45:V45)</f>
+      <c r="Z45" s="21">
+        <f>MAX(C45:X45)</f>
         <v>44.979999999999997</v>
       </c>
-      <c r="Y45" s="20">
-        <f>AVERAGE(C45:V45)</f>
-        <v>36.72117647058824</v>
-      </c>
-      <c r="Z45" s="20">
-        <f>AVERAGE(Q45:V45)</f>
-        <v>37.153333333333336</v>
-      </c>
       <c r="AA45" s="21">
+        <f>AVERAGE(C45:X45)</f>
+        <v>36.421578947368424</v>
+      </c>
+      <c r="AB45" s="21">
+        <f>AVERAGE(Q45:X45)</f>
+        <v>36.333750000000002</v>
+      </c>
+      <c r="AC45" s="22">
+        <f>(AB45/AA45)-1</f>
+        <v>-2.4114535917111324e-003</v>
+      </c>
+      <c r="AD45" s="22">
+        <f>(AB45/Y45)-1</f>
+        <v>0.2115288429476494</v>
+      </c>
+      <c r="AE45" s="22">
         <f>(Z45/Y45)-1</f>
-        <v>1.1768600689883391e-002</v>
-      </c>
-      <c r="AB45" s="21">
-        <f>(Z45/W45)-1</f>
-        <v>0.23885739691008134</v>
-      </c>
-      <c r="AC45" s="21">
-        <f>(X45/W45)-1</f>
         <v>0.49983327775925313</v>
       </c>
-      <c r="AD45" s="22" t="s">
+      <c r="AF45" s="23" t="s">
         <v>125</v>
       </c>
     </row>
@@ -4811,7 +5049,7 @@
       </c>
       <c r="E46" s="17"/>
       <c r="F46" s="17"/>
-      <c r="G46" s="33">
+      <c r="G46" s="34">
         <v>27.489999999999998</v>
       </c>
       <c r="H46" s="17">
@@ -4820,74 +5058,80 @@
       <c r="I46" s="17">
         <v>35.990000000000002</v>
       </c>
-      <c r="J46" s="33">
+      <c r="J46" s="34">
         <v>25.989999999999998</v>
       </c>
-      <c r="K46" s="33">
+      <c r="K46" s="34">
         <v>25.989999999999998</v>
       </c>
-      <c r="L46" s="33">
+      <c r="L46" s="34">
         <v>25.989999999999998</v>
       </c>
-      <c r="M46" s="33">
+      <c r="M46" s="34">
         <v>25.989999999999998</v>
       </c>
-      <c r="N46" s="17">
+      <c r="N46" s="18">
         <v>36.43</v>
       </c>
-      <c r="O46" s="17">
+      <c r="O46" s="19">
         <v>42</v>
       </c>
-      <c r="P46" s="17">
+      <c r="P46" s="18">
         <v>36.369999999999997</v>
       </c>
-      <c r="Q46" s="17">
+      <c r="Q46" s="18">
         <v>35.119999999999997</v>
       </c>
-      <c r="R46" s="17">
+      <c r="R46" s="18">
         <v>36.409999999999997</v>
       </c>
-      <c r="S46" s="17">
+      <c r="S46" s="18">
         <v>36.530000000000001</v>
       </c>
-      <c r="T46" s="33">
+      <c r="T46" s="34">
         <v>27.989999999999998</v>
       </c>
-      <c r="U46" s="33">
+      <c r="U46" s="34">
         <v>27.989999999999998</v>
       </c>
-      <c r="V46" s="35">
+      <c r="V46" s="36">
         <v>30.989999999999998</v>
       </c>
-      <c r="W46" s="19">
-        <f>MIN(C46:V46)</f>
+      <c r="W46" s="36">
+        <v>30.989999999999998</v>
+      </c>
+      <c r="X46" s="35">
+        <v>36.530000000000001</v>
+      </c>
+      <c r="Y46" s="20">
+        <f>MIN(C46:X46)</f>
         <v>25.989999999999998</v>
       </c>
-      <c r="X46" s="20">
-        <f>MAX(C46:V46)</f>
+      <c r="Z46" s="21">
+        <f>MAX(C46:X46)</f>
         <v>42</v>
       </c>
-      <c r="Y46" s="20">
-        <f>AVERAGE(C46:V46)</f>
-        <v>31.720588235294116</v>
-      </c>
-      <c r="Z46" s="20">
-        <f>AVERAGE(Q46:V46)</f>
-        <v>32.505000000000003</v>
-      </c>
       <c r="AA46" s="21">
+        <f>AVERAGE(C46:X46)</f>
+        <v>31.935263157894735</v>
+      </c>
+      <c r="AB46" s="21">
+        <f>AVERAGE(Q46:X46)</f>
+        <v>32.818750000000009</v>
+      </c>
+      <c r="AC46" s="22">
+        <f>(AB46/AA46)-1</f>
+        <v>2.766493069861764e-002</v>
+      </c>
+      <c r="AD46" s="22">
+        <f>(AB46/Y46)-1</f>
+        <v>0.26274528664871144</v>
+      </c>
+      <c r="AE46" s="22">
         <f>(Z46/Y46)-1</f>
-        <v>2.4728789986091959e-002</v>
-      </c>
-      <c r="AB46" s="21">
-        <f>(Z46/W46)-1</f>
-        <v>0.25067333589842256</v>
-      </c>
-      <c r="AC46" s="21">
-        <f>(X46/W46)-1</f>
         <v>0.61600615621392851</v>
       </c>
-      <c r="AD46" s="22" t="s">
+      <c r="AF46" s="23" t="s">
         <v>128</v>
       </c>
     </row>
@@ -4907,7 +5151,7 @@
       <c r="G47" s="17">
         <v>22.989999999999998</v>
       </c>
-      <c r="H47" s="24">
+      <c r="H47" s="25">
         <v>21.690000000000001</v>
       </c>
       <c r="I47" s="17">
@@ -4949,38 +5193,44 @@
       <c r="U47" s="17">
         <v>24.899999999999999</v>
       </c>
-      <c r="V47" s="33">
+      <c r="V47" s="34">
         <v>21.690000000000001</v>
       </c>
-      <c r="W47" s="19">
-        <f>MIN(C47:V47)</f>
+      <c r="W47" s="36">
+        <v>28.899999999999999</v>
+      </c>
+      <c r="X47" s="36">
+        <v>28.899999999999999</v>
+      </c>
+      <c r="Y47" s="20">
+        <f>MIN(C47:X47)</f>
         <v>21.690000000000001</v>
       </c>
-      <c r="X47" s="20">
-        <f>MAX(C47:V47)</f>
+      <c r="Z47" s="21">
+        <f>MAX(C47:X47)</f>
         <v>43.990000000000002</v>
       </c>
-      <c r="Y47" s="20">
-        <f>AVERAGE(C47:V47)</f>
-        <v>29.504705882352933</v>
-      </c>
-      <c r="Z47" s="20">
-        <f>AVERAGE(Q47:V47)</f>
-        <v>27.628333333333334</v>
-      </c>
       <c r="AA47" s="21">
+        <f>AVERAGE(C47:X47)</f>
+        <v>29.441052631578941</v>
+      </c>
+      <c r="AB47" s="21">
+        <f>AVERAGE(Q47:X47)</f>
+        <v>27.946250000000003</v>
+      </c>
+      <c r="AC47" s="22">
+        <f>(AB47/AA47)-1</f>
+        <v>-5.0772730523078846e-002</v>
+      </c>
+      <c r="AD47" s="22">
+        <f>(AB47/Y47)-1</f>
+        <v>0.28843937298294153</v>
+      </c>
+      <c r="AE47" s="22">
         <f>(Z47/Y47)-1</f>
-        <v>-6.3595704241264039e-002</v>
-      </c>
-      <c r="AB47" s="21">
-        <f>(Z47/W47)-1</f>
-        <v>0.27378208083602273</v>
-      </c>
-      <c r="AC47" s="21">
-        <f>(X47/W47)-1</f>
         <v>1.0281235592438911</v>
       </c>
-      <c r="AD47" s="22" t="s">
+      <c r="AF47" s="23" t="s">
         <v>131</v>
       </c>
     </row>
@@ -5015,7 +5265,7 @@
       <c r="L48" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="M48" s="24">
+      <c r="M48" s="25">
         <v>1449.28</v>
       </c>
       <c r="N48" s="18">
@@ -5045,74 +5295,80 @@
       <c r="V48" s="17">
         <v>1611.4100000000001</v>
       </c>
-      <c r="W48" s="19">
-        <f>MIN(C48:V48)</f>
+      <c r="W48" s="17">
+        <v>1611.4100000000001</v>
+      </c>
+      <c r="X48" s="17">
+        <v>1611.4100000000001</v>
+      </c>
+      <c r="Y48" s="20">
+        <f>MIN(C48:X48)</f>
         <v>1449.28</v>
       </c>
-      <c r="X48" s="20">
-        <f>MAX(C48:V48)</f>
+      <c r="Z48" s="21">
+        <f>MAX(C48:X48)</f>
         <v>1820.77</v>
       </c>
-      <c r="Y48" s="20">
-        <f>AVERAGE(C48:V48)</f>
-        <v>1702.3566666666666</v>
-      </c>
-      <c r="Z48" s="20">
-        <f>AVERAGE(Q48:V48)</f>
-        <v>1675.5600000000002</v>
-      </c>
       <c r="AA48" s="21">
+        <f>AVERAGE(C48:X48)</f>
+        <v>1691.6570588235293</v>
+      </c>
+      <c r="AB48" s="21">
+        <f>AVERAGE(Q48:X48)</f>
+        <v>1659.5225</v>
+      </c>
+      <c r="AC48" s="22">
+        <f>(AB48/AA48)-1</f>
+        <v>-1.899590620682734e-002</v>
+      </c>
+      <c r="AD48" s="22">
+        <f>(AB48/Y48)-1</f>
+        <v>0.14506686078604547</v>
+      </c>
+      <c r="AE48" s="22">
         <f>(Z48/Y48)-1</f>
-        <v>-1.5740923856536027e-002</v>
-      </c>
-      <c r="AB48" s="21">
-        <f>(Z48/W48)-1</f>
-        <v>0.15613270037535898</v>
-      </c>
-      <c r="AC48" s="21">
-        <f>(X48/W48)-1</f>
         <v>0.25632727975270475</v>
       </c>
-      <c r="AD48" s="1" t="s">
+      <c r="AF48" s="1" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="49" ht="18">
-      <c r="A49" s="25" t="s">
+      <c r="A49" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="B49" s="26" t="s">
+      <c r="B49" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-      <c r="F49" s="28"/>
-      <c r="G49" s="28">
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="29"/>
+      <c r="F49" s="29"/>
+      <c r="G49" s="29">
         <v>33.890000000000001</v>
       </c>
-      <c r="H49" s="28">
+      <c r="H49" s="29">
         <v>33.890000000000001</v>
       </c>
-      <c r="I49" s="28">
+      <c r="I49" s="29">
         <v>33.890000000000001</v>
       </c>
-      <c r="J49" s="28">
+      <c r="J49" s="29">
         <v>33.890000000000001</v>
       </c>
-      <c r="K49" s="28">
+      <c r="K49" s="29">
         <v>33.890000000000001</v>
       </c>
-      <c r="L49" s="28">
+      <c r="L49" s="29">
         <v>38.039999999999999</v>
       </c>
-      <c r="M49" s="28">
+      <c r="M49" s="29">
         <v>38.369999999999997</v>
       </c>
-      <c r="N49" s="28">
+      <c r="N49" s="29">
         <v>38.369999999999997</v>
       </c>
-      <c r="O49" s="28">
+      <c r="O49" s="29">
         <v>38.369999999999997</v>
       </c>
       <c r="P49" s="17">
@@ -5133,38 +5389,44 @@
       <c r="U49" s="17">
         <v>39.899999999999999</v>
       </c>
-      <c r="V49" s="33">
+      <c r="V49" s="34">
         <v>31.989999999999998</v>
       </c>
-      <c r="W49" s="19">
-        <f>MIN(C49:V49)</f>
-        <v>31.989999999999998</v>
-      </c>
-      <c r="X49" s="20">
-        <f>MAX(C49:V49)</f>
+      <c r="W49" s="34">
+        <v>30.989999999999998</v>
+      </c>
+      <c r="X49" s="36">
+        <v>39.899999999999999</v>
+      </c>
+      <c r="Y49" s="20">
+        <f>MIN(C49:X49)</f>
+        <v>30.989999999999998</v>
+      </c>
+      <c r="Z49" s="21">
+        <f>MAX(C49:X49)</f>
         <v>43.210000000000001</v>
       </c>
-      <c r="Y49" s="20">
-        <f>AVERAGE(C49:V49)</f>
-        <v>37.076249999999995</v>
-      </c>
-      <c r="Z49" s="20">
-        <f>AVERAGE(Q49:V49)</f>
-        <v>38.708333333333336</v>
-      </c>
       <c r="AA49" s="21">
+        <f>AVERAGE(C49:X49)</f>
+        <v>36.894999999999996</v>
+      </c>
+      <c r="AB49" s="21">
+        <f>AVERAGE(Q49:X49)</f>
+        <v>37.892499999999998</v>
+      </c>
+      <c r="AC49" s="22">
+        <f>(AB49/AA49)-1</f>
+        <v>2.7036183764737931e-002</v>
+      </c>
+      <c r="AD49" s="22">
+        <f>(AB49/Y49)-1</f>
+        <v>0.2227331397224912</v>
+      </c>
+      <c r="AE49" s="22">
         <f>(Z49/Y49)-1</f>
-        <v>4.4019644201701569e-002</v>
-      </c>
-      <c r="AB49" s="21">
-        <f>(Z49/W49)-1</f>
-        <v>0.21001354589976051</v>
-      </c>
-      <c r="AC49" s="21">
-        <f>(X49/W49)-1</f>
-        <v>0.35073460456392636</v>
-      </c>
-      <c r="AD49" s="22" t="s">
+        <v>0.39432074862859001</v>
+      </c>
+      <c r="AF49" s="23" t="s">
         <v>136</v>
       </c>
     </row>
@@ -5185,13 +5447,13 @@
       <c r="H50" s="17">
         <v>90.739999999999995</v>
       </c>
-      <c r="I50" s="24">
+      <c r="I50" s="25">
         <v>89.950000000000003</v>
       </c>
-      <c r="J50" s="24">
+      <c r="J50" s="25">
         <v>89.950000000000003</v>
       </c>
-      <c r="K50" s="24">
+      <c r="K50" s="25">
         <v>89.950000000000003</v>
       </c>
       <c r="L50" s="17">
@@ -5227,35 +5489,41 @@
       <c r="V50" s="17">
         <v>83.079999999999998</v>
       </c>
-      <c r="W50" s="19">
-        <f>MIN(C50:V50)</f>
+      <c r="W50" s="17">
+        <v>84.099999999999994</v>
+      </c>
+      <c r="X50" s="17">
+        <v>84.680000000000007</v>
+      </c>
+      <c r="Y50" s="20">
+        <f>MIN(C50:X50)</f>
         <v>81.689999999999998</v>
       </c>
-      <c r="X50" s="20">
-        <f>MAX(C50:V50)</f>
+      <c r="Z50" s="21">
+        <f>MAX(C50:X50)</f>
         <v>93.280000000000001</v>
       </c>
-      <c r="Y50" s="20">
-        <f>AVERAGE(C50:V50)</f>
-        <v>88.674375000000026</v>
-      </c>
-      <c r="Z50" s="20">
-        <f>AVERAGE(Q50:V50)</f>
-        <v>85.695000000000007</v>
-      </c>
       <c r="AA50" s="21">
+        <f>AVERAGE(C50:X50)</f>
+        <v>88.198333333333352</v>
+      </c>
+      <c r="AB50" s="21">
+        <f>AVERAGE(Q50:X50)</f>
+        <v>85.368750000000006</v>
+      </c>
+      <c r="AC50" s="22">
+        <f>(AB50/AA50)-1</f>
+        <v>-3.2082049925357792e-002</v>
+      </c>
+      <c r="AD50" s="22">
+        <f>(AB50/Y50)-1</f>
+        <v>4.5033051781123934e-002</v>
+      </c>
+      <c r="AE50" s="22">
         <f>(Z50/Y50)-1</f>
-        <v>-3.3599052713932487e-002</v>
-      </c>
-      <c r="AB50" s="21">
-        <f>(Z50/W50)-1</f>
-        <v>4.902680866691167e-002</v>
-      </c>
-      <c r="AC50" s="21">
-        <f>(X50/W50)-1</f>
         <v>0.1418778308238462</v>
       </c>
-      <c r="AD50" s="1" t="s">
+      <c r="AF50" s="1" t="s">
         <v>139</v>
       </c>
     </row>
@@ -5320,35 +5588,41 @@
       <c r="V51" s="17">
         <v>309.05000000000001</v>
       </c>
-      <c r="W51" s="19">
-        <f>MIN(C51:V51)</f>
+      <c r="W51" s="34">
+        <v>298.80000000000001</v>
+      </c>
+      <c r="X51" s="34">
+        <v>298.80000000000001</v>
+      </c>
+      <c r="Y51" s="20">
+        <f>MIN(C51:X51)</f>
+        <v>298.80000000000001</v>
+      </c>
+      <c r="Z51" s="21">
+        <f>MAX(C51:X51)</f>
         <v>309.05000000000001</v>
       </c>
-      <c r="X51" s="20">
-        <f>MAX(C51:V51)</f>
-        <v>309.05000000000001</v>
-      </c>
-      <c r="Y51" s="20">
-        <f>AVERAGE(C51:V51)</f>
-        <v>309.05000000000007</v>
-      </c>
-      <c r="Z51" s="20">
-        <f>AVERAGE(Q51:V51)</f>
-        <v>309.05000000000001</v>
-      </c>
       <c r="AA51" s="21">
+        <f>AVERAGE(C51:X51)</f>
+        <v>307.97105263157903</v>
+      </c>
+      <c r="AB51" s="21">
+        <f>AVERAGE(Q51:X51)</f>
+        <v>306.48750000000001</v>
+      </c>
+      <c r="AC51" s="22">
+        <f>(AB51/AA51)-1</f>
+        <v>-4.817182065983916e-003</v>
+      </c>
+      <c r="AD51" s="22">
+        <f>(AB51/Y51)-1</f>
+        <v>2.5727911646586277e-002</v>
+      </c>
+      <c r="AE51" s="22">
         <f>(Z51/Y51)-1</f>
-        <v>-2.2204460492503131e-016</v>
-      </c>
-      <c r="AB51" s="21">
-        <f>(Z51/W51)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AC51" s="21">
-        <f>(X51/W51)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AD51" s="22" t="s">
+        <v>3.4303882195448443e-002</v>
+      </c>
+      <c r="AF51" s="23" t="s">
         <v>142</v>
       </c>
     </row>
@@ -5411,35 +5685,41 @@
       <c r="V52" s="17">
         <v>108.98999999999999</v>
       </c>
-      <c r="W52" s="19">
-        <f>MIN(C52:V52)</f>
+      <c r="W52" s="17">
         <v>108.98999999999999</v>
       </c>
-      <c r="X52" s="20">
-        <f>MAX(C52:V52)</f>
+      <c r="X52" s="17">
         <v>108.98999999999999</v>
       </c>
       <c r="Y52" s="20">
-        <f>AVERAGE(C52:V52)</f>
+        <f>MIN(C52:X52)</f>
         <v>108.98999999999999</v>
       </c>
-      <c r="Z52" s="20">
-        <f>AVERAGE(Q52:V52)</f>
+      <c r="Z52" s="21">
+        <f>MAX(C52:X52)</f>
         <v>108.98999999999999</v>
       </c>
       <c r="AA52" s="21">
+        <f>AVERAGE(C52:X52)</f>
+        <v>108.98999999999999</v>
+      </c>
+      <c r="AB52" s="21">
+        <f>AVERAGE(Q52:X52)</f>
+        <v>108.98999999999999</v>
+      </c>
+      <c r="AC52" s="22">
+        <f>(AB52/AA52)-1</f>
+        <v>0</v>
+      </c>
+      <c r="AD52" s="22">
+        <f>(AB52/Y52)-1</f>
+        <v>0</v>
+      </c>
+      <c r="AE52" s="22">
         <f>(Z52/Y52)-1</f>
         <v>0</v>
       </c>
-      <c r="AB52" s="21">
-        <f>(Z52/W52)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AC52" s="21">
-        <f>(X52/W52)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AD52" s="37" t="s">
+      <c r="AF52" s="38" t="s">
         <v>144</v>
       </c>
     </row>
@@ -5471,93 +5751,98 @@
       <c r="V53" s="17">
         <v>1.99</v>
       </c>
-      <c r="W53" s="19">
-        <f>MIN(C53:V53)</f>
+      <c r="W53" s="17">
+        <v>1.99</v>
+      </c>
+      <c r="X53" s="17">
+        <v>1.99</v>
+      </c>
+      <c r="Y53" s="20">
+        <f>MIN(C53:X53)</f>
         <v>1.49</v>
       </c>
-      <c r="X53" s="20">
-        <f>MAX(C53:V53)</f>
+      <c r="Z53" s="21">
+        <f>MAX(C53:X53)</f>
         <v>1.99</v>
       </c>
-      <c r="Y53" s="20">
-        <f>AVERAGE(C53:V53)</f>
-        <v>1.6775</v>
-      </c>
-      <c r="Z53" s="20">
-        <f>AVERAGE(Q53:V53)</f>
-        <v>1.74</v>
-      </c>
       <c r="AA53" s="21">
+        <f>AVERAGE(C53:X53)</f>
+        <v>1.7399999999999998</v>
+      </c>
+      <c r="AB53" s="21">
+        <f>AVERAGE(Q53:X53)</f>
+        <v>1.8025</v>
+      </c>
+      <c r="AC53" s="22">
+        <f>(AB53/AA53)-1</f>
+        <v>3.5919540229885083e-002</v>
+      </c>
+      <c r="AD53" s="22">
+        <f>(AB53/Y53)-1</f>
+        <v>0.20973154362416113</v>
+      </c>
+      <c r="AE53" s="22">
         <f>(Z53/Y53)-1</f>
-        <v>3.7257824143070106e-002</v>
-      </c>
-      <c r="AB53" s="21">
-        <f>(Z53/W53)-1</f>
-        <v>0.16778523489932895</v>
-      </c>
-      <c r="AC53" s="21">
-        <f>(X53/W53)-1</f>
         <v>0.33557046979865768</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="W1:W6"/>
-    <mergeCell ref="X1:X6"/>
     <mergeCell ref="Y1:Y6"/>
     <mergeCell ref="Z1:Z6"/>
     <mergeCell ref="AA1:AA6"/>
     <mergeCell ref="AB1:AB6"/>
     <mergeCell ref="AC1:AC6"/>
+    <mergeCell ref="AD1:AD6"/>
+    <mergeCell ref="AE1:AE6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B5"/>
-    <hyperlink r:id="rId2" ref="AD8"/>
-    <hyperlink r:id="rId3" ref="AD9"/>
-    <hyperlink r:id="rId4" ref="AD10"/>
-    <hyperlink r:id="rId5" ref="AD11"/>
-    <hyperlink r:id="rId6" ref="AD12"/>
-    <hyperlink r:id="rId7" ref="AD13"/>
-    <hyperlink r:id="rId8" ref="AD14"/>
-    <hyperlink r:id="rId9" ref="AD15"/>
-    <hyperlink r:id="rId10" ref="AD16"/>
-    <hyperlink r:id="rId11" ref="AD17"/>
-    <hyperlink r:id="rId12" ref="AD18"/>
-    <hyperlink r:id="rId13" ref="AD19"/>
-    <hyperlink r:id="rId14" ref="AD20"/>
-    <hyperlink r:id="rId15" ref="AD21"/>
-    <hyperlink r:id="rId16" ref="AD22"/>
-    <hyperlink r:id="rId17" ref="AD23"/>
-    <hyperlink r:id="rId18" ref="AD24"/>
-    <hyperlink r:id="rId19" ref="AD25"/>
-    <hyperlink r:id="rId20" ref="AD26"/>
-    <hyperlink r:id="rId21" ref="AD27"/>
-    <hyperlink r:id="rId22" ref="AD28"/>
-    <hyperlink r:id="rId23" ref="AD29"/>
-    <hyperlink r:id="rId24" ref="AD30"/>
-    <hyperlink r:id="rId25" ref="AD31"/>
-    <hyperlink r:id="rId26" ref="AD32"/>
-    <hyperlink r:id="rId27" ref="AD33"/>
-    <hyperlink r:id="rId28" ref="AD34"/>
-    <hyperlink r:id="rId29" ref="AD35"/>
-    <hyperlink r:id="rId30" ref="AD36"/>
-    <hyperlink r:id="rId30" ref="AD37"/>
-    <hyperlink r:id="rId30" ref="AD38"/>
-    <hyperlink r:id="rId30" ref="AD39"/>
-    <hyperlink r:id="rId30" ref="AD40"/>
-    <hyperlink r:id="rId30" ref="AD41"/>
-    <hyperlink r:id="rId31" ref="AD43"/>
-    <hyperlink r:id="rId32" ref="AD44"/>
-    <hyperlink r:id="rId33" ref="AD45"/>
-    <hyperlink r:id="rId34" ref="AD46"/>
-    <hyperlink r:id="rId35" ref="AD47"/>
-    <hyperlink r:id="rId36" ref="AD49"/>
-    <hyperlink r:id="rId37" ref="AD51"/>
-    <hyperlink r:id="rId38" ref="AD52"/>
+    <hyperlink r:id="rId1" ref="AF8"/>
+    <hyperlink r:id="rId2" ref="AF9"/>
+    <hyperlink r:id="rId3" ref="AF10"/>
+    <hyperlink r:id="rId4" ref="AF11"/>
+    <hyperlink r:id="rId5" ref="AF12"/>
+    <hyperlink r:id="rId6" ref="AF13"/>
+    <hyperlink r:id="rId7" ref="AF14"/>
+    <hyperlink r:id="rId8" ref="AF15"/>
+    <hyperlink r:id="rId9" ref="AF16"/>
+    <hyperlink r:id="rId10" ref="AF17"/>
+    <hyperlink r:id="rId11" ref="AF18"/>
+    <hyperlink r:id="rId12" ref="AF19"/>
+    <hyperlink r:id="rId13" ref="AF20"/>
+    <hyperlink r:id="rId14" ref="AF21"/>
+    <hyperlink r:id="rId15" ref="AF22"/>
+    <hyperlink r:id="rId16" ref="AF23"/>
+    <hyperlink r:id="rId17" ref="AF24"/>
+    <hyperlink r:id="rId18" ref="AF25"/>
+    <hyperlink r:id="rId19" ref="AF26"/>
+    <hyperlink r:id="rId20" ref="AF27"/>
+    <hyperlink r:id="rId21" ref="AF28"/>
+    <hyperlink r:id="rId22" ref="AF29"/>
+    <hyperlink r:id="rId23" ref="AF30"/>
+    <hyperlink r:id="rId24" ref="AF31"/>
+    <hyperlink r:id="rId25" ref="AF32"/>
+    <hyperlink r:id="rId26" ref="AF33"/>
+    <hyperlink r:id="rId27" ref="AF34"/>
+    <hyperlink r:id="rId28" ref="AF35"/>
+    <hyperlink r:id="rId29" ref="AF36"/>
+    <hyperlink r:id="rId29" ref="AF37"/>
+    <hyperlink r:id="rId29" ref="AF38"/>
+    <hyperlink r:id="rId29" ref="AF39"/>
+    <hyperlink r:id="rId29" ref="AF40"/>
+    <hyperlink r:id="rId29" ref="AF41"/>
+    <hyperlink r:id="rId30" ref="AF43"/>
+    <hyperlink r:id="rId31" ref="AF44"/>
+    <hyperlink r:id="rId32" ref="AF45"/>
+    <hyperlink r:id="rId33" ref="AF46"/>
+    <hyperlink r:id="rId34" ref="AF47"/>
+    <hyperlink r:id="rId35" ref="AF49"/>
+    <hyperlink r:id="rId36" ref="AF51"/>
+    <hyperlink r:id="rId37" ref="AF52"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.25196850393700787" right="0.25196850393700787" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="37" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="36" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Prices update on 2026-04-11
</commit_message>
<xml_diff>
--- a/analyse-prix-composants.xlsx
+++ b/analyse-prix-composants.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuille1!$A:$AF</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuille1!$A:$AG</definedName>
     <definedName name="Print_Titles" localSheetId="0">Feuille1!$7:$7</definedName>
   </definedNames>
   <calcPr/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t xml:space="preserve">Le prix des composants IT</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t xml:space="preserve">4 avr 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 avr 2026</t>
   </si>
   <si>
     <t>Min</t>
@@ -1349,12 +1352,12 @@
     <col bestFit="1" min="12" max="12" style="4" width="11.7109375"/>
     <col bestFit="1" min="13" max="13" style="4" width="13.00390625"/>
     <col bestFit="1" min="14" max="15" style="4" width="14.140625"/>
-    <col customWidth="1" min="16" max="25" style="1" width="12.7109375"/>
-    <col customWidth="1" min="26" max="29" style="2" width="12.7109375"/>
-    <col customWidth="1" min="30" max="30" style="2" width="14.140625"/>
-    <col customWidth="1" min="31" max="32" style="2" width="12.7109375"/>
-    <col customWidth="1" min="33" max="33" style="5" width="42.28125"/>
-    <col min="34" max="16384" style="1" width="9.140625"/>
+    <col customWidth="1" min="16" max="26" style="1" width="12.7109375"/>
+    <col customWidth="1" min="27" max="30" style="2" width="12.7109375"/>
+    <col customWidth="1" min="31" max="31" style="2" width="14.140625"/>
+    <col customWidth="1" min="32" max="33" style="2" width="12.7109375"/>
+    <col customWidth="1" min="34" max="34" style="5" width="42.28125"/>
+    <col min="35" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="33">
@@ -1372,28 +1375,29 @@
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
-      <c r="Z1" s="7" t="s">
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="AA1" s="7" t="s">
+      <c r="AB1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="AB1" s="7" t="s">
+      <c r="AC1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="AC1" s="7" t="s">
+      <c r="AD1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="AD1" s="7" t="s">
+      <c r="AE1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AE1" s="7" t="s">
+      <c r="AF1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AF1" s="7" t="s">
+      <c r="AG1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="AG1" s="5"/>
+      <c r="AH1" s="5"/>
     </row>
     <row r="2" ht="23.25">
       <c r="A2" s="2"/>
@@ -1410,13 +1414,14 @@
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
-      <c r="Z2" s="7"/>
+      <c r="Z2" s="1"/>
       <c r="AA2" s="7"/>
       <c r="AB2" s="7"/>
       <c r="AC2" s="7"/>
       <c r="AD2" s="7"/>
       <c r="AE2" s="7"/>
       <c r="AF2" s="7"/>
+      <c r="AG2" s="7"/>
     </row>
     <row r="3" ht="18">
       <c r="A3" s="2"/>
@@ -1431,13 +1436,14 @@
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
-      <c r="Z3" s="7"/>
+      <c r="Z3" s="1"/>
       <c r="AA3" s="7"/>
       <c r="AB3" s="7"/>
       <c r="AC3" s="7"/>
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
+      <c r="AG3" s="7"/>
     </row>
     <row r="4" ht="18">
       <c r="A4" s="2"/>
@@ -1453,13 +1459,14 @@
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
-      <c r="Z4" s="7"/>
+      <c r="Z4" s="1"/>
       <c r="AA4" s="7"/>
       <c r="AB4" s="7"/>
       <c r="AC4" s="7"/>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
+      <c r="AG4" s="7"/>
     </row>
     <row r="5" ht="23.25">
       <c r="A5" s="2"/>
@@ -1474,13 +1481,14 @@
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
-      <c r="Z5" s="7"/>
+      <c r="Z5" s="1"/>
       <c r="AA5" s="7"/>
       <c r="AB5" s="7"/>
       <c r="AC5" s="7"/>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
+      <c r="AG5" s="7"/>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2"/>
@@ -1494,13 +1502,14 @@
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
-      <c r="Z6" s="7"/>
+      <c r="Z6" s="1"/>
       <c r="AA6" s="7"/>
       <c r="AB6" s="7"/>
       <c r="AC6" s="7"/>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
+      <c r="AG6" s="7"/>
     </row>
     <row r="7" ht="18">
       <c r="A7" s="10" t="s">
@@ -1578,7 +1587,7 @@
       <c r="Y7" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="Z7" s="13" t="s">
+      <c r="Z7" s="12" t="s">
         <v>34</v>
       </c>
       <c r="AA7" s="13" t="s">
@@ -1599,16 +1608,19 @@
       <c r="AF7" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="AG7" s="5" t="s">
+      <c r="AG7" s="13" t="s">
         <v>41</v>
+      </c>
+      <c r="AH7" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="8" ht="36">
       <c r="A8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" s="15">
         <v>171.88</v>
@@ -1635,7 +1647,7 @@
         <v>341.57999999999998</v>
       </c>
       <c r="M8" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N8" s="18">
         <v>321.14999999999998</v>
@@ -1673,48 +1685,51 @@
       <c r="Y8" s="19">
         <v>418.17000000000002</v>
       </c>
-      <c r="Z8" s="20">
-        <f>MIN(C8:Y8)</f>
+      <c r="Z8" s="18">
+        <v>397.13</v>
+      </c>
+      <c r="AA8" s="20">
+        <f>MIN(C8:Z8)</f>
         <v>171.88</v>
       </c>
-      <c r="AA8" s="21">
-        <f>MAX(C8:Y8)</f>
+      <c r="AB8" s="21">
+        <f>MAX(C8:Z8)</f>
         <v>418.17000000000002</v>
       </c>
-      <c r="AB8" s="21">
-        <f>AVERAGE(C8:Y8)</f>
-        <v>346.57684210526332</v>
-      </c>
       <c r="AC8" s="21">
-        <f>AVERAGE(Q8:Y8)</f>
-        <v>378.22999999999996</v>
-      </c>
-      <c r="AD8" s="22">
-        <f>(AC8/AB8)-1</f>
-        <v>9.1330850908736938e-002</v>
+        <f>AVERAGE(C8:Z8)</f>
+        <v>349.10450000000014</v>
+      </c>
+      <c r="AD8" s="21">
+        <f>AVERAGE(Q8:Z8)</f>
+        <v>380.12</v>
       </c>
       <c r="AE8" s="22">
-        <f>(AC8/Z8)-1</f>
-        <v>1.200546893181289</v>
+        <f>(AD8/AC8)-1</f>
+        <v>8.8843025512417739e-002</v>
       </c>
       <c r="AF8" s="22">
-        <f>(AA8/Z8)-1</f>
+        <f>(AD8/AA8)-1</f>
+        <v>1.211542936932744</v>
+      </c>
+      <c r="AG8" s="22">
+        <f>(AB8/AA8)-1</f>
         <v>1.4329183151035609</v>
       </c>
-      <c r="AG8" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="AH8" s="24">
+      <c r="AH8" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI8" s="24">
         <f>C2*1</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" ht="36">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="25">
@@ -1726,7 +1741,7 @@
         <v>686</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I9" s="17">
         <v>613.99000000000001</v>
@@ -1779,44 +1794,47 @@
       <c r="Y9" s="18">
         <v>978.75</v>
       </c>
-      <c r="Z9" s="20">
-        <f>MIN(C9:Y9)</f>
+      <c r="Z9" s="18">
+        <v>978.75</v>
+      </c>
+      <c r="AA9" s="20">
+        <f>MIN(C9:Z9)</f>
         <v>200.47999999999999</v>
       </c>
-      <c r="AA9" s="21">
-        <f>MAX(C9:Y9)</f>
+      <c r="AB9" s="21">
+        <f>MAX(C9:Z9)</f>
         <v>978.75</v>
       </c>
-      <c r="AB9" s="21">
-        <f>AVERAGE(C9:Y9)</f>
-        <v>810.12473684210534</v>
-      </c>
       <c r="AC9" s="21">
-        <f>AVERAGE(Q9:Y9)</f>
-        <v>892.68888888888887</v>
-      </c>
-      <c r="AD9" s="22">
-        <f>(AC9/AB9)-1</f>
-        <v>0.10191535734190937</v>
+        <f>AVERAGE(C9:Z9)</f>
+        <v>818.55600000000004</v>
+      </c>
+      <c r="AD9" s="21">
+        <f>AVERAGE(Q9:Z9)</f>
+        <v>901.29500000000007</v>
       </c>
       <c r="AE9" s="22">
-        <f>(AC9/Z9)-1</f>
-        <v>3.4527578256628537</v>
+        <f>(AD9/AC9)-1</f>
+        <v>0.1010792175489521</v>
       </c>
       <c r="AF9" s="22">
-        <f>(AA9/Z9)-1</f>
+        <f>(AD9/AA9)-1</f>
+        <v>3.4956853551476463</v>
+      </c>
+      <c r="AG9" s="22">
+        <f>(AB9/AA9)-1</f>
         <v>3.8820331205107745</v>
       </c>
-      <c r="AG9" s="23" t="s">
-        <v>47</v>
+      <c r="AH9" s="23" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" ht="36">
       <c r="A10" s="26" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="28"/>
       <c r="D10" s="25">
@@ -1881,44 +1899,47 @@
       <c r="Y10" s="18">
         <v>709.99000000000001</v>
       </c>
-      <c r="Z10" s="20">
-        <f>MIN(C10:Y10)</f>
+      <c r="Z10" s="18">
+        <v>709.99000000000001</v>
+      </c>
+      <c r="AA10" s="20">
+        <f>MIN(C10:Z10)</f>
         <v>284.13</v>
       </c>
-      <c r="AA10" s="21">
-        <f>MAX(C10:Y10)</f>
+      <c r="AB10" s="21">
+        <f>MAX(C10:Z10)</f>
         <v>717.78999999999996</v>
       </c>
-      <c r="AB10" s="21">
-        <f>AVERAGE(C10:Y10)</f>
-        <v>604.33849999999995</v>
-      </c>
       <c r="AC10" s="21">
-        <f>AVERAGE(Q10:Y10)</f>
-        <v>666.87777777777774</v>
-      </c>
-      <c r="AD10" s="22">
-        <f>(AC10/AB10)-1</f>
-        <v>0.10348385512056213</v>
+        <f>AVERAGE(C10:Z10)</f>
+        <v>609.36952380952368</v>
+      </c>
+      <c r="AD10" s="21">
+        <f>AVERAGE(Q10:Z10)</f>
+        <v>671.18899999999996</v>
       </c>
       <c r="AE10" s="22">
-        <f>(AC10/Z10)-1</f>
-        <v>1.3470868186315341</v>
+        <f>(AD10/AC10)-1</f>
+        <v>0.10144825721510764</v>
       </c>
       <c r="AF10" s="22">
-        <f>(AA10/Z10)-1</f>
+        <f>(AD10/AA10)-1</f>
+        <v>1.3622602329919404</v>
+      </c>
+      <c r="AG10" s="22">
+        <f>(AB10/AA10)-1</f>
         <v>1.5262731848097699</v>
       </c>
-      <c r="AG10" s="23" t="s">
-        <v>49</v>
+      <c r="AH10" s="23" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="11" ht="36">
       <c r="A11" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
@@ -1977,44 +1998,47 @@
       <c r="Y11" s="19">
         <v>824.50999999999999</v>
       </c>
-      <c r="Z11" s="20">
-        <f>MIN(C11:Y11)</f>
+      <c r="Z11" s="18">
+        <v>796.15999999999997</v>
+      </c>
+      <c r="AA11" s="20">
+        <f>MIN(C11:Z11)</f>
         <v>685.71000000000004</v>
       </c>
-      <c r="AA11" s="21">
-        <f>MAX(C11:Y11)</f>
+      <c r="AB11" s="21">
+        <f>MAX(C11:Z11)</f>
         <v>863.60000000000002</v>
       </c>
-      <c r="AB11" s="21">
-        <f>AVERAGE(C11:Y11)</f>
-        <v>787.89588235294116</v>
-      </c>
       <c r="AC11" s="21">
-        <f>AVERAGE(Q11:Y11)</f>
-        <v>810.80444444444447</v>
-      </c>
-      <c r="AD11" s="22">
-        <f>(AC11/AB11)-1</f>
-        <v>2.9075621036487753e-002</v>
+        <f>AVERAGE(C11:Z11)</f>
+        <v>788.35500000000002</v>
+      </c>
+      <c r="AD11" s="21">
+        <f>AVERAGE(Q11:Z11)</f>
+        <v>809.33999999999992</v>
       </c>
       <c r="AE11" s="22">
-        <f>(AC11/Z11)-1</f>
-        <v>0.18243053833901279</v>
+        <f>(AD11/AC11)-1</f>
+        <v>2.6618718724432444e-002</v>
       </c>
       <c r="AF11" s="22">
-        <f>(AA11/Z11)-1</f>
+        <f>(AD11/AA11)-1</f>
+        <v>0.18029487684298018</v>
+      </c>
+      <c r="AG11" s="22">
+        <f>(AB11/AA11)-1</f>
         <v>0.25942453807002952</v>
       </c>
-      <c r="AG11" s="23" t="s">
-        <v>51</v>
+      <c r="AH11" s="23" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="12" ht="18">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="17">
@@ -2079,44 +2103,47 @@
       <c r="Y12" s="18">
         <v>547.98000000000002</v>
       </c>
-      <c r="Z12" s="20">
-        <f>MIN(C12:Y12)</f>
+      <c r="Z12" s="18">
+        <v>547.98000000000002</v>
+      </c>
+      <c r="AA12" s="20">
+        <f>MIN(C12:Z12)</f>
         <v>465</v>
       </c>
-      <c r="AA12" s="21">
-        <f>MAX(C12:Y12)</f>
+      <c r="AB12" s="21">
+        <f>MAX(C12:Z12)</f>
         <v>623.12</v>
       </c>
-      <c r="AB12" s="21">
-        <f>AVERAGE(C12:Y12)</f>
-        <v>552.63599999999974</v>
-      </c>
       <c r="AC12" s="21">
-        <f>AVERAGE(Q12:Y12)</f>
-        <v>542.19999999999993</v>
-      </c>
-      <c r="AD12" s="22">
-        <f>(AC12/AB12)-1</f>
-        <v>-1.8884039403874953e-002</v>
+        <f>AVERAGE(C12:Z12)</f>
+        <v>552.41428571428548</v>
+      </c>
+      <c r="AD12" s="21">
+        <f>AVERAGE(Q12:Z12)</f>
+        <v>542.77799999999991</v>
       </c>
       <c r="AE12" s="22">
-        <f>(AC12/Z12)-1</f>
-        <v>0.16602150537634386</v>
+        <f>(AD12/AC12)-1</f>
+        <v>-1.7443947348004585e-002</v>
       </c>
       <c r="AF12" s="22">
-        <f>(AA12/Z12)-1</f>
+        <f>(AD12/AA12)-1</f>
+        <v>0.16726451612903204</v>
+      </c>
+      <c r="AG12" s="22">
+        <f>(AB12/AA12)-1</f>
         <v>0.34004301075268817</v>
       </c>
-      <c r="AG12" s="23" t="s">
-        <v>54</v>
+      <c r="AH12" s="23" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="13" ht="36">
       <c r="A13" s="26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C13" s="28"/>
       <c r="D13" s="25">
@@ -2152,19 +2179,19 @@
         <v>1084.8299999999999</v>
       </c>
       <c r="P13" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q13" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R13" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S13" s="30">
         <v>1426.5699999999999</v>
       </c>
       <c r="T13" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U13" s="25">
         <v>592.17999999999995</v>
@@ -2179,46 +2206,49 @@
         <v>623.23000000000002</v>
       </c>
       <c r="Y13" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z13" s="20">
-        <f>MIN(C13:Y13)</f>
+        <v>45</v>
+      </c>
+      <c r="Z13" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA13" s="20">
+        <f>MIN(C13:Z13)</f>
         <v>592.17999999999995</v>
       </c>
-      <c r="AA13" s="21">
-        <f>MAX(C13:Y13)</f>
+      <c r="AB13" s="21">
+        <f>MAX(C13:Z13)</f>
         <v>1426.5699999999999</v>
       </c>
-      <c r="AB13" s="21">
-        <f>AVERAGE(C13:Y13)</f>
+      <c r="AC13" s="21">
+        <f>AVERAGE(C13:Z13)</f>
         <v>853.96466666666674</v>
       </c>
-      <c r="AC13" s="21">
-        <f>AVERAGE(Q13:Y13)</f>
+      <c r="AD13" s="21">
+        <f>AVERAGE(Q13:Z13)</f>
         <v>771.42200000000003</v>
       </c>
-      <c r="AD13" s="22">
-        <f>(AC13/AB13)-1</f>
+      <c r="AE13" s="22">
+        <f>(AD13/AC13)-1</f>
         <v>-9.665817555293077e-002</v>
       </c>
-      <c r="AE13" s="22">
-        <f>(AC13/Z13)-1</f>
+      <c r="AF13" s="22">
+        <f>(AD13/AA13)-1</f>
         <v>0.30268161707588925</v>
       </c>
-      <c r="AF13" s="22">
-        <f>(AA13/Z13)-1</f>
+      <c r="AG13" s="22">
+        <f>(AB13/AA13)-1</f>
         <v>1.4090141511027054</v>
       </c>
-      <c r="AG13" s="23" t="s">
-        <v>57</v>
+      <c r="AH13" s="23" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="14" ht="18">
       <c r="A14" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
@@ -2275,44 +2305,47 @@
       <c r="Y14" s="18">
         <v>678</v>
       </c>
-      <c r="Z14" s="20">
-        <f>MIN(C14:Y14)</f>
+      <c r="Z14" s="18">
+        <v>597.99000000000001</v>
+      </c>
+      <c r="AA14" s="20">
+        <f>MIN(C14:Z14)</f>
         <v>580.98000000000002</v>
       </c>
-      <c r="AA14" s="21">
-        <f>MAX(C14:Y14)</f>
+      <c r="AB14" s="21">
+        <f>MAX(C14:Z14)</f>
         <v>709.99000000000001</v>
       </c>
-      <c r="AB14" s="21">
-        <f>AVERAGE(C14:Y14)</f>
-        <v>653.76499999999987</v>
-      </c>
       <c r="AC14" s="21">
-        <f>AVERAGE(Q14:Y14)</f>
-        <v>676.88333333333344</v>
-      </c>
-      <c r="AD14" s="22">
-        <f>(AC14/AB14)-1</f>
-        <v>3.5361840008770073e-002</v>
+        <f>AVERAGE(C14:Z14)</f>
+        <v>650.48411764705872</v>
+      </c>
+      <c r="AD14" s="21">
+        <f>AVERAGE(Q14:Z14)</f>
+        <v>668.99400000000003</v>
       </c>
       <c r="AE14" s="22">
-        <f>(AC14/Z14)-1</f>
-        <v>0.16507166052761435</v>
+        <f>(AD14/AC14)-1</f>
+        <v>2.8455548491937988e-002</v>
       </c>
       <c r="AF14" s="22">
-        <f>(AA14/Z14)-1</f>
+        <f>(AD14/AA14)-1</f>
+        <v>0.1514923061034803</v>
+      </c>
+      <c r="AG14" s="22">
+        <f>(AB14/AA14)-1</f>
         <v>0.22205583668973117</v>
       </c>
-      <c r="AG14" s="23" t="s">
-        <v>59</v>
+      <c r="AH14" s="23" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="15" ht="18">
       <c r="A15" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -2369,44 +2402,47 @@
       <c r="Y15" s="17">
         <v>679</v>
       </c>
-      <c r="Z15" s="20">
-        <f>MIN(C15:Y15)</f>
+      <c r="Z15" s="17">
+        <v>679</v>
+      </c>
+      <c r="AA15" s="20">
+        <f>MIN(C15:Z15)</f>
         <v>622.63</v>
       </c>
-      <c r="AA15" s="21">
-        <f>MAX(C15:Y15)</f>
+      <c r="AB15" s="21">
+        <f>MAX(C15:Z15)</f>
         <v>728.61000000000001</v>
       </c>
-      <c r="AB15" s="21">
-        <f>AVERAGE(C15:Y15)</f>
-        <v>682.04812499999991</v>
-      </c>
       <c r="AC15" s="21">
-        <f>AVERAGE(Q15:Y15)</f>
-        <v>694.21222222222218</v>
-      </c>
-      <c r="AD15" s="22">
-        <f>(AC15/AB15)-1</f>
-        <v>1.7834661186440837e-002</v>
+        <f>AVERAGE(C15:Z15)</f>
+        <v>681.86882352941166</v>
+      </c>
+      <c r="AD15" s="21">
+        <f>AVERAGE(Q15:Z15)</f>
+        <v>692.69100000000003</v>
       </c>
       <c r="AE15" s="22">
-        <f>(AC15/Z15)-1</f>
-        <v>0.11496751236243385</v>
+        <f>(AD15/AC15)-1</f>
+        <v>1.5871346653703711e-002</v>
       </c>
       <c r="AF15" s="22">
-        <f>(AA15/Z15)-1</f>
+        <f>(AD15/AA15)-1</f>
+        <v>0.11252429211570281</v>
+      </c>
+      <c r="AG15" s="22">
+        <f>(AB15/AA15)-1</f>
         <v>0.17021344940012528</v>
       </c>
-      <c r="AG15" s="23" t="s">
-        <v>61</v>
+      <c r="AH15" s="23" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="16" ht="18">
       <c r="A16" s="26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C16" s="28"/>
       <c r="D16" s="29"/>
@@ -2469,44 +2505,47 @@
       <c r="Y16" s="17">
         <v>10799.02</v>
       </c>
-      <c r="Z16" s="20">
-        <f>MIN(C16:Y16)</f>
+      <c r="Z16" s="17">
+        <v>10798.99</v>
+      </c>
+      <c r="AA16" s="20">
+        <f>MIN(C16:Z16)</f>
         <v>9100</v>
       </c>
-      <c r="AA16" s="21">
-        <f>MAX(C16:Y16)</f>
+      <c r="AB16" s="21">
+        <f>MAX(C16:Z16)</f>
         <v>11315.18</v>
       </c>
-      <c r="AB16" s="21">
-        <f>AVERAGE(C16:Y16)</f>
-        <v>9843.9163157894709</v>
-      </c>
       <c r="AC16" s="21">
-        <f>AVERAGE(Q16:Y16)</f>
-        <v>10627.263333333334</v>
-      </c>
-      <c r="AD16" s="22">
-        <f>(AC16/AB16)-1</f>
-        <v>7.9576765223754231e-002</v>
+        <f>AVERAGE(C16:Z16)</f>
+        <v>9891.6699999999964</v>
+      </c>
+      <c r="AD16" s="21">
+        <f>AVERAGE(Q16:Z16)</f>
+        <v>10644.436000000002</v>
       </c>
       <c r="AE16" s="22">
-        <f>(AC16/Z16)-1</f>
-        <v>0.16783113553113571</v>
+        <f>(AD16/AC16)-1</f>
+        <v>7.6101002156360398e-002</v>
       </c>
       <c r="AF16" s="22">
-        <f>(AA16/Z16)-1</f>
+        <f>(AD16/AA16)-1</f>
+        <v>0.16971824175824191</v>
+      </c>
+      <c r="AG16" s="22">
+        <f>(AB16/AA16)-1</f>
         <v>0.24342637362637376</v>
       </c>
-      <c r="AG16" s="23" t="s">
-        <v>63</v>
+      <c r="AH16" s="23" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="17" ht="36">
       <c r="A17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
@@ -2561,44 +2600,47 @@
       <c r="Y17" s="18">
         <v>1610.8900000000001</v>
       </c>
-      <c r="Z17" s="20">
-        <f>MIN(C17:Y17)</f>
+      <c r="Z17" s="18">
+        <v>1558.77</v>
+      </c>
+      <c r="AA17" s="20">
+        <f>MIN(C17:Z17)</f>
         <v>1297.6199999999999</v>
       </c>
-      <c r="AA17" s="21">
-        <f>MAX(C17:Y17)</f>
+      <c r="AB17" s="21">
+        <f>MAX(C17:Z17)</f>
         <v>1697.6199999999999</v>
       </c>
-      <c r="AB17" s="21">
-        <f>AVERAGE(C17:Y17)</f>
-        <v>1538.7153333333331</v>
-      </c>
       <c r="AC17" s="21">
-        <f>AVERAGE(Q17:Y17)</f>
-        <v>1584.6888888888889</v>
-      </c>
-      <c r="AD17" s="22">
-        <f>(AC17/AB17)-1</f>
-        <v>2.9877882256468258e-002</v>
+        <f>AVERAGE(C17:Z17)</f>
+        <v>1539.9687499999998</v>
+      </c>
+      <c r="AD17" s="21">
+        <f>AVERAGE(Q17:Z17)</f>
+        <v>1582.097</v>
       </c>
       <c r="AE17" s="22">
-        <f>(AC17/Z17)-1</f>
-        <v>0.22122723824300561</v>
+        <f>(AD17/AC17)-1</f>
+        <v>2.7356561618539388e-002</v>
       </c>
       <c r="AF17" s="22">
-        <f>(AA17/Z17)-1</f>
+        <f>(AD17/AA17)-1</f>
+        <v>0.21922982074875552</v>
+      </c>
+      <c r="AG17" s="22">
+        <f>(AB17/AA17)-1</f>
         <v>0.30825665449052875</v>
       </c>
-      <c r="AG17" s="23" t="s">
-        <v>65</v>
+      <c r="AH17" s="23" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="18" ht="18">
       <c r="A18" s="26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C18" s="28"/>
       <c r="D18" s="29"/>
@@ -2607,100 +2649,103 @@
         <v>2279</v>
       </c>
       <c r="G18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="L18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O18" s="29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="R18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="S18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="T18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="U18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="V18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="W18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X18" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Y18" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z18" s="20">
-        <f>MIN(C18:Y18)</f>
+        <v>68</v>
+      </c>
+      <c r="Z18" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="AA18" s="20">
+        <f>MIN(C18:Z18)</f>
         <v>2279</v>
       </c>
-      <c r="AA18" s="21">
-        <f>MAX(C18:Y18)</f>
+      <c r="AB18" s="21">
+        <f>MAX(C18:Z18)</f>
         <v>2279</v>
       </c>
-      <c r="AB18" s="21">
-        <f>AVERAGE(C18:Y18)</f>
+      <c r="AC18" s="21">
+        <f>AVERAGE(C18:Z18)</f>
         <v>2279</v>
       </c>
-      <c r="AC18" s="21" t="e">
-        <f>AVERAGE(Q18:Y18)</f>
+      <c r="AD18" s="21" t="e">
+        <f>AVERAGE(Q18:Z18)</f>
         <v>#NUM!</v>
       </c>
-      <c r="AD18" s="22" t="e">
-        <f>(AC18/AB18)-1</f>
+      <c r="AE18" s="22" t="e">
+        <f>(AD18/AC18)-1</f>
         <v>#NUM!</v>
       </c>
-      <c r="AE18" s="22" t="e">
-        <f>(AC18/Z18)-1</f>
+      <c r="AF18" s="22" t="e">
+        <f>(AD18/AA18)-1</f>
         <v>#NUM!</v>
       </c>
-      <c r="AF18" s="22">
-        <f>(AA18/Z18)-1</f>
+      <c r="AG18" s="22">
+        <f>(AB18/AA18)-1</f>
         <v>0</v>
       </c>
-      <c r="AG18" s="23" t="s">
-        <v>68</v>
+      <c r="AH18" s="23" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="19" ht="18">
       <c r="A19" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C19" s="25">
         <v>176.69</v>
@@ -2765,44 +2810,47 @@
       <c r="Y19" s="30">
         <v>260</v>
       </c>
-      <c r="Z19" s="20">
-        <f>MIN(C19:Y19)</f>
+      <c r="Z19" s="30">
+        <v>260</v>
+      </c>
+      <c r="AA19" s="20">
+        <f>MIN(C19:Z19)</f>
         <v>145</v>
       </c>
-      <c r="AA19" s="21">
-        <f>MAX(C19:Y19)</f>
+      <c r="AB19" s="21">
+        <f>MAX(C19:Z19)</f>
         <v>260</v>
       </c>
-      <c r="AB19" s="21">
-        <f>AVERAGE(C19:Y19)</f>
-        <v>200.94649999999996</v>
-      </c>
       <c r="AC19" s="21">
-        <f>AVERAGE(Q19:Y19)</f>
-        <v>236.94444444444446</v>
-      </c>
-      <c r="AD19" s="22">
-        <f>(AC19/AB19)-1</f>
-        <v>0.17914193302418568</v>
+        <f>AVERAGE(C19:Z19)</f>
+        <v>203.7585714285714</v>
+      </c>
+      <c r="AD19" s="21">
+        <f>AVERAGE(Q19:Z19)</f>
+        <v>239.25</v>
       </c>
       <c r="AE19" s="22">
-        <f>(AC19/Z19)-1</f>
-        <v>0.63409961685823757</v>
+        <f>(AD19/AC19)-1</f>
+        <v>0.17418373284910027</v>
       </c>
       <c r="AF19" s="22">
-        <f>(AA19/Z19)-1</f>
+        <f>(AD19/AA19)-1</f>
+        <v>0.64999999999999991</v>
+      </c>
+      <c r="AG19" s="22">
+        <f>(AB19/AA19)-1</f>
         <v>0.7931034482758621</v>
       </c>
-      <c r="AG19" s="23" t="s">
-        <v>70</v>
+      <c r="AH19" s="23" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="20" ht="18">
       <c r="A20" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
@@ -2851,7 +2899,7 @@
         <v>212.31</v>
       </c>
       <c r="U20" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V20" s="19">
         <v>229.94999999999999</v>
@@ -2865,44 +2913,47 @@
       <c r="Y20" s="30">
         <v>270</v>
       </c>
-      <c r="Z20" s="20">
-        <f>MIN(C20:Y20)</f>
+      <c r="Z20" s="30">
+        <v>270</v>
+      </c>
+      <c r="AA20" s="20">
+        <f>MIN(C20:Z20)</f>
         <v>176.91999999999999</v>
       </c>
-      <c r="AA20" s="21">
-        <f>MAX(C20:Y20)</f>
+      <c r="AB20" s="21">
+        <f>MAX(C20:Z20)</f>
         <v>270</v>
       </c>
-      <c r="AB20" s="21">
-        <f>AVERAGE(C20:Y20)</f>
-        <v>200.04277777777779</v>
-      </c>
       <c r="AC20" s="21">
-        <f>AVERAGE(Q20:Y20)</f>
-        <v>224.64875000000001</v>
-      </c>
-      <c r="AD20" s="22">
-        <f>(AC20/AB20)-1</f>
-        <v>0.12300355201804059</v>
+        <f>AVERAGE(C20:Z20)</f>
+        <v>203.72473684210527</v>
+      </c>
+      <c r="AD20" s="21">
+        <f>AVERAGE(Q20:Z20)</f>
+        <v>229.6877777777778</v>
       </c>
       <c r="AE20" s="22">
-        <f>(AC20/Z20)-1</f>
-        <v>0.26977588740673775</v>
+        <f>(AD20/AC20)-1</f>
+        <v>0.12744176940964658</v>
       </c>
       <c r="AF20" s="22">
-        <f>(AA20/Z20)-1</f>
+        <f>(AD20/AA20)-1</f>
+        <v>0.2982578440977719</v>
+      </c>
+      <c r="AG20" s="22">
+        <f>(AB20/AA20)-1</f>
         <v>0.52611349762604576</v>
       </c>
-      <c r="AG20" s="23" t="s">
-        <v>72</v>
+      <c r="AH20" s="23" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="21" ht="18">
       <c r="A21" s="26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C21" s="29"/>
       <c r="D21" s="29"/>
@@ -2915,31 +2966,31 @@
         <v>396.77999999999997</v>
       </c>
       <c r="I21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O21" s="29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P21" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q21" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R21" s="17">
         <v>413</v>
@@ -2951,7 +3002,7 @@
         <v>408.87</v>
       </c>
       <c r="U21" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V21" s="17">
         <v>453.04000000000002</v>
@@ -2965,44 +3016,47 @@
       <c r="Y21" s="17">
         <v>349</v>
       </c>
-      <c r="Z21" s="20">
-        <f>MIN(C21:Y21)</f>
+      <c r="Z21" s="17">
         <v>349</v>
       </c>
-      <c r="AA21" s="21">
-        <f>MAX(C21:Y21)</f>
+      <c r="AA21" s="20">
+        <f>MIN(C21:Z21)</f>
+        <v>349</v>
+      </c>
+      <c r="AB21" s="21">
+        <f>MAX(C21:Z21)</f>
         <v>453.04000000000002</v>
       </c>
-      <c r="AB21" s="21">
-        <f>AVERAGE(C21:Y21)</f>
-        <v>408.05888888888887</v>
-      </c>
       <c r="AC21" s="21">
-        <f>AVERAGE(Q21:Y21)</f>
-        <v>411.28142857142853</v>
-      </c>
-      <c r="AD21" s="22">
-        <f>(AC21/AB21)-1</f>
-        <v>7.8972417224247859e-003</v>
+        <f>AVERAGE(C21:Z21)</f>
+        <v>402.15299999999996</v>
+      </c>
+      <c r="AD21" s="21">
+        <f>AVERAGE(Q21:Z21)</f>
+        <v>403.49624999999997</v>
       </c>
       <c r="AE21" s="22">
-        <f>(AC21/Z21)-1</f>
-        <v>0.17845681539091274</v>
+        <f>(AD21/AC21)-1</f>
+        <v>3.3401466605993413e-003</v>
       </c>
       <c r="AF21" s="22">
-        <f>(AA21/Z21)-1</f>
+        <f>(AD21/AA21)-1</f>
+        <v>0.15614971346704865</v>
+      </c>
+      <c r="AG21" s="22">
+        <f>(AB21/AA21)-1</f>
         <v>0.29810888252148993</v>
       </c>
-      <c r="AG21" s="32" t="s">
-        <v>74</v>
+      <c r="AH21" s="32" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="22" ht="54">
       <c r="A22" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
@@ -3065,44 +3119,47 @@
       <c r="Y22" s="17">
         <v>600</v>
       </c>
-      <c r="Z22" s="20">
-        <f>MIN(C22:Y22)</f>
+      <c r="Z22" s="17">
+        <v>600</v>
+      </c>
+      <c r="AA22" s="20">
+        <f>MIN(C22:Z22)</f>
         <v>550</v>
       </c>
-      <c r="AA22" s="21">
-        <f>MAX(C22:Y22)</f>
+      <c r="AB22" s="21">
+        <f>MAX(C22:Z22)</f>
         <v>600</v>
       </c>
-      <c r="AB22" s="21">
-        <f>AVERAGE(C22:Y22)</f>
-        <v>572.63157894736844</v>
-      </c>
       <c r="AC22" s="21">
-        <f>AVERAGE(Q22:Y22)</f>
-        <v>597.77777777777783</v>
-      </c>
-      <c r="AD22" s="22">
-        <f>(AC22/AB22)-1</f>
-        <v>4.3913398692810413e-002</v>
+        <f>AVERAGE(C22:Z22)</f>
+        <v>574</v>
+      </c>
+      <c r="AD22" s="21">
+        <f>AVERAGE(Q22:Z22)</f>
+        <v>598</v>
       </c>
       <c r="AE22" s="22">
-        <f>(AC22/Z22)-1</f>
-        <v>8.6868686868686984e-002</v>
+        <f>(AD22/AC22)-1</f>
+        <v>4.1811846689895571e-002</v>
       </c>
       <c r="AF22" s="22">
-        <f>(AA22/Z22)-1</f>
+        <f>(AD22/AA22)-1</f>
+        <v>8.7272727272727169e-002</v>
+      </c>
+      <c r="AG22" s="22">
+        <f>(AB22/AA22)-1</f>
         <v>9.0909090909090828e-002</v>
       </c>
-      <c r="AG22" s="23" t="s">
-        <v>77</v>
+      <c r="AH22" s="23" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="23" ht="18">
       <c r="A23" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
@@ -3165,44 +3222,47 @@
       <c r="Y23" s="19">
         <v>549</v>
       </c>
-      <c r="Z23" s="20">
-        <f>MIN(C23:Y23)</f>
+      <c r="Z23" s="19">
+        <v>549</v>
+      </c>
+      <c r="AA23" s="20">
+        <f>MIN(C23:Z23)</f>
         <v>329</v>
       </c>
-      <c r="AA23" s="21">
-        <f>MAX(C23:Y23)</f>
+      <c r="AB23" s="21">
+        <f>MAX(C23:Z23)</f>
         <v>549</v>
       </c>
-      <c r="AB23" s="21">
-        <f>AVERAGE(C23:Y23)</f>
-        <v>483.14473684210526</v>
-      </c>
       <c r="AC23" s="21">
-        <f>AVERAGE(Q23:Y23)</f>
-        <v>527.20555555555563</v>
-      </c>
-      <c r="AD23" s="22">
-        <f>(AC23/AB23)-1</f>
-        <v>9.1195899186313101e-002</v>
+        <f>AVERAGE(C23:Z23)</f>
+        <v>486.4375</v>
+      </c>
+      <c r="AD23" s="21">
+        <f>AVERAGE(Q23:Z23)</f>
+        <v>529.38499999999999</v>
       </c>
       <c r="AE23" s="22">
-        <f>(AC23/Z23)-1</f>
-        <v>0.60244849712934845</v>
+        <f>(AD23/AC23)-1</f>
+        <v>8.8289862520878781e-002</v>
       </c>
       <c r="AF23" s="22">
-        <f>(AA23/Z23)-1</f>
+        <f>(AD23/AA23)-1</f>
+        <v>0.60907294832826753</v>
+      </c>
+      <c r="AG23" s="22">
+        <f>(AB23/AA23)-1</f>
         <v>0.66869300911854102</v>
       </c>
-      <c r="AG23" s="23" t="s">
-        <v>80</v>
+      <c r="AH23" s="23" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="24" ht="18">
       <c r="A24" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
@@ -3265,44 +3325,47 @@
       <c r="Y24" s="18">
         <v>472.97000000000003</v>
       </c>
-      <c r="Z24" s="20">
-        <f>MIN(C24:Y24)</f>
+      <c r="Z24" s="18">
+        <v>435.14999999999998</v>
+      </c>
+      <c r="AA24" s="20">
+        <f>MIN(C24:Z24)</f>
         <v>371.14999999999998</v>
       </c>
-      <c r="AA24" s="21">
-        <f>MAX(C24:Y24)</f>
+      <c r="AB24" s="21">
+        <f>MAX(C24:Z24)</f>
         <v>513.71000000000004</v>
       </c>
-      <c r="AB24" s="21">
-        <f>AVERAGE(C24:Y24)</f>
-        <v>446.79263157894724</v>
-      </c>
       <c r="AC24" s="21">
-        <f>AVERAGE(Q24:Y24)</f>
-        <v>474.48222222222222</v>
-      </c>
-      <c r="AD24" s="22">
-        <f>(AC24/AB24)-1</f>
-        <v>6.1974143453129571e-002</v>
+        <f>AVERAGE(C24:Z24)</f>
+        <v>446.21049999999985</v>
+      </c>
+      <c r="AD24" s="21">
+        <f>AVERAGE(Q24:Z24)</f>
+        <v>470.54899999999998</v>
       </c>
       <c r="AE24" s="22">
-        <f>(AC24/Z24)-1</f>
-        <v>0.27841094496085739</v>
+        <f>(AD24/AC24)-1</f>
+        <v>5.454488408497804e-002</v>
       </c>
       <c r="AF24" s="22">
-        <f>(AA24/Z24)-1</f>
+        <f>(AD24/AA24)-1</f>
+        <v>0.26781355247204641</v>
+      </c>
+      <c r="AG24" s="22">
+        <f>(AB24/AA24)-1</f>
         <v>0.38410346221204383</v>
       </c>
-      <c r="AG24" s="23" t="s">
-        <v>82</v>
+      <c r="AH24" s="23" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="25" ht="36">
       <c r="A25" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C25" s="29"/>
       <c r="D25" s="29"/>
@@ -3369,44 +3432,47 @@
       <c r="Y25" s="30">
         <v>619.59000000000003</v>
       </c>
-      <c r="Z25" s="20">
-        <f>MIN(C25:Y25)</f>
+      <c r="Z25" s="30">
+        <v>619.58000000000004</v>
+      </c>
+      <c r="AA25" s="20">
+        <f>MIN(C25:Z25)</f>
         <v>396</v>
       </c>
-      <c r="AA25" s="21">
-        <f>MAX(C25:Y25)</f>
+      <c r="AB25" s="21">
+        <f>MAX(C25:Z25)</f>
         <v>619.59000000000003</v>
       </c>
-      <c r="AB25" s="21">
-        <f>AVERAGE(C25:Y25)</f>
-        <v>532.2395238095238</v>
-      </c>
       <c r="AC25" s="21">
-        <f>AVERAGE(Q25:Y25)</f>
-        <v>569.80888888888887</v>
-      </c>
-      <c r="AD25" s="22">
-        <f>(AC25/AB25)-1</f>
-        <v>7.0587326567671971e-002</v>
+        <f>AVERAGE(C25:Z25)</f>
+        <v>536.20954545454549</v>
+      </c>
+      <c r="AD25" s="21">
+        <f>AVERAGE(Q25:Z25)</f>
+        <v>574.78599999999994</v>
       </c>
       <c r="AE25" s="22">
-        <f>(AC25/Z25)-1</f>
-        <v>0.4389113355780021</v>
+        <f>(AD25/AC25)-1</f>
+        <v>7.1942871723317037e-002</v>
       </c>
       <c r="AF25" s="22">
-        <f>(AA25/Z25)-1</f>
+        <f>(AD25/AA25)-1</f>
+        <v>0.45147979797979776</v>
+      </c>
+      <c r="AG25" s="22">
+        <f>(AB25/AA25)-1</f>
         <v>0.56462121212121219</v>
       </c>
-      <c r="AG25" s="23" t="s">
-        <v>85</v>
+      <c r="AH25" s="23" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="26" ht="18">
       <c r="A26" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="25">
@@ -3471,44 +3537,47 @@
       <c r="Y26" s="30">
         <v>1592.45</v>
       </c>
-      <c r="Z26" s="20">
-        <f>MIN(C26:Y26)</f>
+      <c r="Z26" s="30">
+        <v>1561.8099999999999</v>
+      </c>
+      <c r="AA26" s="20">
+        <f>MIN(C26:Z26)</f>
         <v>370</v>
       </c>
-      <c r="AA26" s="21">
-        <f>MAX(C26:Y26)</f>
+      <c r="AB26" s="21">
+        <f>MAX(C26:Z26)</f>
         <v>1678.0799999999999</v>
       </c>
-      <c r="AB26" s="21">
-        <f>AVERAGE(C26:Y26)</f>
-        <v>1169.4424999999999</v>
-      </c>
       <c r="AC26" s="21">
-        <f>AVERAGE(Q26:Y26)</f>
-        <v>1337.3800000000001</v>
-      </c>
-      <c r="AD26" s="22">
-        <f>(AC26/AB26)-1</f>
-        <v>0.14360475183687971</v>
+        <f>AVERAGE(C26:Z26)</f>
+        <v>1188.1266666666666</v>
+      </c>
+      <c r="AD26" s="21">
+        <f>AVERAGE(Q26:Z26)</f>
+        <v>1359.8229999999999</v>
       </c>
       <c r="AE26" s="22">
-        <f>(AC26/Z26)-1</f>
-        <v>2.6145405405405406</v>
+        <f>(AD26/AC26)-1</f>
+        <v>0.14451012518306139</v>
       </c>
       <c r="AF26" s="22">
-        <f>(AA26/Z26)-1</f>
+        <f>(AD26/AA26)-1</f>
+        <v>2.6751972972972968</v>
+      </c>
+      <c r="AG26" s="22">
+        <f>(AB26/AA26)-1</f>
         <v>3.535351351351351</v>
       </c>
-      <c r="AG26" s="23" t="s">
-        <v>87</v>
+      <c r="AH26" s="23" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="27" ht="18">
       <c r="A27" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
@@ -3563,44 +3632,47 @@
       <c r="Y27" s="19">
         <v>166.99000000000001</v>
       </c>
-      <c r="Z27" s="20">
-        <f>MIN(C27:Y27)</f>
+      <c r="Z27" s="19">
+        <v>166.99000000000001</v>
+      </c>
+      <c r="AA27" s="20">
+        <f>MIN(C27:Z27)</f>
         <v>109.98999999999999</v>
       </c>
-      <c r="AA27" s="21">
-        <f>MAX(C27:Y27)</f>
+      <c r="AB27" s="21">
+        <f>MAX(C27:Z27)</f>
         <v>166.99000000000001</v>
       </c>
-      <c r="AB27" s="21">
-        <f>AVERAGE(C27:Y27)</f>
-        <v>147.83933333333334</v>
-      </c>
       <c r="AC27" s="21">
-        <f>AVERAGE(Q27:Y27)</f>
-        <v>159.10111111111112</v>
-      </c>
-      <c r="AD27" s="22">
-        <f>(AC27/AB27)-1</f>
-        <v>7.6175788430984381e-002</v>
+        <f>AVERAGE(C27:Z27)</f>
+        <v>149.03625</v>
+      </c>
+      <c r="AD27" s="21">
+        <f>AVERAGE(Q27:Z27)</f>
+        <v>159.89000000000001</v>
       </c>
       <c r="AE27" s="22">
-        <f>(AC27/Z27)-1</f>
-        <v>0.4465052378499057</v>
+        <f>(AD27/AC27)-1</f>
+        <v>7.2826241937783642e-002</v>
       </c>
       <c r="AF27" s="22">
-        <f>(AA27/Z27)-1</f>
+        <f>(AD27/AA27)-1</f>
+        <v>0.45367760705518712</v>
+      </c>
+      <c r="AG27" s="22">
+        <f>(AB27/AA27)-1</f>
         <v>0.51822892990271852</v>
       </c>
-      <c r="AG27" s="23" t="s">
-        <v>89</v>
+      <c r="AH27" s="23" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="28" ht="18">
       <c r="A28" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" s="29"/>
       <c r="D28" s="29"/>
@@ -3655,44 +3727,47 @@
       <c r="Y28" s="18">
         <v>81.480000000000004</v>
       </c>
-      <c r="Z28" s="20">
-        <f>MIN(C28:Y28)</f>
+      <c r="Z28" s="18">
+        <v>81.480000000000004</v>
+      </c>
+      <c r="AA28" s="20">
+        <f>MIN(C28:Z28)</f>
         <v>68</v>
       </c>
-      <c r="AA28" s="21">
-        <f>MAX(C28:Y28)</f>
+      <c r="AB28" s="21">
+        <f>MAX(C28:Z28)</f>
         <v>85.700000000000003</v>
       </c>
-      <c r="AB28" s="21">
-        <f>AVERAGE(C28:Y28)</f>
-        <v>78.812666666666672</v>
-      </c>
       <c r="AC28" s="21">
-        <f>AVERAGE(Q28:Y28)</f>
-        <v>82.154444444444437</v>
-      </c>
-      <c r="AD28" s="22">
-        <f>(AC28/AB28)-1</f>
-        <v>4.240153162069249e-002</v>
+        <f>AVERAGE(C28:Z28)</f>
+        <v>78.979375000000005</v>
+      </c>
+      <c r="AD28" s="21">
+        <f>AVERAGE(Q28:Z28)</f>
+        <v>82.087000000000003</v>
       </c>
       <c r="AE28" s="22">
-        <f>(AC28/Z28)-1</f>
-        <v>0.20815359477124162</v>
+        <f>(AD28/AC28)-1</f>
+        <v>3.9347297949622995e-002</v>
       </c>
       <c r="AF28" s="22">
-        <f>(AA28/Z28)-1</f>
+        <f>(AD28/AA28)-1</f>
+        <v>0.20716176470588232</v>
+      </c>
+      <c r="AG28" s="22">
+        <f>(AB28/AA28)-1</f>
         <v>0.26029411764705879</v>
       </c>
-      <c r="AG28" s="23" t="s">
-        <v>91</v>
+      <c r="AH28" s="23" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="29" ht="18">
       <c r="A29" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -3747,44 +3822,47 @@
       <c r="Y29" s="33">
         <v>99.900000000000006</v>
       </c>
-      <c r="Z29" s="20">
-        <f>MIN(C29:Y29)</f>
+      <c r="Z29" s="33">
+        <v>99.900000000000006</v>
+      </c>
+      <c r="AA29" s="20">
+        <f>MIN(C29:Z29)</f>
         <v>55</v>
       </c>
-      <c r="AA29" s="21">
-        <f>MAX(C29:Y29)</f>
+      <c r="AB29" s="21">
+        <f>MAX(C29:Z29)</f>
         <v>111</v>
       </c>
-      <c r="AB29" s="21">
-        <f>AVERAGE(C29:Y29)</f>
-        <v>85.936000000000007</v>
-      </c>
       <c r="AC29" s="21">
-        <f>AVERAGE(Q29:Y29)</f>
-        <v>95.475555555555559</v>
-      </c>
-      <c r="AD29" s="22">
-        <f>(AC29/AB29)-1</f>
-        <v>0.11100767496224573</v>
+        <f>AVERAGE(C29:Z29)</f>
+        <v>86.808750000000018</v>
+      </c>
+      <c r="AD29" s="21">
+        <f>AVERAGE(Q29:Z29)</f>
+        <v>95.917999999999992</v>
       </c>
       <c r="AE29" s="22">
-        <f>(AC29/Z29)-1</f>
-        <v>0.73591919191919208</v>
+        <f>(AD29/AC29)-1</f>
+        <v>0.10493469840309855</v>
       </c>
       <c r="AF29" s="22">
-        <f>(AA29/Z29)-1</f>
+        <f>(AD29/AA29)-1</f>
+        <v>0.74396363636363616</v>
+      </c>
+      <c r="AG29" s="22">
+        <f>(AB29/AA29)-1</f>
         <v>1.0181818181818181</v>
       </c>
-      <c r="AG29" s="23" t="s">
-        <v>93</v>
+      <c r="AH29" s="23" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="30" ht="18">
       <c r="A30" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
@@ -3837,44 +3915,47 @@
       <c r="Y30" s="18">
         <v>89.700000000000003</v>
       </c>
-      <c r="Z30" s="20">
-        <f>MIN(C30:Y30)</f>
+      <c r="Z30" s="19">
+        <v>91</v>
+      </c>
+      <c r="AA30" s="20">
+        <f>MIN(C30:Z30)</f>
         <v>47.359999999999999</v>
       </c>
-      <c r="AA30" s="21">
-        <f>MAX(C30:Y30)</f>
+      <c r="AB30" s="21">
+        <f>MAX(C30:Z30)</f>
         <v>100.68000000000001</v>
       </c>
-      <c r="AB30" s="21">
-        <f>AVERAGE(C30:Y30)</f>
-        <v>74.729285714285723</v>
-      </c>
       <c r="AC30" s="21">
-        <f>AVERAGE(Q30:Y30)</f>
-        <v>85.973333333333358</v>
-      </c>
-      <c r="AD30" s="22">
-        <f>(AC30/AB30)-1</f>
-        <v>0.15046373736311724</v>
+        <f>AVERAGE(C30:Z30)</f>
+        <v>75.814000000000007</v>
+      </c>
+      <c r="AD30" s="21">
+        <f>AVERAGE(Q30:Z30)</f>
+        <v>86.476000000000028</v>
       </c>
       <c r="AE30" s="22">
-        <f>(AC30/Z30)-1</f>
-        <v>0.81531531531531587</v>
+        <f>(AD30/AC30)-1</f>
+        <v>0.14063365605297196</v>
       </c>
       <c r="AF30" s="22">
-        <f>(AA30/Z30)-1</f>
+        <f>(AD30/AA30)-1</f>
+        <v>0.8259290540540547</v>
+      </c>
+      <c r="AG30" s="22">
+        <f>(AB30/AA30)-1</f>
         <v>1.1258445945945947</v>
       </c>
-      <c r="AG30" s="23" t="s">
-        <v>95</v>
+      <c r="AH30" s="23" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="31" ht="18">
       <c r="A31" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="29"/>
@@ -3910,7 +3991,7 @@
         <v>132.33000000000001</v>
       </c>
       <c r="T31" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U31" s="18">
         <v>156</v>
@@ -3927,44 +4008,47 @@
       <c r="Y31" s="18">
         <v>151.22</v>
       </c>
-      <c r="Z31" s="20">
-        <f>MIN(C31:Y31)</f>
+      <c r="Z31" s="18">
+        <v>151.22</v>
+      </c>
+      <c r="AA31" s="20">
+        <f>MIN(C31:Z31)</f>
         <v>92.5</v>
       </c>
-      <c r="AA31" s="21">
-        <f>MAX(C31:Y31)</f>
+      <c r="AB31" s="21">
+        <f>MAX(C31:Z31)</f>
         <v>156</v>
       </c>
-      <c r="AB31" s="21">
-        <f>AVERAGE(C31:Y31)</f>
-        <v>127.68461538461541</v>
-      </c>
       <c r="AC31" s="21">
-        <f>AVERAGE(Q31:Y31)</f>
-        <v>141.30125000000001</v>
-      </c>
-      <c r="AD31" s="22">
-        <f>(AC31/AB31)-1</f>
-        <v>0.10664271944093007</v>
+        <f>AVERAGE(C31:Z31)</f>
+        <v>129.36571428571432</v>
+      </c>
+      <c r="AD31" s="21">
+        <f>AVERAGE(Q31:Z31)</f>
+        <v>142.40333333333334</v>
       </c>
       <c r="AE31" s="22">
-        <f>(AC31/Z31)-1</f>
-        <v>0.52758108108108126</v>
+        <f>(AD31/AC31)-1</f>
+        <v>0.10078110046085631</v>
       </c>
       <c r="AF31" s="22">
-        <f>(AA31/Z31)-1</f>
+        <f>(AD31/AA31)-1</f>
+        <v>0.53949549549549558</v>
+      </c>
+      <c r="AG31" s="22">
+        <f>(AB31/AA31)-1</f>
         <v>0.68648648648648658</v>
       </c>
-      <c r="AG31" s="23" t="s">
-        <v>97</v>
+      <c r="AH31" s="23" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="32" ht="18">
       <c r="A32" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -4015,44 +4099,47 @@
       <c r="Y32" s="18">
         <v>221.25</v>
       </c>
-      <c r="Z32" s="20">
-        <f>MIN(C32:Y32)</f>
+      <c r="Z32" s="17">
+        <v>209.99000000000001</v>
+      </c>
+      <c r="AA32" s="20">
+        <f>MIN(C32:Z32)</f>
         <v>148.88</v>
       </c>
-      <c r="AA32" s="21">
-        <f>MAX(C32:Y32)</f>
+      <c r="AB32" s="21">
+        <f>MAX(C32:Z32)</f>
         <v>257.87</v>
       </c>
-      <c r="AB32" s="21">
-        <f>AVERAGE(C32:Y32)</f>
-        <v>221.98615384615388</v>
-      </c>
       <c r="AC32" s="21">
-        <f>AVERAGE(Q32:Y32)</f>
-        <v>233.86000000000001</v>
-      </c>
-      <c r="AD32" s="22">
-        <f>(AC32/AB32)-1</f>
-        <v>5.3489129606143049e-002</v>
+        <f>AVERAGE(C32:Z32)</f>
+        <v>221.12928571428574</v>
+      </c>
+      <c r="AD32" s="21">
+        <f>AVERAGE(Q32:Z32)</f>
+        <v>231.47300000000004</v>
       </c>
       <c r="AE32" s="22">
-        <f>(AC32/Z32)-1</f>
-        <v>0.57079527135948438</v>
+        <f>(AD32/AC32)-1</f>
+        <v>4.6776772476347039e-002</v>
       </c>
       <c r="AF32" s="22">
-        <f>(AA32/Z32)-1</f>
+        <f>(AD32/AA32)-1</f>
+        <v>0.5547622246104249</v>
+      </c>
+      <c r="AG32" s="22">
+        <f>(AB32/AA32)-1</f>
         <v>0.73206609349811935</v>
       </c>
-      <c r="AG32" s="23" t="s">
-        <v>99</v>
+      <c r="AH32" s="23" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="33" ht="18">
       <c r="A33" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
@@ -4099,44 +4186,47 @@
       <c r="Y33" s="18">
         <v>168.28999999999999</v>
       </c>
-      <c r="Z33" s="20">
-        <f>MIN(C33:Y33)</f>
+      <c r="Z33" s="18">
+        <v>149.88999999999999</v>
+      </c>
+      <c r="AA33" s="20">
+        <f>MIN(C33:Z33)</f>
         <v>144.94999999999999</v>
       </c>
-      <c r="AA33" s="21">
-        <f>MAX(C33:Y33)</f>
+      <c r="AB33" s="21">
+        <f>MAX(C33:Z33)</f>
         <v>168.28999999999999</v>
       </c>
-      <c r="AB33" s="21">
-        <f>AVERAGE(C33:Y33)</f>
-        <v>156.73727272727274</v>
-      </c>
       <c r="AC33" s="21">
-        <f>AVERAGE(Q33:Y33)</f>
-        <v>157.29666666666668</v>
-      </c>
-      <c r="AD33" s="22">
-        <f>(AC33/AB33)-1</f>
-        <v>3.5689911509899641e-003</v>
+        <f>AVERAGE(C33:Z33)</f>
+        <v>156.16666666666666</v>
+      </c>
+      <c r="AD33" s="21">
+        <f>AVERAGE(Q33:Z33)</f>
+        <v>156.55599999999998</v>
       </c>
       <c r="AE33" s="22">
-        <f>(AC33/Z33)-1</f>
-        <v>8.517879728642086e-002</v>
+        <f>(AD33/AC33)-1</f>
+        <v>2.493062966915538e-003</v>
       </c>
       <c r="AF33" s="22">
-        <f>(AA33/Z33)-1</f>
+        <f>(AD33/AA33)-1</f>
+        <v>8.0068989306657512e-002</v>
+      </c>
+      <c r="AG33" s="22">
+        <f>(AB33/AA33)-1</f>
         <v>0.16102104173853049</v>
       </c>
-      <c r="AG33" s="23" t="s">
-        <v>101</v>
+      <c r="AH33" s="23" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="34" ht="18">
       <c r="A34" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B34" s="27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C34" s="29"/>
       <c r="D34" s="29"/>
@@ -4183,44 +4273,47 @@
       <c r="Y34" s="18">
         <v>159</v>
       </c>
-      <c r="Z34" s="20">
-        <f>MIN(C34:Y34)</f>
+      <c r="Z34" s="19">
+        <v>195.22999999999999</v>
+      </c>
+      <c r="AA34" s="20">
+        <f>MIN(C34:Z34)</f>
         <v>144</v>
       </c>
-      <c r="AA34" s="21">
-        <f>MAX(C34:Y34)</f>
+      <c r="AB34" s="21">
+        <f>MAX(C34:Z34)</f>
         <v>199.94999999999999</v>
       </c>
-      <c r="AB34" s="21">
-        <f>AVERAGE(C34:Y34)</f>
-        <v>177.22636363636363</v>
-      </c>
       <c r="AC34" s="21">
-        <f>AVERAGE(Q34:Y34)</f>
-        <v>176.40666666666664</v>
-      </c>
-      <c r="AD34" s="22">
-        <f>(AC34/AB34)-1</f>
-        <v>-4.6251412762655653e-003</v>
+        <f>AVERAGE(C34:Z34)</f>
+        <v>178.72666666666666</v>
+      </c>
+      <c r="AD34" s="21">
+        <f>AVERAGE(Q34:Z34)</f>
+        <v>178.28899999999999</v>
       </c>
       <c r="AE34" s="22">
-        <f>(AC34/Z34)-1</f>
-        <v>0.22504629629629602</v>
+        <f>(AD34/AC34)-1</f>
+        <v>-2.4488045059495311e-003</v>
       </c>
       <c r="AF34" s="22">
-        <f>(AA34/Z34)-1</f>
+        <f>(AD34/AA34)-1</f>
+        <v>0.23811805555555554</v>
+      </c>
+      <c r="AG34" s="22">
+        <f>(AB34/AA34)-1</f>
         <v>0.38854166666666656</v>
       </c>
-      <c r="AG34" s="23" t="s">
-        <v>103</v>
+      <c r="AH34" s="23" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="35" ht="18">
       <c r="A35" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -4245,7 +4338,7 @@
         <v>31941.080000000002</v>
       </c>
       <c r="M35" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N35" s="18"/>
       <c r="O35" s="17"/>
@@ -4259,44 +4352,45 @@
       <c r="W35" s="17"/>
       <c r="X35" s="17"/>
       <c r="Y35" s="17"/>
-      <c r="Z35" s="20">
-        <f>MIN(C35:Y35)</f>
+      <c r="Z35" s="17"/>
+      <c r="AA35" s="20">
+        <f>MIN(C35:Z35)</f>
         <v>30731.380000000001</v>
       </c>
-      <c r="AA35" s="21">
-        <f>MAX(C35:Y35)</f>
+      <c r="AB35" s="21">
+        <f>MAX(C35:Z35)</f>
         <v>32790.889999999999</v>
       </c>
-      <c r="AB35" s="21">
-        <f>AVERAGE(C35:Y35)</f>
+      <c r="AC35" s="21">
+        <f>AVERAGE(C35:Z35)</f>
         <v>31912.133333333331</v>
       </c>
-      <c r="AC35" s="21" t="e">
-        <f>AVERAGE(Q35:Y35)</f>
+      <c r="AD35" s="21" t="e">
+        <f>AVERAGE(Q35:Z35)</f>
         <v>#NUM!</v>
       </c>
-      <c r="AD35" s="22" t="e">
-        <f>(AC35/AB35)-1</f>
+      <c r="AE35" s="22" t="e">
+        <f>(AD35/AC35)-1</f>
         <v>#NUM!</v>
       </c>
-      <c r="AE35" s="22" t="e">
-        <f>(AC35/Z35)-1</f>
+      <c r="AF35" s="22" t="e">
+        <f>(AD35/AA35)-1</f>
         <v>#NUM!</v>
       </c>
-      <c r="AF35" s="22">
-        <f>(AA35/Z35)-1</f>
+      <c r="AG35" s="22">
+        <f>(AB35/AA35)-1</f>
         <v>6.7016515366377982e-002</v>
       </c>
-      <c r="AG35" s="23" t="s">
-        <v>106</v>
+      <c r="AH35" s="23" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="36" ht="18">
       <c r="A36" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
@@ -4328,61 +4422,64 @@
         <v>721.67999999999995</v>
       </c>
       <c r="T36" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="U36" s="17">
+        <v>45</v>
+      </c>
+      <c r="U36" s="19">
         <v>1164</v>
       </c>
-      <c r="V36" s="17">
+      <c r="V36" s="19">
         <v>1150.8</v>
       </c>
-      <c r="W36" s="17">
+      <c r="W36" s="19">
         <v>1150.8</v>
       </c>
-      <c r="X36" s="17">
+      <c r="X36" s="19">
         <v>1150.8</v>
       </c>
-      <c r="Y36" s="17">
+      <c r="Y36" s="19">
         <v>1150.8</v>
       </c>
-      <c r="Z36" s="20">
-        <f>MIN(C36:Y36)</f>
+      <c r="Z36" s="30">
+        <v>1360.8</v>
+      </c>
+      <c r="AA36" s="20">
+        <f>MIN(C36:Z36)</f>
         <v>642.82000000000005</v>
       </c>
-      <c r="AA36" s="21">
-        <f>MAX(C36:Y36)</f>
-        <v>1164</v>
-      </c>
       <c r="AB36" s="21">
-        <f>AVERAGE(C36:Y36)</f>
-        <v>903.59636363636355</v>
+        <f>MAX(C36:Z36)</f>
+        <v>1360.8</v>
       </c>
       <c r="AC36" s="21">
-        <f>AVERAGE(Q36:Y36)</f>
-        <v>991.53000000000009</v>
-      </c>
-      <c r="AD36" s="22">
-        <f>(AC36/AB36)-1</f>
-        <v>9.7315172905038327e-002</v>
+        <f>AVERAGE(C36:Z36)</f>
+        <v>941.6966666666666</v>
+      </c>
+      <c r="AD36" s="21">
+        <f>AVERAGE(Q36:Z36)</f>
+        <v>1032.5600000000002</v>
       </c>
       <c r="AE36" s="22">
-        <f>(AC36/Z36)-1</f>
-        <v>0.54246912043806983</v>
+        <f>(AD36/AC36)-1</f>
+        <v>9.6488961413618846e-002</v>
       </c>
       <c r="AF36" s="22">
-        <f>(AA36/Z36)-1</f>
-        <v>0.81077128900780915</v>
-      </c>
-      <c r="AG36" s="23" t="s">
-        <v>109</v>
+        <f>(AD36/AA36)-1</f>
+        <v>0.60629725273015778</v>
+      </c>
+      <c r="AG36" s="22">
+        <f>(AB36/AA36)-1</f>
+        <v>1.1169223110668614</v>
+      </c>
+      <c r="AH36" s="23" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="37" ht="18">
       <c r="A37" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
@@ -4431,44 +4528,47 @@
       <c r="Y37" s="30">
         <v>2016</v>
       </c>
-      <c r="Z37" s="20">
-        <f>MIN(C37:Y37)</f>
+      <c r="Z37" s="30">
+        <v>2171.4000000000001</v>
+      </c>
+      <c r="AA37" s="20">
+        <f>MIN(C37:Z37)</f>
         <v>1151.71</v>
       </c>
-      <c r="AA37" s="21">
-        <f>MAX(C37:Y37)</f>
-        <v>2064</v>
-      </c>
       <c r="AB37" s="21">
-        <f>AVERAGE(C37:Y37)</f>
-        <v>1634.5116666666665</v>
+        <f>MAX(C37:Z37)</f>
+        <v>2171.4000000000001</v>
       </c>
       <c r="AC37" s="21">
-        <f>AVERAGE(Q37:Y37)</f>
-        <v>1781.2266666666667</v>
-      </c>
-      <c r="AD37" s="22">
-        <f>(AC37/AB37)-1</f>
-        <v>8.9760754231386297e-002</v>
+        <f>AVERAGE(C37:Z37)</f>
+        <v>1675.8107692307692</v>
+      </c>
+      <c r="AD37" s="21">
+        <f>AVERAGE(Q37:Z37)</f>
+        <v>1820.2440000000001</v>
       </c>
       <c r="AE37" s="22">
-        <f>(AC37/Z37)-1</f>
-        <v>0.5465930370203147</v>
+        <f>(AD37/AC37)-1</f>
+        <v>8.6187076381857075e-002</v>
       </c>
       <c r="AF37" s="22">
-        <f>(AA37/Z37)-1</f>
-        <v>0.79211780743416305</v>
-      </c>
-      <c r="AG37" s="23" t="s">
-        <v>109</v>
+        <f>(AD37/AA37)-1</f>
+        <v>0.58047077823410409</v>
+      </c>
+      <c r="AG37" s="22">
+        <f>(AB37/AA37)-1</f>
+        <v>0.88537044915820817</v>
+      </c>
+      <c r="AH37" s="23" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="38" ht="18">
       <c r="A38" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>
@@ -4503,58 +4603,61 @@
         <v>3876</v>
       </c>
       <c r="U38" s="36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V38" s="36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W38" s="36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X38" s="36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Y38" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z38" s="20">
-        <f>MIN(C38:Y38)</f>
+        <v>45</v>
+      </c>
+      <c r="Z38" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA38" s="20">
+        <f>MIN(C38:Z38)</f>
         <v>2159.8299999999999</v>
       </c>
-      <c r="AA38" s="21">
-        <f>MAX(C38:Y38)</f>
+      <c r="AB38" s="21">
+        <f>MAX(C38:Z38)</f>
         <v>3876</v>
       </c>
-      <c r="AB38" s="21">
-        <f>AVERAGE(C38:Y38)</f>
+      <c r="AC38" s="21">
+        <f>AVERAGE(C38:Z38)</f>
         <v>2544.02</v>
       </c>
-      <c r="AC38" s="21">
-        <f>AVERAGE(Q38:Y38)</f>
+      <c r="AD38" s="21">
+        <f>AVERAGE(Q38:Z38)</f>
         <v>2771.3400000000001</v>
       </c>
-      <c r="AD38" s="22">
-        <f>(AC38/AB38)-1</f>
+      <c r="AE38" s="22">
+        <f>(AD38/AC38)-1</f>
         <v>8.9354643438337877e-002</v>
       </c>
-      <c r="AE38" s="22">
-        <f>(AC38/Z38)-1</f>
+      <c r="AF38" s="22">
+        <f>(AD38/AA38)-1</f>
         <v>0.28312876476389359</v>
       </c>
-      <c r="AF38" s="22">
-        <f>(AA38/Z38)-1</f>
+      <c r="AG38" s="22">
+        <f>(AB38/AA38)-1</f>
         <v>0.79458568498446636</v>
       </c>
-      <c r="AG38" s="23" t="s">
-        <v>109</v>
+      <c r="AH38" s="23" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="39" ht="18">
       <c r="A39" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
@@ -4603,44 +4706,47 @@
       <c r="Y39" s="30">
         <v>2218.4400000000001</v>
       </c>
-      <c r="Z39" s="20">
-        <f>MIN(C39:Y39)</f>
+      <c r="Z39" s="30">
+        <v>2804.7600000000002</v>
+      </c>
+      <c r="AA39" s="20">
+        <f>MIN(C39:Z39)</f>
         <v>1310.1800000000001</v>
       </c>
-      <c r="AA39" s="21">
-        <f>MAX(C39:Y39)</f>
-        <v>2218.4400000000001</v>
-      </c>
       <c r="AB39" s="21">
-        <f>AVERAGE(C39:Y39)</f>
-        <v>1753.9116666666666</v>
+        <f>MAX(C39:Z39)</f>
+        <v>2804.7600000000002</v>
       </c>
       <c r="AC39" s="21">
-        <f>AVERAGE(Q39:Y39)</f>
-        <v>1899.5066666666669</v>
-      </c>
-      <c r="AD39" s="22">
-        <f>(AC39/AB39)-1</f>
-        <v>8.3011592183947158e-002</v>
+        <f>AVERAGE(C39:Z39)</f>
+        <v>1834.7461538461537</v>
+      </c>
+      <c r="AD39" s="21">
+        <f>AVERAGE(Q39:Z39)</f>
+        <v>1990.0319999999999</v>
       </c>
       <c r="AE39" s="22">
-        <f>(AC39/Z39)-1</f>
-        <v>0.44980587909040493</v>
+        <f>(AD39/AC39)-1</f>
+        <v>8.4636147528268424e-002</v>
       </c>
       <c r="AF39" s="22">
-        <f>(AA39/Z39)-1</f>
-        <v>0.69323299088674828</v>
-      </c>
-      <c r="AG39" s="23" t="s">
-        <v>109</v>
+        <f>(AD39/AA39)-1</f>
+        <v>0.51889969317193052</v>
+      </c>
+      <c r="AG39" s="22">
+        <f>(AB39/AA39)-1</f>
+        <v>1.1407440199056618</v>
+      </c>
+      <c r="AH39" s="23" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="40" ht="18">
       <c r="A40" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -4677,44 +4783,47 @@
       <c r="Y40" s="19">
         <v>1592.6400000000001</v>
       </c>
-      <c r="Z40" s="20">
-        <f>MIN(C40:Y40)</f>
+      <c r="Z40" s="19">
         <v>1592.6400000000001</v>
       </c>
-      <c r="AA40" s="21">
-        <f>MAX(C40:Y40)</f>
+      <c r="AA40" s="20">
+        <f>MIN(C40:Z40)</f>
+        <v>1592.6400000000001</v>
+      </c>
+      <c r="AB40" s="21">
+        <f>MAX(C40:Z40)</f>
         <v>1896</v>
       </c>
-      <c r="AB40" s="21">
-        <f>AVERAGE(C40:Y40)</f>
-        <v>1693.76</v>
-      </c>
       <c r="AC40" s="21">
-        <f>AVERAGE(Q40:Y40)</f>
-        <v>1693.76</v>
-      </c>
-      <c r="AD40" s="22">
-        <f>(AC40/AB40)-1</f>
+        <f>AVERAGE(C40:Z40)</f>
+        <v>1679.3142857142855</v>
+      </c>
+      <c r="AD40" s="21">
+        <f>AVERAGE(Q40:Z40)</f>
+        <v>1679.3142857142855</v>
+      </c>
+      <c r="AE40" s="22">
+        <f>(AD40/AC40)-1</f>
         <v>0</v>
       </c>
-      <c r="AE40" s="22">
-        <f>(AC40/Z40)-1</f>
-        <v>6.3492063492063489e-002</v>
-      </c>
       <c r="AF40" s="22">
-        <f>(AA40/Z40)-1</f>
+        <f>(AD40/AA40)-1</f>
+        <v>5.4421768707482832e-002</v>
+      </c>
+      <c r="AG40" s="22">
+        <f>(AB40/AA40)-1</f>
         <v>0.19047619047619047</v>
       </c>
-      <c r="AG40" s="23" t="s">
-        <v>109</v>
+      <c r="AH40" s="23" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="41" ht="18">
       <c r="A41" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
@@ -4746,13 +4855,13 @@
         <v>1628.6199999999999</v>
       </c>
       <c r="T41" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U41" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V41" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W41" s="19">
         <v>1985.76</v>
@@ -4763,44 +4872,47 @@
       <c r="Y41" s="19">
         <v>1985.76</v>
       </c>
-      <c r="Z41" s="20">
-        <f>MIN(C41:Y41)</f>
+      <c r="Z41" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA41" s="20">
+        <f>MIN(C41:Z41)</f>
         <v>1480.5599999999999</v>
       </c>
-      <c r="AA41" s="21">
-        <f>MAX(C41:Y41)</f>
+      <c r="AB41" s="21">
+        <f>MAX(C41:Z41)</f>
         <v>1985.76</v>
       </c>
-      <c r="AB41" s="21">
-        <f>AVERAGE(C41:Y41)</f>
+      <c r="AC41" s="21">
+        <f>AVERAGE(C41:Z41)</f>
         <v>1714.7644444444443</v>
       </c>
-      <c r="AC41" s="21">
-        <f>AVERAGE(Q41:Y41)</f>
+      <c r="AD41" s="21">
+        <f>AVERAGE(Q41:Z41)</f>
         <v>1807.1899999999998</v>
       </c>
-      <c r="AD41" s="22">
-        <f>(AC41/AB41)-1</f>
+      <c r="AE41" s="22">
+        <f>(AD41/AC41)-1</f>
         <v>5.389985537372155e-002</v>
       </c>
-      <c r="AE41" s="22">
-        <f>(AC41/Z41)-1</f>
+      <c r="AF41" s="22">
+        <f>(AD41/AA41)-1</f>
         <v>0.22061247095693504</v>
       </c>
-      <c r="AF41" s="22">
-        <f>(AA41/Z41)-1</f>
+      <c r="AG41" s="22">
+        <f>(AB41/AA41)-1</f>
         <v>0.34122224023342529</v>
       </c>
-      <c r="AG41" s="23" t="s">
-        <v>109</v>
+      <c r="AH41" s="23" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="42" ht="18">
       <c r="A42" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C42" s="17"/>
       <c r="D42" s="17">
@@ -4827,41 +4939,42 @@
       <c r="W42" s="17"/>
       <c r="X42" s="17"/>
       <c r="Y42" s="17"/>
-      <c r="Z42" s="20">
-        <f>MIN(C42:Y42)</f>
+      <c r="Z42" s="17"/>
+      <c r="AA42" s="20">
+        <f>MIN(C42:Z42)</f>
         <v>339.45999999999998</v>
       </c>
-      <c r="AA42" s="21">
-        <f>MAX(C42:Y42)</f>
+      <c r="AB42" s="21">
+        <f>MAX(C42:Z42)</f>
         <v>339.45999999999998</v>
       </c>
-      <c r="AB42" s="21">
-        <f>AVERAGE(C42:Y42)</f>
+      <c r="AC42" s="21">
+        <f>AVERAGE(C42:Z42)</f>
         <v>339.45999999999998</v>
       </c>
-      <c r="AC42" s="21" t="e">
-        <f>AVERAGE(Q42:Y42)</f>
+      <c r="AD42" s="21" t="e">
+        <f>AVERAGE(Q42:Z42)</f>
         <v>#NUM!</v>
       </c>
-      <c r="AD42" s="22" t="e">
-        <f>(AC42/AB42)-1</f>
+      <c r="AE42" s="22" t="e">
+        <f>(AD42/AC42)-1</f>
         <v>#NUM!</v>
       </c>
-      <c r="AE42" s="22" t="e">
-        <f>(AC42/Z42)-1</f>
+      <c r="AF42" s="22" t="e">
+        <f>(AD42/AA42)-1</f>
         <v>#NUM!</v>
       </c>
-      <c r="AF42" s="22">
-        <f>(AA42/Z42)-1</f>
+      <c r="AG42" s="22">
+        <f>(AB42/AA42)-1</f>
         <v>0</v>
       </c>
     </row>
     <row r="43" ht="18">
       <c r="A43" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>
@@ -4924,44 +5037,47 @@
       <c r="Y43" s="17">
         <v>378.99000000000001</v>
       </c>
-      <c r="Z43" s="20">
-        <f>MIN(C43:Y43)</f>
+      <c r="Z43" s="17">
         <v>378.99000000000001</v>
       </c>
-      <c r="AA43" s="21">
-        <f>MAX(C43:Y43)</f>
+      <c r="AA43" s="20">
+        <f>MIN(C43:Z43)</f>
         <v>378.99000000000001</v>
       </c>
       <c r="AB43" s="21">
-        <f>AVERAGE(C43:Y43)</f>
+        <f>MAX(C43:Z43)</f>
+        <v>378.99000000000001</v>
+      </c>
+      <c r="AC43" s="21">
+        <f>AVERAGE(C43:Z43)</f>
         <v>378.9899999999999</v>
       </c>
-      <c r="AC43" s="21">
-        <f>AVERAGE(Q43:Y43)</f>
-        <v>378.99000000000001</v>
-      </c>
-      <c r="AD43" s="22">
-        <f>(AC43/AB43)-1</f>
+      <c r="AD43" s="21">
+        <f>AVERAGE(Q43:Z43)</f>
+        <v>378.98999999999995</v>
+      </c>
+      <c r="AE43" s="22">
+        <f>(AD43/AC43)-1</f>
         <v>2.2204460492503131e-016</v>
       </c>
-      <c r="AE43" s="22">
-        <f>(AC43/Z43)-1</f>
+      <c r="AF43" s="22">
+        <f>(AD43/AA43)-1</f>
+        <v>-1.1102230246251565e-016</v>
+      </c>
+      <c r="AG43" s="22">
+        <f>(AB43/AA43)-1</f>
         <v>0</v>
       </c>
-      <c r="AF43" s="22">
-        <f>(AA43/Z43)-1</f>
-        <v>0</v>
-      </c>
-      <c r="AG43" s="23" t="s">
-        <v>120</v>
+      <c r="AH43" s="23" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="44" ht="18">
       <c r="A44" s="26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C44" s="29"/>
       <c r="D44" s="29"/>
@@ -5024,44 +5140,47 @@
       <c r="Y44" s="30">
         <v>191.19</v>
       </c>
-      <c r="Z44" s="20">
-        <f>MIN(C44:Y44)</f>
+      <c r="Z44" s="30">
+        <v>191.19</v>
+      </c>
+      <c r="AA44" s="20">
+        <f>MIN(C44:Z44)</f>
         <v>88.329999999999998</v>
       </c>
-      <c r="AA44" s="21">
-        <f>MAX(C44:Y44)</f>
+      <c r="AB44" s="21">
+        <f>MAX(C44:Z44)</f>
         <v>191.19</v>
       </c>
-      <c r="AB44" s="21">
-        <f>AVERAGE(C44:Y44)</f>
-        <v>107.45789473684212</v>
-      </c>
       <c r="AC44" s="21">
-        <f>AVERAGE(Q44:Y44)</f>
-        <v>128.71111111111111</v>
-      </c>
-      <c r="AD44" s="22">
-        <f>(AC44/AB44)-1</f>
-        <v>0.19778180492291253</v>
+        <f>AVERAGE(C44:Z44)</f>
+        <v>111.64450000000002</v>
+      </c>
+      <c r="AD44" s="21">
+        <f>AVERAGE(Q44:Z44)</f>
+        <v>134.959</v>
       </c>
       <c r="AE44" s="22">
-        <f>(AC44/Z44)-1</f>
-        <v>0.4571619054807099</v>
+        <f>(AD44/AC44)-1</f>
+        <v>0.20882802108478238</v>
       </c>
       <c r="AF44" s="22">
-        <f>(AA44/Z44)-1</f>
+        <f>(AD44/AA44)-1</f>
+        <v>0.52789539227895399</v>
+      </c>
+      <c r="AG44" s="22">
+        <f>(AB44/AA44)-1</f>
         <v>1.1644967734631497</v>
       </c>
-      <c r="AG44" s="23" t="s">
-        <v>123</v>
+      <c r="AH44" s="23" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="45" ht="18">
       <c r="A45" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C45" s="17"/>
       <c r="D45" s="17">
@@ -5126,44 +5245,47 @@
       <c r="Y45" s="36">
         <v>40.039999999999999</v>
       </c>
-      <c r="Z45" s="20">
-        <f>MIN(C45:Y45)</f>
+      <c r="Z45" s="36">
+        <v>39.899999999999999</v>
+      </c>
+      <c r="AA45" s="20">
+        <f>MIN(C45:Z45)</f>
         <v>29.989999999999998</v>
       </c>
-      <c r="AA45" s="21">
-        <f>MAX(C45:Y45)</f>
+      <c r="AB45" s="21">
+        <f>MAX(C45:Z45)</f>
         <v>44.979999999999997</v>
       </c>
-      <c r="AB45" s="21">
-        <f>AVERAGE(C45:Y45)</f>
-        <v>36.602500000000006</v>
-      </c>
       <c r="AC45" s="21">
-        <f>AVERAGE(Q45:Y45)</f>
-        <v>36.745555555555562</v>
-      </c>
-      <c r="AD45" s="22">
-        <f>(AC45/AB45)-1</f>
-        <v>3.9083547723668399e-003</v>
+        <f>AVERAGE(C45:Z45)</f>
+        <v>36.759523809523813</v>
+      </c>
+      <c r="AD45" s="21">
+        <f>AVERAGE(Q45:Z45)</f>
+        <v>37.061</v>
       </c>
       <c r="AE45" s="22">
-        <f>(AC45/Z45)-1</f>
-        <v>0.22526027194249965</v>
+        <f>(AD45/AC45)-1</f>
+        <v>8.2013083748946336e-003</v>
       </c>
       <c r="AF45" s="22">
-        <f>(AA45/Z45)-1</f>
+        <f>(AD45/AA45)-1</f>
+        <v>0.23577859286428815</v>
+      </c>
+      <c r="AG45" s="22">
+        <f>(AB45/AA45)-1</f>
         <v>0.49983327775925313</v>
       </c>
-      <c r="AG45" s="23" t="s">
-        <v>126</v>
+      <c r="AH45" s="23" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="46" ht="18">
       <c r="A46" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C46" s="17"/>
       <c r="D46" s="17">
@@ -5228,44 +5350,47 @@
       <c r="Y46" s="36">
         <v>30.989999999999998</v>
       </c>
-      <c r="Z46" s="20">
-        <f>MIN(C46:Y46)</f>
+      <c r="Z46" s="36">
+        <v>30.989999999999998</v>
+      </c>
+      <c r="AA46" s="20">
+        <f>MIN(C46:Z46)</f>
         <v>25.989999999999998</v>
       </c>
-      <c r="AA46" s="21">
-        <f>MAX(C46:Y46)</f>
+      <c r="AB46" s="21">
+        <f>MAX(C46:Z46)</f>
         <v>42</v>
       </c>
-      <c r="AB46" s="21">
-        <f>AVERAGE(C46:Y46)</f>
-        <v>31.887999999999998</v>
-      </c>
       <c r="AC46" s="21">
-        <f>AVERAGE(Q46:Y46)</f>
-        <v>32.615555555555567</v>
-      </c>
-      <c r="AD46" s="22">
-        <f>(AC46/AB46)-1</f>
-        <v>2.2815966995596071e-002</v>
+        <f>AVERAGE(C46:Z46)</f>
+        <v>31.845238095238095</v>
+      </c>
+      <c r="AD46" s="21">
+        <f>AVERAGE(Q46:Z46)</f>
+        <v>32.45300000000001</v>
       </c>
       <c r="AE46" s="22">
-        <f>(AC46/Z46)-1</f>
-        <v>0.25492710871702839</v>
+        <f>(AD46/AC46)-1</f>
+        <v>1.9084859813084387e-002</v>
       </c>
       <c r="AF46" s="22">
-        <f>(AA46/Z46)-1</f>
+        <f>(AD46/AA46)-1</f>
+        <v>0.24867256637168178</v>
+      </c>
+      <c r="AG46" s="22">
+        <f>(AB46/AA46)-1</f>
         <v>0.61600615621392851</v>
       </c>
-      <c r="AG46" s="23" t="s">
-        <v>129</v>
+      <c r="AH46" s="23" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="47" ht="18">
       <c r="A47" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C47" s="17"/>
       <c r="D47" s="17">
@@ -5330,44 +5455,47 @@
       <c r="Y47" s="36">
         <v>28.899999999999999</v>
       </c>
-      <c r="Z47" s="20">
-        <f>MIN(C47:Y47)</f>
+      <c r="Z47" s="36">
+        <v>28.899999999999999</v>
+      </c>
+      <c r="AA47" s="20">
+        <f>MIN(C47:Z47)</f>
         <v>21.690000000000001</v>
       </c>
-      <c r="AA47" s="21">
-        <f>MAX(C47:Y47)</f>
+      <c r="AB47" s="21">
+        <f>MAX(C47:Z47)</f>
         <v>43.990000000000002</v>
       </c>
-      <c r="AB47" s="21">
-        <f>AVERAGE(C47:Y47)</f>
-        <v>29.413999999999994</v>
-      </c>
       <c r="AC47" s="21">
-        <f>AVERAGE(Q47:Y47)</f>
-        <v>28.052222222222227</v>
-      </c>
-      <c r="AD47" s="22">
-        <f>(AC47/AB47)-1</f>
-        <v>-4.6296925878077322e-002</v>
+        <f>AVERAGE(C47:Z47)</f>
+        <v>29.389523809523801</v>
+      </c>
+      <c r="AD47" s="21">
+        <f>AVERAGE(Q47:Z47)</f>
+        <v>28.137</v>
       </c>
       <c r="AE47" s="22">
-        <f>(AC47/Z47)-1</f>
-        <v>0.29332513703191454</v>
+        <f>(AD47/AC47)-1</f>
+        <v>-4.2618036877409837e-002</v>
       </c>
       <c r="AF47" s="22">
-        <f>(AA47/Z47)-1</f>
+        <f>(AD47/AA47)-1</f>
+        <v>0.29723374827109272</v>
+      </c>
+      <c r="AG47" s="22">
+        <f>(AB47/AA47)-1</f>
         <v>1.0281235592438911</v>
       </c>
-      <c r="AG47" s="23" t="s">
-        <v>132</v>
+      <c r="AH47" s="23" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="48" ht="54">
       <c r="A48" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C48" s="17"/>
       <c r="D48" s="17"/>
@@ -5388,10 +5516,10 @@
         <v>1714.0799999999999</v>
       </c>
       <c r="K48" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L48" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M48" s="25">
         <v>1449.28</v>
@@ -5432,44 +5560,47 @@
       <c r="Y48" s="18">
         <v>1820.77</v>
       </c>
-      <c r="Z48" s="20">
-        <f>MIN(C48:Y48)</f>
+      <c r="Z48" s="18">
+        <v>1820.77</v>
+      </c>
+      <c r="AA48" s="20">
+        <f>MIN(C48:Z48)</f>
         <v>1449.28</v>
       </c>
-      <c r="AA48" s="21">
-        <f>MAX(C48:Y48)</f>
+      <c r="AB48" s="21">
+        <f>MAX(C48:Z48)</f>
         <v>1820.77</v>
       </c>
-      <c r="AB48" s="21">
-        <f>AVERAGE(C48:Y48)</f>
-        <v>1698.8299999999999</v>
-      </c>
       <c r="AC48" s="21">
-        <f>AVERAGE(Q48:Y48)</f>
-        <v>1677.4388888888889</v>
-      </c>
-      <c r="AD48" s="22">
-        <f>(AC48/AB48)-1</f>
-        <v>-1.2591672569421952e-002</v>
+        <f>AVERAGE(C48:Z48)</f>
+        <v>1705.247894736842</v>
+      </c>
+      <c r="AD48" s="21">
+        <f>AVERAGE(Q48:Z48)</f>
+        <v>1691.7720000000002</v>
       </c>
       <c r="AE48" s="22">
-        <f>(AC48/Z48)-1</f>
-        <v>0.15742912956011867</v>
+        <f>(AD48/AC48)-1</f>
+        <v>-7.9026015973597818e-003</v>
       </c>
       <c r="AF48" s="22">
-        <f>(AA48/Z48)-1</f>
+        <f>(AD48/AA48)-1</f>
+        <v>0.16731894457937746</v>
+      </c>
+      <c r="AG48" s="22">
+        <f>(AB48/AA48)-1</f>
         <v>0.25632727975270475</v>
       </c>
-      <c r="AG48" s="1" t="s">
-        <v>134</v>
+      <c r="AH48" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="49" ht="18">
       <c r="A49" s="26" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B49" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C49" s="29"/>
       <c r="D49" s="29"/>
@@ -5532,44 +5663,47 @@
       <c r="Y49" s="36">
         <v>43.990000000000002</v>
       </c>
-      <c r="Z49" s="20">
-        <f>MIN(C49:Y49)</f>
+      <c r="Z49" s="36">
+        <v>36.990000000000002</v>
+      </c>
+      <c r="AA49" s="20">
+        <f>MIN(C49:Z49)</f>
         <v>30.989999999999998</v>
       </c>
-      <c r="AA49" s="21">
-        <f>MAX(C49:Y49)</f>
+      <c r="AB49" s="21">
+        <f>MAX(C49:Z49)</f>
         <v>43.990000000000002</v>
       </c>
-      <c r="AB49" s="21">
-        <f>AVERAGE(C49:Y49)</f>
-        <v>37.268421052631574</v>
-      </c>
       <c r="AC49" s="21">
-        <f>AVERAGE(Q49:Y49)</f>
-        <v>38.57</v>
-      </c>
-      <c r="AD49" s="22">
-        <f>(AC49/AB49)-1</f>
-        <v>3.4924445699760165e-002</v>
+        <f>AVERAGE(C49:Z49)</f>
+        <v>37.254499999999993</v>
+      </c>
+      <c r="AD49" s="21">
+        <f>AVERAGE(Q49:Z49)</f>
+        <v>38.411999999999999</v>
       </c>
       <c r="AE49" s="22">
-        <f>(AC49/Z49)-1</f>
-        <v>0.24459503065505017</v>
+        <f>(AD49/AC49)-1</f>
+        <v>3.1070072071830435e-002</v>
       </c>
       <c r="AF49" s="22">
-        <f>(AA49/Z49)-1</f>
+        <f>(AD49/AA49)-1</f>
+        <v>0.23949661181026149</v>
+      </c>
+      <c r="AG49" s="22">
+        <f>(AB49/AA49)-1</f>
         <v>0.41949015811552126</v>
       </c>
-      <c r="AG49" s="23" t="s">
-        <v>137</v>
+      <c r="AH49" s="23" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="50" ht="18">
       <c r="A50" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C50" s="17"/>
       <c r="D50" s="17"/>
@@ -5632,44 +5766,47 @@
       <c r="Y50" s="17">
         <v>85.209999999999994</v>
       </c>
-      <c r="Z50" s="20">
-        <f>MIN(C50:Y50)</f>
+      <c r="Z50" s="17">
+        <v>85.209999999999994</v>
+      </c>
+      <c r="AA50" s="20">
+        <f>MIN(C50:Z50)</f>
         <v>81.689999999999998</v>
       </c>
-      <c r="AA50" s="21">
-        <f>MAX(C50:Y50)</f>
+      <c r="AB50" s="21">
+        <f>MAX(C50:Z50)</f>
         <v>93.280000000000001</v>
       </c>
-      <c r="AB50" s="21">
-        <f>AVERAGE(C50:Y50)</f>
-        <v>88.041052631578964</v>
-      </c>
       <c r="AC50" s="21">
-        <f>AVERAGE(Q50:Y50)</f>
-        <v>85.351111111111123</v>
-      </c>
-      <c r="AD50" s="22">
-        <f>(AC50/AB50)-1</f>
-        <v>-3.0553263961124011e-002</v>
+        <f>AVERAGE(C50:Z50)</f>
+        <v>87.899500000000018</v>
+      </c>
+      <c r="AD50" s="21">
+        <f>AVERAGE(Q50:Z50)</f>
+        <v>85.337000000000018</v>
       </c>
       <c r="AE50" s="22">
-        <f>(AC50/Z50)-1</f>
-        <v>4.4817127079338048e-002</v>
+        <f>(AD50/AC50)-1</f>
+        <v>-2.9152611789600602e-002</v>
       </c>
       <c r="AF50" s="22">
-        <f>(AA50/Z50)-1</f>
+        <f>(AD50/AA50)-1</f>
+        <v>4.4644387317909429e-002</v>
+      </c>
+      <c r="AG50" s="22">
+        <f>(AB50/AA50)-1</f>
         <v>0.1418778308238462</v>
       </c>
-      <c r="AG50" s="1" t="s">
-        <v>140</v>
+      <c r="AH50" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="51" ht="18">
       <c r="A51" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C51" s="17"/>
       <c r="D51" s="17"/>
@@ -5734,44 +5871,47 @@
       <c r="Y51" s="34">
         <v>298.80000000000001</v>
       </c>
-      <c r="Z51" s="20">
-        <f>MIN(C51:Y51)</f>
+      <c r="Z51" s="34">
         <v>298.80000000000001</v>
       </c>
-      <c r="AA51" s="21">
-        <f>MAX(C51:Y51)</f>
+      <c r="AA51" s="20">
+        <f>MIN(C51:Z51)</f>
+        <v>298.80000000000001</v>
+      </c>
+      <c r="AB51" s="21">
+        <f>MAX(C51:Z51)</f>
         <v>309.05000000000001</v>
       </c>
-      <c r="AB51" s="21">
-        <f>AVERAGE(C51:Y51)</f>
-        <v>307.5125000000001</v>
-      </c>
       <c r="AC51" s="21">
-        <f>AVERAGE(Q51:Y51)</f>
-        <v>305.63333333333338</v>
-      </c>
-      <c r="AD51" s="22">
-        <f>(AC51/AB51)-1</f>
-        <v>-6.1108627020584061e-003</v>
+        <f>AVERAGE(C51:Z51)</f>
+        <v>307.09761904761916</v>
+      </c>
+      <c r="AD51" s="21">
+        <f>AVERAGE(Q51:Z51)</f>
+        <v>304.95000000000005</v>
       </c>
       <c r="AE51" s="22">
-        <f>(AC51/Z51)-1</f>
-        <v>2.2869254796965777e-002</v>
+        <f>(AD51/AC51)-1</f>
+        <v>-6.993278079717391e-003</v>
       </c>
       <c r="AF51" s="22">
-        <f>(AA51/Z51)-1</f>
+        <f>(AD51/AA51)-1</f>
+        <v>2.058232931726911e-002</v>
+      </c>
+      <c r="AG51" s="22">
+        <f>(AB51/AA51)-1</f>
         <v>3.4303882195448443e-002</v>
       </c>
-      <c r="AG51" s="23" t="s">
-        <v>143</v>
+      <c r="AH51" s="23" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="52" ht="18">
       <c r="A52" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C52" s="17"/>
       <c r="D52" s="17"/>
@@ -5834,41 +5974,44 @@
       <c r="Y52" s="25">
         <v>100.44</v>
       </c>
-      <c r="Z52" s="20">
-        <f>MIN(C52:Y52)</f>
+      <c r="Z52" s="25">
         <v>100.44</v>
       </c>
-      <c r="AA52" s="21">
-        <f>MAX(C52:Y52)</f>
+      <c r="AA52" s="20">
+        <f>MIN(C52:Z52)</f>
+        <v>100.44</v>
+      </c>
+      <c r="AB52" s="21">
+        <f>MAX(C52:Z52)</f>
         <v>108.98999999999999</v>
       </c>
-      <c r="AB52" s="21">
-        <f>AVERAGE(C52:Y52)</f>
-        <v>108.53999999999999</v>
-      </c>
       <c r="AC52" s="21">
-        <f>AVERAGE(Q52:Y52)</f>
-        <v>108.03999999999999</v>
-      </c>
-      <c r="AD52" s="22">
-        <f>(AC52/AB52)-1</f>
-        <v>-4.6065966463976205e-003</v>
+        <f>AVERAGE(C52:Z52)</f>
+        <v>108.13499999999999</v>
+      </c>
+      <c r="AD52" s="21">
+        <f>AVERAGE(Q52:Z52)</f>
+        <v>107.28</v>
       </c>
       <c r="AE52" s="22">
-        <f>(AC52/Z52)-1</f>
-        <v>7.5667064914376692e-002</v>
+        <f>(AD52/AC52)-1</f>
+        <v>-7.9067831876820094e-003</v>
       </c>
       <c r="AF52" s="22">
-        <f>(AA52/Z52)-1</f>
+        <f>(AD52/AA52)-1</f>
+        <v>6.8100358422939156e-002</v>
+      </c>
+      <c r="AG52" s="22">
+        <f>(AB52/AA52)-1</f>
         <v>8.5125448028673834e-002</v>
       </c>
-      <c r="AG52" s="38" t="s">
-        <v>145</v>
+      <c r="AH52" s="38" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="53" ht="18">
       <c r="B53" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O53" s="17">
         <v>1.49</v>
@@ -5903,92 +6046,95 @@
       <c r="Y53" s="17">
         <v>1.99</v>
       </c>
-      <c r="Z53" s="20">
-        <f>MIN(C53:Y53)</f>
+      <c r="Z53" s="17">
+        <v>1.99</v>
+      </c>
+      <c r="AA53" s="20">
+        <f>MIN(C53:Z53)</f>
         <v>1.49</v>
       </c>
-      <c r="AA53" s="21">
-        <f>MAX(C53:Y53)</f>
+      <c r="AB53" s="21">
+        <f>MAX(C53:Z53)</f>
         <v>1.99</v>
       </c>
-      <c r="AB53" s="21">
-        <f>AVERAGE(C53:Y53)</f>
-        <v>1.7627272727272725</v>
-      </c>
       <c r="AC53" s="21">
-        <f>AVERAGE(Q53:Y53)</f>
-        <v>1.8233333333333333</v>
-      </c>
-      <c r="AD53" s="22">
-        <f>(AC53/AB53)-1</f>
-        <v>3.4381983840467756e-002</v>
+        <f>AVERAGE(C53:Z53)</f>
+        <v>1.7816666666666663</v>
+      </c>
+      <c r="AD53" s="21">
+        <f>AVERAGE(Q53:Z53)</f>
+        <v>1.8399999999999999</v>
       </c>
       <c r="AE53" s="22">
-        <f>(AC53/Z53)-1</f>
-        <v>0.22371364653243853</v>
+        <f>(AD53/AC53)-1</f>
+        <v>3.2740879326473404e-002</v>
       </c>
       <c r="AF53" s="22">
-        <f>(AA53/Z53)-1</f>
+        <f>(AD53/AA53)-1</f>
+        <v>0.2348993288590604</v>
+      </c>
+      <c r="AG53" s="22">
+        <f>(AB53/AA53)-1</f>
         <v>0.33557046979865768</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="Z1:Z6"/>
     <mergeCell ref="AA1:AA6"/>
     <mergeCell ref="AB1:AB6"/>
     <mergeCell ref="AC1:AC6"/>
     <mergeCell ref="AD1:AD6"/>
     <mergeCell ref="AE1:AE6"/>
     <mergeCell ref="AF1:AF6"/>
+    <mergeCell ref="AG1:AG6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="AG8"/>
-    <hyperlink r:id="rId2" ref="AG9"/>
-    <hyperlink r:id="rId3" ref="AG10"/>
-    <hyperlink r:id="rId4" ref="AG11"/>
-    <hyperlink r:id="rId5" ref="AG12"/>
-    <hyperlink r:id="rId6" ref="AG13"/>
-    <hyperlink r:id="rId7" ref="AG14"/>
-    <hyperlink r:id="rId8" ref="AG15"/>
-    <hyperlink r:id="rId9" ref="AG16"/>
-    <hyperlink r:id="rId10" ref="AG17"/>
-    <hyperlink r:id="rId11" ref="AG18"/>
-    <hyperlink r:id="rId12" ref="AG19"/>
-    <hyperlink r:id="rId13" ref="AG20"/>
-    <hyperlink r:id="rId14" ref="AG21"/>
-    <hyperlink r:id="rId15" ref="AG22"/>
-    <hyperlink r:id="rId16" ref="AG23"/>
-    <hyperlink r:id="rId17" ref="AG24"/>
-    <hyperlink r:id="rId18" ref="AG25"/>
-    <hyperlink r:id="rId19" ref="AG26"/>
-    <hyperlink r:id="rId20" ref="AG27"/>
-    <hyperlink r:id="rId21" ref="AG28"/>
-    <hyperlink r:id="rId22" ref="AG29"/>
-    <hyperlink r:id="rId23" ref="AG30"/>
-    <hyperlink r:id="rId24" ref="AG31"/>
-    <hyperlink r:id="rId25" ref="AG32"/>
-    <hyperlink r:id="rId26" ref="AG33"/>
-    <hyperlink r:id="rId27" ref="AG34"/>
-    <hyperlink r:id="rId28" ref="AG35"/>
-    <hyperlink r:id="rId29" ref="AG36"/>
-    <hyperlink r:id="rId29" ref="AG37"/>
-    <hyperlink r:id="rId29" ref="AG38"/>
-    <hyperlink r:id="rId29" ref="AG39"/>
-    <hyperlink r:id="rId29" ref="AG40"/>
-    <hyperlink r:id="rId29" ref="AG41"/>
-    <hyperlink r:id="rId30" ref="AG43"/>
-    <hyperlink r:id="rId31" ref="AG44"/>
-    <hyperlink r:id="rId32" ref="AG45"/>
-    <hyperlink r:id="rId33" ref="AG46"/>
-    <hyperlink r:id="rId34" ref="AG47"/>
-    <hyperlink r:id="rId35" ref="AG49"/>
-    <hyperlink r:id="rId36" ref="AG51"/>
-    <hyperlink r:id="rId37" ref="AG52"/>
+    <hyperlink r:id="rId1" ref="AH8"/>
+    <hyperlink r:id="rId2" ref="AH9"/>
+    <hyperlink r:id="rId3" ref="AH10"/>
+    <hyperlink r:id="rId4" ref="AH11"/>
+    <hyperlink r:id="rId5" ref="AH12"/>
+    <hyperlink r:id="rId6" ref="AH13"/>
+    <hyperlink r:id="rId7" ref="AH14"/>
+    <hyperlink r:id="rId8" ref="AH15"/>
+    <hyperlink r:id="rId9" ref="AH16"/>
+    <hyperlink r:id="rId10" ref="AH17"/>
+    <hyperlink r:id="rId11" ref="AH18"/>
+    <hyperlink r:id="rId12" ref="AH19"/>
+    <hyperlink r:id="rId13" ref="AH20"/>
+    <hyperlink r:id="rId14" ref="AH21"/>
+    <hyperlink r:id="rId15" ref="AH22"/>
+    <hyperlink r:id="rId16" ref="AH23"/>
+    <hyperlink r:id="rId17" ref="AH24"/>
+    <hyperlink r:id="rId18" ref="AH25"/>
+    <hyperlink r:id="rId19" ref="AH26"/>
+    <hyperlink r:id="rId20" ref="AH27"/>
+    <hyperlink r:id="rId21" ref="AH28"/>
+    <hyperlink r:id="rId22" ref="AH29"/>
+    <hyperlink r:id="rId23" ref="AH30"/>
+    <hyperlink r:id="rId24" ref="AH31"/>
+    <hyperlink r:id="rId25" ref="AH32"/>
+    <hyperlink r:id="rId26" ref="AH33"/>
+    <hyperlink r:id="rId27" ref="AH34"/>
+    <hyperlink r:id="rId28" ref="AH35"/>
+    <hyperlink r:id="rId29" ref="AH36"/>
+    <hyperlink r:id="rId29" ref="AH37"/>
+    <hyperlink r:id="rId29" ref="AH38"/>
+    <hyperlink r:id="rId29" ref="AH39"/>
+    <hyperlink r:id="rId29" ref="AH40"/>
+    <hyperlink r:id="rId29" ref="AH41"/>
+    <hyperlink r:id="rId30" ref="AH43"/>
+    <hyperlink r:id="rId31" ref="AH44"/>
+    <hyperlink r:id="rId32" ref="AH45"/>
+    <hyperlink r:id="rId33" ref="AH46"/>
+    <hyperlink r:id="rId34" ref="AH47"/>
+    <hyperlink r:id="rId35" ref="AH49"/>
+    <hyperlink r:id="rId36" ref="AH51"/>
+    <hyperlink r:id="rId37" ref="AH52"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.25196850393700787" right="0.25196850393700787" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="34" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="32" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>